<commit_message>
Registra el telefono de la ponente del modulo 2
Anade el numero de contacto de la docente de patrones alimentarios, cuyo
curriculo no traia ningun dato de contacto, y confirma el de la presidenta
de la Sociedad, que coincide exactamente con el que figura en su hoja de
vida.

Quedan tres numeros registrados de catorce docentes identificados.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -237,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -371,6 +371,9 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2350,7 +2353,11 @@
         </is>
       </c>
       <c r="E6" s="41" t="n"/>
-      <c r="F6" s="41" t="n"/>
+      <c r="F6" s="60" t="inlineStr">
+        <is>
+          <t>+593 98 765 4330</t>
+        </is>
+      </c>
       <c r="G6" s="41" t="n"/>
       <c r="H6" s="41" t="n"/>
       <c r="I6" s="40" t="inlineStr">
@@ -2582,7 +2589,7 @@
           <t>lizrg@hotmail.com</t>
         </is>
       </c>
-      <c r="F12" s="53" t="inlineStr">
+      <c r="F12" s="60" t="inlineStr">
         <is>
           <t>+593 99 907 3471</t>
         </is>
@@ -2809,7 +2816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3111,11 +3118,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Registra el telefono del ponente internacional de Costa Rica
El prefijo del numero corresponde al pais que consta en su curriculo.
Con este son cuatro los contactos registrados de catorce docentes.

Este contacto abre ademas la via directa para proponerle la clase que
quedo vacante sobre sindrome cardiorrenometabolico, materia que coordina
en el grupo de investigacion regional.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2513,7 +2513,11 @@
         </is>
       </c>
       <c r="E10" s="41" t="n"/>
-      <c r="F10" s="41" t="n"/>
+      <c r="F10" s="60" t="inlineStr">
+        <is>
+          <t>+506 8392 7083</t>
+        </is>
+      </c>
       <c r="G10" s="41" t="n"/>
       <c r="H10" s="41" t="n"/>
       <c r="I10" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Registra el telefono del co-coordinador academico
Anade tambien su correo, ya conocido por los hilos previos de la Sociedad.
Con este son cinco los contactos registrados de catorce docentes.

Es el primer contacto disponible de los diez ponentes que figuran en el
programa sin aceptacion escrita, requisito para el expediente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2630,8 +2630,16 @@
       </c>
       <c r="C13" s="41" t="n"/>
       <c r="D13" s="41" t="n"/>
-      <c r="E13" s="41" t="n"/>
-      <c r="F13" s="41" t="n"/>
+      <c r="E13" s="60" t="inlineStr">
+        <is>
+          <t>pablo.vanegas90@gmail.com</t>
+        </is>
+      </c>
+      <c r="F13" s="60" t="inlineStr">
+        <is>
+          <t>+593 98 765 3136</t>
+        </is>
+      </c>
       <c r="G13" s="41" t="n"/>
       <c r="H13" s="41" t="n"/>
       <c r="I13" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Registra cuatro contactos mas y marca un numero duplicado para verificar
Entran los contactos de la ponente de terapia nutricional, el de
insulinoterapia y las dos docentes que llevan dos clases cada una. Con
ellos son nueve los contactos en firme de catorce docentes, y quedan
cubiertas las tres clases que vencen el 29 de octubre.

El numero recibido para la coordinadora de salud digital es identico al
de otra docente, por lo que no se escribe en la ficha: la celda queda
marcada para verificacion en lugar de guardar un dato probablemente
equivocado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -167,6 +167,12 @@
       <color rgb="006B6B6B"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -237,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -373,6 +379,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2281,7 +2290,11 @@
       </c>
       <c r="D4" s="41" t="n"/>
       <c r="E4" s="41" t="n"/>
-      <c r="F4" s="41" t="n"/>
+      <c r="F4" s="61" t="inlineStr">
+        <is>
+          <t>⚠ VERIFICAR — el número recibido coincide con el de la Dra. Astudillo</t>
+        </is>
+      </c>
       <c r="G4" s="41" t="n"/>
       <c r="H4" s="41" t="n"/>
       <c r="I4" s="40" t="inlineStr">
@@ -2315,7 +2328,11 @@
       </c>
       <c r="D5" s="41" t="n"/>
       <c r="E5" s="41" t="n"/>
-      <c r="F5" s="41" t="n"/>
+      <c r="F5" s="60" t="inlineStr">
+        <is>
+          <t>+593 98 736 8816</t>
+        </is>
+      </c>
       <c r="G5" s="41" t="n"/>
       <c r="H5" s="41" t="n"/>
       <c r="I5" s="40" t="inlineStr">
@@ -2669,7 +2686,11 @@
       <c r="C14" s="41" t="n"/>
       <c r="D14" s="41" t="n"/>
       <c r="E14" s="41" t="n"/>
-      <c r="F14" s="41" t="n"/>
+      <c r="F14" s="60" t="inlineStr">
+        <is>
+          <t>+593 99 811 1635</t>
+        </is>
+      </c>
       <c r="G14" s="41" t="n"/>
       <c r="H14" s="41" t="n"/>
       <c r="I14" s="40" t="inlineStr">
@@ -2699,7 +2720,11 @@
       <c r="C15" s="41" t="n"/>
       <c r="D15" s="41" t="n"/>
       <c r="E15" s="41" t="n"/>
-      <c r="F15" s="41" t="n"/>
+      <c r="F15" s="60" t="inlineStr">
+        <is>
+          <t>+593 99 807 8964</t>
+        </is>
+      </c>
       <c r="G15" s="41" t="n"/>
       <c r="H15" s="41" t="n"/>
       <c r="I15" s="40" t="inlineStr">
@@ -2729,7 +2754,11 @@
       <c r="C16" s="41" t="n"/>
       <c r="D16" s="41" t="n"/>
       <c r="E16" s="41" t="n"/>
-      <c r="F16" s="41" t="n"/>
+      <c r="F16" s="60" t="inlineStr">
+        <is>
+          <t>+593 99 862 5711</t>
+        </is>
+      </c>
       <c r="G16" s="41" t="n"/>
       <c r="H16" s="41" t="n"/>
       <c r="I16" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Resuelve el contacto marcado para verificacion
El numero correcto coincide con el que constaba en un registro de
inscripcion de 2023 hallado en el propio buzon, de modo que queda
confirmado por dos fuentes independientes. Se anade tambien el correo
institucional.

Verificado que no quedan numeros duplicados en la ficha. Son diez
contactos de catorce docentes; faltan cuatro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2289,10 +2289,14 @@
         </is>
       </c>
       <c r="D4" s="41" t="n"/>
-      <c r="E4" s="41" t="n"/>
-      <c r="F4" s="61" t="inlineStr">
-        <is>
-          <t>⚠ VERIFICAR — el número recibido coincide con el de la Dra. Astudillo</t>
+      <c r="E4" s="60" t="inlineStr">
+        <is>
+          <t>info@draomidresperez.com</t>
+        </is>
+      </c>
+      <c r="F4" s="60" t="inlineStr">
+        <is>
+          <t>+593 98 206 2988</t>
         </is>
       </c>
       <c r="G4" s="41" t="n"/>

</xml_diff>

<commit_message>
Registra el correo del ponente de Costa Rica y envia su invitacion
La direccion procede del propio buzon: consta en la correspondencia
directa de noviembre de 2025 y en las listas de la junta directiva de la
asociacion regional.

El mensaje se envio adaptado a formato de correo. Se retiro la mencion a
documentos adjuntos, que no pueden incorporarse desde esta sesion, y se
sustituyo por el anuncio de un envio posterior con la plantilla de
diapositivas y el formato de declaracion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2533,7 +2533,11 @@
           <t>Clínica Los Yoses · San José, Costa Rica</t>
         </is>
       </c>
-      <c r="E10" s="41" t="n"/>
+      <c r="E10" s="60" t="inlineStr">
+        <is>
+          <t>chenku2409@gmail.com</t>
+        </is>
+      </c>
       <c r="F10" s="60" t="inlineStr">
         <is>
           <t>+506 8392 7083</t>

</xml_diff>

<commit_message>
Anade la propuesta a la endocrinologa sugerida por la coordinacion
Su especialidad y lugar de trabajo confirman que es localizable de forma
directa, por lo que deja de ser una pregunta pendiente para la
coordinacion academica.

Se le ofrecen las dos vacantes de endocrinologia con plazos mas holgados,
adecuadas para quien se incorpora tarde, una de ellas en el modulo
coordinado internamente. Ambas quedan anotadas en la hoja de vacantes con
su nombre como candidata.

El mensaje se redacta en registro cercano por tratarse de una colega de la
misma institucion, y recomienda plantearlo en persona antes que por
mensajeria.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -173,6 +173,10 @@
       <color rgb="009C0006"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -243,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -382,6 +386,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2865,7 +2875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2993,9 +3003,17 @@
           <t>Nutricionista clínico o endocrinólogo; tema de alta demanda</t>
         </is>
       </c>
-      <c r="E6" s="41" t="n"/>
+      <c r="E6" s="62" t="inlineStr">
+        <is>
+          <t>Dra. Janeth Bermeo (propuesta)</t>
+        </is>
+      </c>
       <c r="F6" s="41" t="n"/>
-      <c r="G6" s="41" t="n"/>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>Endocrinóloga, Hospital del Río · contacto directo</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="50" t="n">
@@ -3016,9 +3034,17 @@
           <t>Endocrinólogo con experiencia en MCG/tecnología en diabetes</t>
         </is>
       </c>
-      <c r="E7" s="41" t="n"/>
+      <c r="E7" s="62" t="inlineStr">
+        <is>
+          <t>Dra. Janeth Bermeo (propuesta)</t>
+        </is>
+      </c>
       <c r="F7" s="41" t="n"/>
-      <c r="G7" s="41" t="n"/>
+      <c r="G7" s="63" t="inlineStr">
+        <is>
+          <t>Endocrinóloga, Hospital del Río · contacto directo</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="50" t="n">
@@ -3167,6 +3193,11 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Registra la incorporacion de la endocrinologa al modulo 2
Acepto la clase de nutricion conductual, con lo que las clases sin
ponente bajan de diez a nueve y los docentes identificados suben a
quince. Se incorpora a la ficha del expediente, se actualiza el estado de
la clase en la matriz y se retira de la hoja de vacantes, junto con las
anotaciones de candidatura en las dos clases que finalmente no tomo.

El mensaje de confirmacion advierte que su grabacion vence el 29 de
octubre, el plazo mas corto del programa porque su modulo lo abre, y le
ofrece cambiar a un tema con mas margen: eligio sin conocer ese dato.

Verificado el reparto de las veintiocho clases: nueve confirmadas, diez
por confirmar y nueve vacantes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -247,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -393,6 +393,12 @@
     </xf>
     <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1333,10 +1339,14 @@
           <t>Hambre fisiológica y emocional; conducta alimentaria; adherencia terapéutica</t>
         </is>
       </c>
-      <c r="E9" s="28" t="inlineStr"/>
-      <c r="F9" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E9" s="64" t="inlineStr">
+        <is>
+          <t>Dra. Janeth Bermeo</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G9" s="23" t="n">
@@ -1344,7 +1354,7 @@
       </c>
       <c r="H9" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: nutricionista clínico o psicólogo de la conducta alimentaria.</t>
+          <t>Aceptó el 22/09/2026. Endocrinóloga del Hospital del Río. Pendiente: hoja de vida, cédula, foto y declaración COI.</t>
         </is>
       </c>
     </row>
@@ -2825,20 +2835,42 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="54" t="n"/>
-      <c r="B18" s="52" t="n"/>
-      <c r="C18" s="53" t="n"/>
-      <c r="D18" s="53" t="n"/>
-      <c r="E18" s="53" t="n"/>
-      <c r="F18" s="53" t="n"/>
-      <c r="G18" s="53" t="n"/>
-      <c r="H18" s="53" t="n"/>
-      <c r="I18" s="53" t="n"/>
-      <c r="J18" s="54" t="n"/>
-      <c r="K18" s="54" t="n"/>
-      <c r="L18" s="54" t="n"/>
-      <c r="M18" s="54" t="n"/>
-      <c r="N18" s="55" t="n"/>
+      <c r="A18" s="54" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Janeth Bermeo</t>
+        </is>
+      </c>
+      <c r="C18" s="53" t="inlineStr">
+        <is>
+          <t>Endocrinología</t>
+        </is>
+      </c>
+      <c r="D18" s="53" t="inlineStr">
+        <is>
+          <t>Hospital del Río · Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="41" t="n"/>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="41" t="n"/>
+      <c r="I18" s="54" t="inlineStr">
+        <is>
+          <t>M2 · C3</t>
+        </is>
+      </c>
+      <c r="J18" s="42" t="n"/>
+      <c r="K18" s="42" t="n"/>
+      <c r="L18" s="42" t="n"/>
+      <c r="M18" s="42" t="n"/>
+      <c r="N18" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="46" t="n"/>
@@ -3003,17 +3035,9 @@
           <t>Nutricionista clínico o endocrinólogo; tema de alta demanda</t>
         </is>
       </c>
-      <c r="E6" s="62" t="inlineStr">
-        <is>
-          <t>Dra. Janeth Bermeo (propuesta)</t>
-        </is>
-      </c>
+      <c r="E6" s="62" t="n"/>
       <c r="F6" s="41" t="n"/>
-      <c r="G6" s="63" t="inlineStr">
-        <is>
-          <t>Endocrinóloga, Hospital del Río · contacto directo</t>
-        </is>
-      </c>
+      <c r="G6" s="63" t="n"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="50" t="n">
@@ -3034,17 +3058,9 @@
           <t>Endocrinólogo con experiencia en MCG/tecnología en diabetes</t>
         </is>
       </c>
-      <c r="E7" s="62" t="inlineStr">
-        <is>
-          <t>Dra. Janeth Bermeo (propuesta)</t>
-        </is>
-      </c>
+      <c r="E7" s="62" t="n"/>
       <c r="F7" s="41" t="n"/>
-      <c r="G7" s="63" t="inlineStr">
-        <is>
-          <t>Endocrinóloga, Hospital del Río · contacto directo</t>
-        </is>
-      </c>
+      <c r="G7" s="63" t="n"/>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="50" t="n">
@@ -3116,27 +3132,13 @@
       <c r="G10" s="41" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="50" t="n">
-        <v>3</v>
-      </c>
-      <c r="B11" s="39" t="inlineStr">
-        <is>
-          <t>M2 · C3</t>
-        </is>
-      </c>
-      <c r="C11" s="40" t="inlineStr">
-        <is>
-          <t>Nutrición conductual</t>
-        </is>
-      </c>
-      <c r="D11" s="40" t="inlineStr">
-        <is>
-          <t>Nutricionista clínico o psicólogo de la conducta alimentaria</t>
-        </is>
-      </c>
-      <c r="E11" s="41" t="n"/>
-      <c r="F11" s="41" t="n"/>
-      <c r="G11" s="41" t="n"/>
+      <c r="A11" s="55" t="n"/>
+      <c r="B11" s="52" t="n"/>
+      <c r="C11" s="53" t="n"/>
+      <c r="D11" s="53" t="n"/>
+      <c r="E11" s="53" t="n"/>
+      <c r="F11" s="53" t="n"/>
+      <c r="G11" s="53" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="50" t="n">

</xml_diff>

<commit_message>
Matriz: Dr. Chen Ku acepta M6-C3, vacantes 9 -> 8
El Dr. Chih Hao Chen Ku respondio el 22/09/2026 aceptando las dos clases
del Modulo 6 (C2 Riesgo cardiovascular y C3 Sindrome cardiorrenometabolico,
esta ultima en reemplazo del Dr. Harold, que declino el 19/09/2026).
Confirma la fecha de entrega del 26/11/2026 y adjunta su declaracion de
conflicto de interes.

- Matriz 28 clases: M6-C3 pasa de VACANTE a CONFIRMADO
- Ponentes - datos aval: Chen Ku queda con M6-C2 y M6-C3, COI recibida
- Vacantes por cubrir: M6-C3 marcada como cubierta

Resumen recalculado y verificado: 28 = 10 confirmadas + 10 por confirmar
+ 8 vacantes. Modulo 6 queda completo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1911,10 +1911,14 @@
           <t>Conceptos actuales; insuficiencia cardíaca; beneficios CV y renales de nuevas terapias</t>
         </is>
       </c>
-      <c r="E25" s="28" t="n"/>
-      <c r="F25" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Dr. Chih Hao Chen Ku</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G25" s="23" t="n">
@@ -1922,7 +1926,7 @@
       </c>
       <c r="H25" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. El Dr. Harold declinó (19/09/2026). Candidato natural: Dr. Chen Ku coordina el grupo de complicaciones cardio-reno-metabólicas de ALAD y ya está en M6·C2.</t>
+          <t>Aceptó el 22/09/2026 por correo, en reemplazo del Dr. Harold (declinó 19/09/2026). Segunda clase del mismo docente. Graba él y envía enlace del video. Faltan pasaporte y fotografía.</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2571,7 @@
       <c r="H10" s="41" t="n"/>
       <c r="I10" s="40" t="inlineStr">
         <is>
-          <t>M6 · C2</t>
+          <t>M6 · C2  /  M6 · C3</t>
         </is>
       </c>
       <c r="J10" s="54" t="inlineStr">
@@ -2576,8 +2580,16 @@
         </is>
       </c>
       <c r="K10" s="42" t="n"/>
-      <c r="L10" s="42" t="n"/>
-      <c r="M10" s="42" t="n"/>
+      <c r="L10" s="42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="M10" s="42" t="inlineStr">
+        <is>
+          <t>26/11/2026</t>
+        </is>
+      </c>
       <c r="N10" s="43" t="inlineStr">
         <is>
           <t>CONFIRMADO</t>
@@ -2907,7 +2919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3184,9 +3196,21 @@
           <t>Endocrinología o cardiología — el Dr. Harold declinó el 19/09/2026</t>
         </is>
       </c>
-      <c r="E13" s="59" t="n"/>
-      <c r="F13" s="59" t="n"/>
-      <c r="G13" s="59" t="n"/>
+      <c r="E13" s="59" t="inlineStr">
+        <is>
+          <t>Dr. Chih Hao Chen Ku</t>
+        </is>
+      </c>
+      <c r="F13" s="59" t="inlineStr">
+        <is>
+          <t>chenku2409@gmail.com · +506 8392 7083</t>
+        </is>
+      </c>
+      <c r="G13" s="59" t="inlineStr">
+        <is>
+          <t>CUBIERTA — aceptó el 22/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="C14" s="51" t="inlineStr">
@@ -3195,11 +3219,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Matriz: WhatsApp de la Dra. Janeth Bermeo
Con este numero el cuerpo docente queda con telefono completo: 15 de 15.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2894,7 +2894,11 @@
         </is>
       </c>
       <c r="E18" s="41" t="n"/>
-      <c r="F18" s="41" t="n"/>
+      <c r="F18" s="41" t="inlineStr">
+        <is>
+          <t>+593 96 198 1203</t>
+        </is>
+      </c>
       <c r="G18" s="41" t="n"/>
       <c r="H18" s="41" t="n"/>
       <c r="I18" s="54" t="inlineStr">

</xml_diff>

<commit_message>
M7-C4 la asume la Dra. Omidres: vacantes de 8 a 7
Implementacion, etica y seguridad de datos (Modulo 7, Clase 4) queda a
cargo de la Dra. Omidres, que ya dicta M7-C1. Entrega de la grabacion:
3 de diciembre.

- Matriz 28 clases: M7-C4 pasa de VACANTE a CONFIRMADO.
- Ponentes - datos aval: sus clases pasan a M7-C1 / M7-C4.
- Vacantes por cubrir: M7-C4 marcada como cubierta.
- whatsapp-nuevos-ponentes.md: el tema sale de la version de salud
  digital, que pasa de tres opciones a dos, y de la tabla de urgencias.

Resumen recalculado y verificado: 28 = 11 confirmadas + 10 por confirmar
+ 7 vacantes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2087,10 +2087,14 @@
           <t>Programas híbridos (teleconsulta y telenutrición); protección de datos; interoperabilidad</t>
         </is>
       </c>
-      <c r="E30" s="28" t="inlineStr"/>
-      <c r="F30" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>Dra. Omidres Pérez de Carvelli</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G30" s="23" t="n">
@@ -2098,7 +2102,7 @@
       </c>
       <c r="H30" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: bioética / derecho sanitario o protección de datos en salud.</t>
+          <t>Asumida por la Dra. Omidres el 23/09/2026. Segunda clase de la misma docente en el módulo 7. Entrega de la grabación: 3 de diciembre.</t>
         </is>
       </c>
     </row>
@@ -2327,13 +2331,17 @@
       <c r="H4" s="41" t="n"/>
       <c r="I4" s="40" t="inlineStr">
         <is>
-          <t>M7 · C1</t>
+          <t>M7 · C1  /  M7 · C4</t>
         </is>
       </c>
       <c r="J4" s="42" t="n"/>
       <c r="K4" s="42" t="n"/>
       <c r="L4" s="42" t="n"/>
-      <c r="M4" s="42" t="n"/>
+      <c r="M4" s="42" t="inlineStr">
+        <is>
+          <t>03/12/2026</t>
+        </is>
+      </c>
       <c r="N4" s="43" t="inlineStr">
         <is>
           <t>CONFIRMADO</t>
@@ -3148,9 +3156,21 @@
           <t>Bioética, derecho sanitario o protección de datos en salud</t>
         </is>
       </c>
-      <c r="E9" s="41" t="n"/>
-      <c r="F9" s="41" t="n"/>
-      <c r="G9" s="41" t="n"/>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>Dra. Omidres Pérez de Carvelli</t>
+        </is>
+      </c>
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>info@draomidresperez.com</t>
+        </is>
+      </c>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>CUBIERTA — la asume la Dra. Omidres (23/09/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="32" customHeight="1">
       <c r="A10" s="50" t="n">

</xml_diff>

<commit_message>
Especialidad de cuatro docentes mas: endocrinologia
La Dra. Omidres confirma que son endocrinologos el Dr. Vanegas, la Dra.
Astudillo, la Dra. Jimenez y el Dr. Molina. Se registran en la matriz.

Los otros tres que menciono ya constaban y no se tocaron, porque su
registro es mas preciso: Dra. Ruilova (Endocrinologia y Medicina Interna),
Dr. Chen Ku (Endocrinologia y Farmacologia) y Dra. Bermeo (Endocrinologia).

Siguen sin especialidad registrada cuatro: Espinoza, Cuatecontzi, Alvarez
y Andrade. Son precisamente aquellos de los que no hay hoja de vida.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2713,7 +2713,11 @@
           <t>Dr. Pablo Vanegas</t>
         </is>
       </c>
-      <c r="C13" s="41" t="n"/>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Endocrinología</t>
+        </is>
+      </c>
       <c r="D13" s="41" t="n"/>
       <c r="E13" s="60" t="inlineStr">
         <is>
@@ -2751,7 +2755,11 @@
           <t>Dra. María Augusta Astudillo</t>
         </is>
       </c>
-      <c r="C14" s="41" t="n"/>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>Endocrinología</t>
+        </is>
+      </c>
       <c r="D14" s="41" t="n"/>
       <c r="E14" s="41" t="n"/>
       <c r="F14" s="60" t="inlineStr">
@@ -2785,7 +2793,11 @@
           <t>Dra. Gabriela Jiménez</t>
         </is>
       </c>
-      <c r="C15" s="41" t="n"/>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Endocrinología</t>
+        </is>
+      </c>
       <c r="D15" s="41" t="n"/>
       <c r="E15" s="41" t="n"/>
       <c r="F15" s="60" t="inlineStr">
@@ -2819,7 +2831,11 @@
           <t>Dr. Juan Molina</t>
         </is>
       </c>
-      <c r="C16" s="41" t="n"/>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>Endocrinología</t>
+        </is>
+      </c>
       <c r="D16" s="41" t="n"/>
       <c r="E16" s="41" t="n"/>
       <c r="F16" s="60" t="inlineStr">

</xml_diff>

<commit_message>
Especialidad de la Lcda. Reinoso y la Dra. Piedra
Correccion de la Dra. Omidres: la Lcda. Reinoso es nutriologa y la Dra.
Piedra es nutriologa y diabetologa. Antes constaban como «Nutricion
clinica», que era una lectura mia, no un dato de sus hojas de vida.

En la Dra. Piedra se conserva ademas «Magister en Diabetes», que si viene
de su hoja de vida.

Quedan cuatro sin especialidad: Espinoza, Cuatecontzi, Alvarez y Andrade.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2359,7 +2359,7 @@
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
-          <t>Nutrición clínica</t>
+          <t>Nutriología</t>
         </is>
       </c>
       <c r="D5" s="41" t="n"/>
@@ -2397,7 +2397,7 @@
       </c>
       <c r="C6" s="53" t="inlineStr">
         <is>
-          <t>Nutrición clínica · Magíster en Diabetes</t>
+          <t>Nutriología y Diabetología · Magíster en Diabetes</t>
         </is>
       </c>
       <c r="D6" s="53" t="inlineStr">

</xml_diff>

<commit_message>
Tres invitaciones enviadas y una version formal para M5-C1
Quedan registradas en la hoja «Vacantes por cubrir» las tres invitaciones
que la Dra. Omidres ya envio el 23/09 y cuya respuesta espera:

- M2-C4 Actividad fisica    -> Dr. Cesar Dommar, fisioterapeuta
- M3-C4 Cirugia bariatrica  -> Dr. Verdugo, cirujano
- M5-C2 Estrategias nutric. -> Gaby Villavicencio, nutriologa

Las clases siguen como VACANTE, no como confirmadas: nadie ha respondido
todavia. El estado aparece ahora en la tarjeta de cada vacante en la
pagina HTML, leido de la matriz.

M5-C1 pasa a registro formal, a peticion de la Dra. Omidres: trato de
usted, presentacion de SEDA y firma institucional, para cuando no hay
trato previo. El generador admite ahora los dos registros por tema.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3080,9 +3080,17 @@
           <t>Nutricionista clínico con experiencia en diabetes</t>
         </is>
       </c>
-      <c r="E5" s="41" t="n"/>
+      <c r="E5" s="41" t="inlineStr">
+        <is>
+          <t>Gaby Villavicencio — nutrióloga</t>
+        </is>
+      </c>
       <c r="F5" s="41" t="n"/>
-      <c r="G5" s="41" t="n"/>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>INVITADO 23/09/2026 · esperando respuesta</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="50" t="n">
@@ -3207,9 +3215,17 @@
           <t>Cirujano bariátrico y metabólico acreditado</t>
         </is>
       </c>
-      <c r="E10" s="41" t="n"/>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>Dr. Verdugo — cirujano</t>
+        </is>
+      </c>
       <c r="F10" s="41" t="n"/>
-      <c r="G10" s="41" t="n"/>
+      <c r="G10" s="41" t="inlineStr">
+        <is>
+          <t>INVITADO 23/09/2026 · esperando respuesta</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="55" t="n"/>
@@ -3239,9 +3255,17 @@
           <t>Medicina del deporte, fisiatría o fisioterapia</t>
         </is>
       </c>
-      <c r="E12" s="41" t="n"/>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Dr. César Dommar — fisioterapeuta</t>
+        </is>
+      </c>
       <c r="F12" s="41" t="n"/>
-      <c r="G12" s="41" t="n"/>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>INVITADO 23/09/2026 · esperando respuesta</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="56" t="inlineStr">

</xml_diff>

<commit_message>
Cuarta invitacion enviada: Lcda. Daniela Vintimilla para M5-C1
La Dra. Omidres invito a la Lcda. Daniela Vintimilla, Directora de la
Carrera de Nutricion de la Universidad de Cuenca, a dictar «Nutricion de
precision en diabetes y obesidad» (Modulo 5, Clase 1), con la version
formal del mensaje.

Cuatro de las siete vacantes tienen ya invitacion enviada y esperan
respuesta. Ninguna se cuenta como confirmada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3057,9 +3057,17 @@
           <t>Nutricionista clínico o endocrinólogo con línea en nutrición de precisión</t>
         </is>
       </c>
-      <c r="E4" s="41" t="n"/>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Lcda. Daniela Vintimilla — Directora de la Carrera de Nutrición, Universidad de Cuenca</t>
+        </is>
+      </c>
       <c r="F4" s="41" t="n"/>
-      <c r="G4" s="41" t="n"/>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>INVITADA 23/09/2026 (registro formal) · esperando respuesta</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="50" t="n">

</xml_diff>

<commit_message>
Actividad fisica y cirugia bariatrica ya tienen ponente
- M2-C4 Actividad fisica: el Dr. Cesar Dommar declino. La toma la Dra.
  Julia Castro (24/09). Es la entrega mas apretada del curso, el 29 de
  octubre, y de ella no tenemos ni especialidad ni contacto.
- M3-C4 Cirugia bariatrica: el Dr. Verdugo no respondio, con lo que se
  disuelve la duplicidad. La toma el Dr. Cristian Castillo, que habia
  aceptado via Lizbeth.

Resumen recalculado y verificado: 28 = 13 confirmadas + 10 por confirmar
+ 5 vacantes. Cuerpo docente de 18 personas; los rangos de las formulas
se extienden hasta la fila 21.

Quedan tres temas sin gestionar (M5-C3 y los dos de salud digital) y dos
con invitacion enviada sin respuesta (M5-C1 y M5-C2).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="17">
-        <f>COUNTA('Ponentes - datos aval'!B4:B20)</f>
+        <f>COUNTA('Ponentes - datos aval'!B4:B21)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!J4:J20,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!J4:J21,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="17">
-        <f>COUNTA('Ponentes - datos aval'!F4:F20)</f>
+        <f>COUNTA('Ponentes - datos aval'!F4:F21)</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!L4:L20,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!L4:L21,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -1375,10 +1375,14 @@
           <t>Ejercicio aeróbico; entrenamiento de fuerza; prescripción de ejercicio</t>
         </is>
       </c>
-      <c r="E10" s="28" t="inlineStr"/>
-      <c r="F10" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E10" s="64" t="inlineStr">
+        <is>
+          <t>Dra. Julia Castro</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G10" s="23" t="n">
@@ -1386,7 +1390,7 @@
       </c>
       <c r="H10" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: medicina del deporte o fisiatría / fisioterapia.</t>
+          <t>Aceptó el 24/09/2026. El Dr. César Dommar, invitado el 23/09, declinó. Faltan especialidad, datos de contacto y toda la documentación del aval. Entrega de la grabación: 29 de octubre, la fecha más apretada del curso.</t>
         </is>
       </c>
     </row>
@@ -1519,10 +1523,14 @@
           <t>Indicaciones; técnicas quirúrgicas; seguimiento metabólico</t>
         </is>
       </c>
-      <c r="E14" s="28" t="inlineStr"/>
-      <c r="F14" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>Dr. Cristian Castillo</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G14" s="23" t="n">
@@ -1530,7 +1538,7 @@
       </c>
       <c r="H14" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: cirujano bariátrico/metabólico acreditado.</t>
+          <t>Aceptó vía Dra. Lizbet Ruilova (24/09/2026). El Dr. Verdugo, invitado el 23/09, no respondió. Faltan datos de contacto y documentación del aval.</t>
         </is>
       </c>
     </row>
@@ -2995,7 +3003,7 @@
       <c r="H20" s="41" t="n"/>
       <c r="I20" s="54" t="inlineStr">
         <is>
-          <t>M3 · C4 (en conflicto con el Dr. Verdugo)</t>
+          <t>M3 · C4</t>
         </is>
       </c>
       <c r="J20" s="42" t="n"/>
@@ -3004,12 +3012,39 @@
       <c r="M20" s="42" t="n"/>
       <c r="N20" s="65" t="inlineStr">
         <is>
-          <t>ACEPTÓ — falta resolver duplicidad y datos de contacto</t>
+          <t>CONFIRMADO — faltan datos de contacto y documentación</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="48" t="n"/>
+      <c r="A21" s="54" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Julia Castro</t>
+        </is>
+      </c>
+      <c r="C21" s="53" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="41" t="n"/>
+      <c r="G21" s="41" t="n"/>
+      <c r="H21" s="41" t="n"/>
+      <c r="I21" s="54" t="inlineStr">
+        <is>
+          <t>M2 · C4</t>
+        </is>
+      </c>
+      <c r="J21" s="42" t="n"/>
+      <c r="K21" s="42" t="n"/>
+      <c r="L21" s="42" t="n"/>
+      <c r="M21" s="42" t="n"/>
+      <c r="N21" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — faltan especialidad, contacto y documentación</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3277,13 +3312,13 @@
       </c>
       <c r="E10" s="41" t="inlineStr">
         <is>
-          <t>CONFLICTO: Dr. Verdugo (invitado por Omidres) y Dr. Cristian Castillo (aceptó vía Lizbeth)</t>
+          <t>Dr. Cristian Castillo</t>
         </is>
       </c>
       <c r="F10" s="41" t="n"/>
       <c r="G10" s="41" t="inlineStr">
         <is>
-          <t>DOS CANDIDATOS PARA UNA CLASE · resolver antes de pedirles documentos</t>
+          <t>CUBIERTA — aceptó el 24/09/2026 (el Dr. Verdugo no respondió)</t>
         </is>
       </c>
     </row>
@@ -3317,13 +3352,13 @@
       </c>
       <c r="E12" s="41" t="inlineStr">
         <is>
-          <t>Dr. César Dommar — fisioterapeuta</t>
+          <t>Dra. Julia Castro</t>
         </is>
       </c>
       <c r="F12" s="41" t="n"/>
       <c r="G12" s="41" t="inlineStr">
         <is>
-          <t>INVITADO 23/09/2026 · esperando respuesta</t>
+          <t>CUBIERTA — aceptó el 24/09/2026 (el Dr. Dommar declinó)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
La Lcda. Vintimilla declina pero abre la Carrera de Nutricion
Respondio el 24/09 por WhatsApp: no dicta conferencias, pero propone a la
Lcda. Gabriela Molina para nutricion de precision y ofrece consultar a
otros docentes de la Carrera si se le pasa la lista de temas.

- Matriz: M5-C1 queda con la Lcda. Gabriela Molina como candidata
  propuesta, pendiente de contactar.
- whatsapp-daniela-vintimilla-temas.md (nuevo): la lista prometida, en
  registro formal.

Se le ofrecen tres temas, no los cinco. Se retiene M5-C2 porque hay una
invitacion sin responder con Gaby Villavicencio y ofrecerlo ahora podria
dejar a dos personas preparando la misma clase; y M7-C2 porque su perfil
es endocrinologico y esta reservado para la Dra. Maria Paz Castillo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3146,13 +3146,13 @@
       </c>
       <c r="E4" s="41" t="inlineStr">
         <is>
-          <t>Lcda. Daniela Vintimilla — Directora de la Carrera de Nutrición, Universidad de Cuenca</t>
+          <t>Lcda. Gabriela Molina — propuesta por la Lcda. Daniela Vintimilla</t>
         </is>
       </c>
       <c r="F4" s="41" t="n"/>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>INVITADA 23/09/2026 (registro formal) · esperando respuesta</t>
+          <t>La Lcda. Vintimilla declinó el 24/09 («no suelo dar conferencias») y propuso a la Lcda. Gabriela Molina, con experiencia en el tema. Falta contactarla. La Carrera de Nutrición de la U. Cuenca ofrece más docentes: pidió la lista de temas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Lista para la Carrera de Nutricion: entra M5-C2, sale M7-C3
Por instruccion de la Dra. Omidres. Los tres temas que se le ofrecen a la
Lcda. Vintimilla son ahora los tres del modulo 5, todos de nutricion y
todos con entrega el 19 de noviembre: si la Carrera aporta tres docentes,
el modulo queda cerrado de una vez.

Queda anotado el riesgo: la invitacion a la Dra. Gaby Villavicencio para
M5-C2 sigue viva y sin respuesta desde el 23/09.

Ademas, la Dra. Janneth Bermeo Cabrera envio su hoja de vida el 24/09 y
tiene la declaracion de conflicto de interes llena, a falta de firma
electronica. Se corrige su nombre, se registra su correo y su titulacion
completa: Medicina Interna, subespecialista en Endocrinologia, alta
especialidad en Obesidad y Enfermedades Tiroideas (UNAM).

Hojas de vida recibidas: de 4 a 5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2912,12 +2912,12 @@
       </c>
       <c r="B18" s="52" t="inlineStr">
         <is>
-          <t>Dra. Janeth Bermeo</t>
+          <t>Dra. Janneth Bermeo Cabrera</t>
         </is>
       </c>
       <c r="C18" s="53" t="inlineStr">
         <is>
-          <t>Endocrinología</t>
+          <t>Medicina Interna · Subespecialista en Endocrinología · Alta especialidad en Obesidad y Enfermedades Tiroideas (UNAM)</t>
         </is>
       </c>
       <c r="D18" s="53" t="inlineStr">
@@ -2925,7 +2925,11 @@
           <t>Hospital del Río · Cuenca, Ecuador</t>
         </is>
       </c>
-      <c r="E18" s="41" t="n"/>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>jbendocrino@hotmail.com</t>
+        </is>
+      </c>
       <c r="F18" s="41" t="inlineStr">
         <is>
           <t>+593 96 198 1203</t>
@@ -2938,13 +2942,17 @@
           <t>M2 · C3</t>
         </is>
       </c>
-      <c r="J18" s="42" t="n"/>
+      <c r="J18" s="42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="K18" s="42" t="n"/>
       <c r="L18" s="42" t="n"/>
       <c r="M18" s="42" t="n"/>
       <c r="N18" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO</t>
+          <t>CONFIRMADO — declaración COI llena, pendiente de firma electrónica</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
La Lcda. Gabriela Molina acepta M5-C1
Aceptó el 28/09. La propuso la Lcda. Daniela Vintimilla, y su unica
condicion fue que hubiera certificado de participacion.

- Matriz: M5-C1 pasa a CONFIRMADO. Se incorpora como docente 19 con su
  WhatsApp; los rangos de las formulas llegan ya a la fila 22.
- whatsapp-gabriela-molina-detalles.md: los detalles que la Dra. Omidres
  quedo en pasarle, con la delimitacion de su clase, los documentos que
  faltan y una aclaracion sobre el certificado.

Esa aclaracion importa: acepto por el certificado, y el aval de la
Universidad esta en tramite, no resuelto. El mensaje se lo dice de frente
y precisa que el certificado de SEDA sale en cualquier caso.

Resumen verificado: 28 = 14 confirmadas + 8 por confirmar + 6 vacantes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="17">
-        <f>COUNTA('Ponentes - datos aval'!B4:B21)</f>
+        <f>COUNTA('Ponentes - datos aval'!B4:B22)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!J4:J21,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!J4:J22,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="17">
-        <f>COUNTA('Ponentes - datos aval'!F4:F21)</f>
+        <f>COUNTA('Ponentes - datos aval'!F4:F22)</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!L4:L21,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!L4:L22,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -1703,10 +1703,14 @@
           <t>Fenotipos metabólicos; individualización nutricional</t>
         </is>
       </c>
-      <c r="E19" s="28" t="inlineStr"/>
-      <c r="F19" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E19" s="64" t="inlineStr">
+        <is>
+          <t>Lcda. Gabriela Molina</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G19" s="23" t="n">
@@ -1714,7 +1718,7 @@
       </c>
       <c r="H19" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Módulo 5 es el más descubierto: 3 de 4 clases vacías.</t>
+          <t>Aceptó el 28/09/2026. La propuso la Lcda. Daniela Vintimilla, Directora de la Carrera de Nutrición de la U. Cuenca. Condicionó su participación a recibir certificado de docente, que se le confirmó. Faltan sus documentos.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3043,6 +3047,48 @@
       <c r="N21" s="65" t="inlineStr">
         <is>
           <t>CONFIRMADO — faltan especialidad, contacto y documentación</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="54" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>Lcda. Gabriela Molina</t>
+        </is>
+      </c>
+      <c r="C22" s="53" t="inlineStr">
+        <is>
+          <t>Nutrición</t>
+        </is>
+      </c>
+      <c r="D22" s="53" t="inlineStr">
+        <is>
+          <t>MSP · Cuenca, Ecuador (por confirmar el vínculo con la Carrera de Nutrición de la U. Cuenca)</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 551 4286</t>
+        </is>
+      </c>
+      <c r="G22" s="41" t="n"/>
+      <c r="H22" s="41" t="n"/>
+      <c r="I22" s="54" t="inlineStr">
+        <is>
+          <t>M5 · C1</t>
+        </is>
+      </c>
+      <c r="J22" s="42" t="n"/>
+      <c r="K22" s="42" t="n"/>
+      <c r="L22" s="42" t="n"/>
+      <c r="M22" s="42" t="n"/>
+      <c r="N22" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — faltan todos los documentos</t>
         </is>
       </c>
     </row>
@@ -3146,13 +3192,17 @@
       </c>
       <c r="E4" s="41" t="inlineStr">
         <is>
-          <t>Lcda. Gabriela Molina — propuesta por la Lcda. Daniela Vintimilla</t>
-        </is>
-      </c>
-      <c r="F4" s="41" t="n"/>
+          <t>Lcda. Gabriela Molina</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 551 4286</t>
+        </is>
+      </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>La Lcda. Vintimilla declinó el 24/09 («no suelo dar conferencias») y propuso a la Lcda. Gabriela Molina, con experiencia en el tema. Falta contactarla. La Carrera de Nutrición de la U. Cuenca ofrece más docentes: pidió la lista de temas.</t>
+          <t>CUBIERTA — aceptó el 28/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
La Dra. Gabriela Machado acepta M5-C3: el modulo 5 queda casi cerrado
Acepto el 28/09 a traves de la Lcda. Daniela Vintimilla, que lo consulto
con su equipo. Es el segundo docente que llega por esa via en el mismo
dia, despues de la Lcda. Gabriela Molina.

- Matriz: M5-C3 pasa a CONFIRMADO. Se incorpora como docente 20 con su
  WhatsApp; los rangos de las formulas llegan a la fila 23.
- whatsapp-gabriela-machado-detalles.md: primer contacto, porque la Dra.
  Omidres no ha hablado nunca con ella. Incluye presentacion, delimitacion
  de la clase, condiciones y los documentos, entre ellos su especialidad y
  su institucion, que no constan en ningun lado.

Resumen verificado: 28 = 15 confirmadas + 8 por confirmar + 5 vacantes.
Del modulo 5 solo queda libre C2.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="17">
-        <f>COUNTA('Ponentes - datos aval'!B4:B22)</f>
+        <f>COUNTA('Ponentes - datos aval'!B4:B23)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!J4:J22,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!J4:J23,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="17">
-        <f>COUNTA('Ponentes - datos aval'!F4:F22)</f>
+        <f>COUNTA('Ponentes - datos aval'!F4:F23)</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!L4:L22,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!L4:L23,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -1771,10 +1771,14 @@
           <t>Agonistas de GLP-1; tirzepatida; preservación de la masa muscular</t>
         </is>
       </c>
-      <c r="E21" s="28" t="inlineStr"/>
-      <c r="F21" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E21" s="64" t="inlineStr">
+        <is>
+          <t>Dra. Gabriela Machado</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G21" s="23" t="n">
@@ -1782,7 +1786,7 @@
       </c>
       <c r="H21" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Tema de alta demanda; buen candidato para ponente invitado de peso.</t>
+          <t>Aceptó el 28/09/2026, a través de la Lcda. Daniela Vintimilla, que lo consultó con su equipo. Faltan especialidad, institución y toda la documentación.</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3089,6 +3093,40 @@
       <c r="N22" s="65" t="inlineStr">
         <is>
           <t>CONFIRMADO — faltan todos los documentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="54" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Gabriela Machado</t>
+        </is>
+      </c>
+      <c r="C23" s="53" t="n"/>
+      <c r="D23" s="53" t="n"/>
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 502 5774</t>
+        </is>
+      </c>
+      <c r="G23" s="41" t="n"/>
+      <c r="H23" s="41" t="n"/>
+      <c r="I23" s="54" t="inlineStr">
+        <is>
+          <t>M5 · C3</t>
+        </is>
+      </c>
+      <c r="J23" s="42" t="n"/>
+      <c r="K23" s="42" t="n"/>
+      <c r="L23" s="42" t="n"/>
+      <c r="M23" s="42" t="n"/>
+      <c r="N23" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — faltan especialidad, institución y documentación</t>
         </is>
       </c>
     </row>
@@ -3256,9 +3294,21 @@
           <t>Nutricionista clínico o endocrinólogo; tema de alta demanda</t>
         </is>
       </c>
-      <c r="E6" s="62" t="n"/>
-      <c r="F6" s="41" t="n"/>
-      <c r="G6" s="63" t="n"/>
+      <c r="E6" s="62" t="inlineStr">
+        <is>
+          <t>Dra. Gabriela Machado</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 502 5774</t>
+        </is>
+      </c>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>CUBIERTA — aceptó el 28/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="50" t="n">

</xml_diff>

<commit_message>
Dr. Jose Luis Valverde, candidato a M4-C1, y telefono del Dr. Castillo
La Dra. Ruilova avisa el 28/09 que al Dr. Jose Luis Valverde, endocrinologo
del grupo de delegados, todavia no se le ha asignado charla, y que se le
puede escribir.

Se le propone M4-C1, fisiopatologia y clasificacion de la diabetes: de las
cinco vacantes es la unica que calza con un endocrinologo y la unica sin
ningun candidato. Quedo libre el 25/09 al declinarla la Dra. Astudillo y es
la clase que abre el modulo de diabetes.

Tambien se registra el telefono del Dr. Cristian Castillo, ya confirmado en
M3-C4, que faltaba.

La nota de voz confirma ademas que la Dra. Jimenez se queda solo con M4-C3
y la Dra. Astudillo solo con M1-C3, tal como ya constaba.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3006,7 +3006,11 @@
       </c>
       <c r="D20" s="53" t="n"/>
       <c r="E20" s="41" t="n"/>
-      <c r="F20" s="41" t="n"/>
+      <c r="F20" s="41" t="inlineStr">
+        <is>
+          <t>+593 97 965 3154</t>
+        </is>
+      </c>
       <c r="G20" s="41" t="n"/>
       <c r="H20" s="41" t="n"/>
       <c r="I20" s="54" t="inlineStr">
@@ -3020,7 +3024,7 @@
       <c r="M20" s="42" t="n"/>
       <c r="N20" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — faltan datos de contacto y documentación</t>
+          <t>CONFIRMADO — falta documentación</t>
         </is>
       </c>
     </row>
@@ -3551,11 +3555,19 @@
           <t>Endocrinología o medicina interna</t>
         </is>
       </c>
-      <c r="E15" s="41" t="n"/>
-      <c r="F15" s="41" t="n"/>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>Dr. José Luis Valverde — endocrinólogo</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 111 0822 (móvil) · +593 95 903 2963 (anterior)</t>
+        </is>
+      </c>
       <c r="G15" s="41" t="inlineStr">
         <is>
-          <t>Astudillo declinó 25/09 · SIN CANDIDATO</t>
+          <t>Propuesto por la Dra. Lizbet Ruilova el 28/09: está en el grupo de delegados y todavía no tiene charla asignada. PENDIENTE DE INVITAR.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Telefono de la Dra. Adriana Gonzalez
+593 99 602 1221, enviado por la Dra. Adriana Alvarez. Verificado que no
choca con ningun numero ya registrado. Con esto la invitacion a M1-C4 se
puede enviar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3452,12 +3452,12 @@
       </c>
       <c r="F11" s="41" t="inlineStr">
         <is>
-          <t>contacto enviado por la Dra. Adriana Alvarez</t>
+          <t>+593 99 602 1221</t>
         </is>
       </c>
       <c r="G11" s="41" t="inlineStr">
         <is>
-          <t>Jiménez declinó 25/09 · candidata con charla ya preparada</t>
+          <t>Jiménez declinó 25/09 · candidata con charla ya preparada · PENDIENTE DE INVITAR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
La Dra. Adriana Alvarez lleva tilde: Álvarez
Su tarjeta de contacto la escribe con tilde. Se corrige en la matriz, en
la hoja de clases y en los archivos que la nombran, porque ese nombre va
impreso en el certificado del aval.

Su numero, +54 9 11 6708-1708, coincide con el que ya constaba desde el
23/09.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1957,7 +1957,7 @@
       </c>
       <c r="E26" s="24" t="inlineStr">
         <is>
-          <t>Dra. Adriana Alvarez</t>
+          <t>Dra. Adriana Álvarez</t>
         </is>
       </c>
       <c r="F26" s="27" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="B11" s="39" t="inlineStr">
         <is>
-          <t>Dra. Adriana Alvarez</t>
+          <t>Dra. Adriana Álvarez</t>
         </is>
       </c>
       <c r="C11" s="41" t="n"/>

</xml_diff>

<commit_message>
M6-C4 se queda con MASLD; la sarcopenia pasa a M1-C4
Decision de la Dra. Omidres: la Dra. Adriana Alvarez habla de MASLD y la
Dra. Adriana Gonzalez de sarcopenia.

- El tema de M6-C4 pasa de «MASLD, sarcopenia y complicaciones
  metabolicas» a «MASLD y complicaciones metabolicas», y sus contenidos
  declarados pierden la obesidad sarcopenica.
- La delimitacion de esa clase se actualiza en consecuencia.

Con esto la sarcopenia queda en dos clases del programa y no en tres:
M1-C4, que la da en general, y M5-C4, que la aplica al paciente con
diabetes. Se cierra uno de los seis solapamientos detectados el 24/09.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1947,12 +1947,12 @@
       </c>
       <c r="C26" s="24" t="inlineStr">
         <is>
-          <t>MASLD, sarcopenia y complicaciones metabólicas</t>
+          <t>MASLD y complicaciones metabólicas</t>
         </is>
       </c>
       <c r="D26" s="24" t="inlineStr">
         <is>
-          <t>MASLD; obesidad sarcopénica; enfermedad osteomuscular; estrategias integrales</t>
+          <t>MASLD; enfermedad osteomuscular asociada a la obesidad; estrategias integrales</t>
         </is>
       </c>
       <c r="E26" s="24" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="H26" s="24" t="inlineStr">
         <is>
-          <t>La Dra. Adriana Alvarez confirma MASLD pero NO sarcopenia (25/09/2026). Propuso a la Dra. Adriana González para el tema de sarcopenia. RECOMENDACIÓN: sacar «sarcopenia» del título de esta clase, ya que el programa la cubre en M1 · C4 y M5 · C4. Faltan sus datos y documentación.</t>
+          <t>La Dra. Adriana Álvarez dicta MASLD. La sarcopenia sale de esta clase por decisión de la Dra. Omidres (28/09/2026): la asume la Dra. Adriana González en M1 · C4. Faltan los datos y la documentación de la Dra. Álvarez.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Datos de la Dra. Adriana Mabel Alvarez y su declaracion prellenada
Envio pasaporte, credenciales y la foto de su firma, porque no tiene
impresora. El .docx que adjunto era nuestra plantilla en blanco: no llego
nada lleno.

- Matriz: nombre legal completo, pasaporte AAI843846, DNI, Hospital
  Italiano de Buenos Aires y sus cargos en SAD y ALAD.
- SEDA_COI_Adriana_Alvarez_prellenada.docx (nuevo): el formato con todos
  sus datos cargados y marcada la casilla de «sin conflicto de interes»,
  que es lo que declaro. Queda por pegar su firma y devolverlo.

Sigue faltandole hoja de vida, fotografia profesional y la declaracion ya
firmada. La foto del pasaporte no sirve para el expediente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2630,13 +2630,17 @@
       </c>
       <c r="B11" s="39" t="inlineStr">
         <is>
-          <t>Dra. Adriana Álvarez</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="n"/>
+          <t>Dra. Adriana Mabel Álvarez</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Endocrinología · Comité de Esteatosis Hepática Metabólica (SAD) · Coordinadora del Grupo Obesidad-MASH de ALAD · Vocal Región Sur de ALAD</t>
+        </is>
+      </c>
       <c r="D11" s="41" t="inlineStr">
         <is>
-          <t>Argentina (institución y ciudad por confirmar)</t>
+          <t>Hospital Italiano de Buenos Aires · Buenos Aires, Argentina</t>
         </is>
       </c>
       <c r="E11" s="41" t="n"/>
@@ -2645,20 +2649,36 @@
           <t>+54 9 11 6708-1708</t>
         </is>
       </c>
-      <c r="G11" s="41" t="n"/>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>Pasaporte AAI843846 (vence 28/03/2033) · DNI 14.456.727</t>
+        </is>
+      </c>
       <c r="H11" s="41" t="n"/>
       <c r="I11" s="40" t="inlineStr">
         <is>
-          <t>M6 · C4 (solo MASLD y complicaciones metabólicas)</t>
+          <t>M6 · C4 (MASLD y complicaciones metabólicas)</t>
         </is>
       </c>
       <c r="J11" s="42" t="n"/>
-      <c r="K11" s="42" t="n"/>
-      <c r="L11" s="42" t="n"/>
-      <c r="M11" s="42" t="n"/>
+      <c r="K11" s="42" t="inlineStr">
+        <is>
+          <t>PARCIAL — solo la del pasaporte</t>
+        </is>
+      </c>
+      <c r="L11" s="42" t="inlineStr">
+        <is>
+          <t>PENDIENTE — declaró sin conflicto de palabra; falta el formato firmado</t>
+        </is>
+      </c>
+      <c r="M11" s="42" t="inlineStr">
+        <is>
+          <t>26/11/2026</t>
+        </is>
+      </c>
       <c r="N11" s="43" t="inlineStr">
         <is>
-          <t>CONFIRMADO — declina la parte de sarcopenia</t>
+          <t>CONFIRMADO — faltan hoja de vida, foto profesional y COI firmada</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alvarez con tilde en todas partes
La Dra. Omidres confirma que su apellido lleva tilde, pese a que el
pasaporte lo imprime en mayusculas sin ella. Se corrigen las apariciones
sueltas que la sustitucion anterior no habia alcanzado, porque solo
buscaba el nombre completo: quedaban «Dra. Alvarez» en once archivos y en
una celda de la matriz.

El nombre que ira en el certificado queda fijado como Dra. Adriana Mabel
Álvarez.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D28"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -774,6 +774,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -802,6 +803,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -847,6 +849,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -904,6 +907,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
@@ -1013,6 +1017,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="40" customHeight="1">
       <c r="B28" s="18" t="inlineStr">
         <is>
@@ -1238,7 +1243,7 @@
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>La Dra. Gabriela Jiménez declinó el tema (25/09/2026, vía Lizbet Ruilova): «no quiere sarcopenia». Candidata: Dra. Adriana González, tesorera de ALAD, propuesta por la Dra. Adriana Alvarez — ya tiene preparada una charla de sarcopenia que dictó en Curitiba.</t>
+          <t>La Dra. Gabriela Jiménez declinó el tema (25/09/2026, vía Lizbet Ruilova): «no quiere sarcopenia». Candidata: Dra. Adriana González, tesorera de ALAD, propuesta por la Dra. Adriana Álvarez — ya tiene preparada una charla de sarcopenia que dictó en Curitiba.</t>
         </is>
       </c>
     </row>
@@ -2114,6 +2119,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="C32" s="31" t="inlineStr">
         <is>
@@ -2169,6 +2175,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="C38" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Dra. Gonzalez invitada; Dr. Fabricio propuesto para M7-C3
- M1-C4: la invitacion salio el 29/09. Queda esperando respuesta.
- M7-C3: la Dra. Omidres propone al Dr. Fabricio para el tema de
  inteligencia artificial. Solo se tiene su enlace de LinkedIn
  (linkedin.com/in/fslg); el dominio esta bloqueado por la politica de
  red de este entorno, asi que no se pudo leer el perfil. Faltan su
  nombre completo y un medio de contacto.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="B2:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -774,7 +774,6 @@
     <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -803,7 +802,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -849,7 +847,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -907,7 +904,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
@@ -1017,7 +1013,6 @@
         <v/>
       </c>
     </row>
-    <row r="27"/>
     <row r="28" ht="40" customHeight="1">
       <c r="B28" s="18" t="inlineStr">
         <is>
@@ -2119,7 +2114,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="C32" s="31" t="inlineStr">
         <is>
@@ -2175,7 +2169,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="C38" s="34" t="inlineStr">
         <is>
@@ -3383,9 +3376,17 @@
           <t>Informática médica / IA aplicada a salud</t>
         </is>
       </c>
-      <c r="E8" s="41" t="n"/>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>Dr. Fabricio (apellido por confirmar) — linkedin.com/in/fslg</t>
+        </is>
+      </c>
       <c r="F8" s="41" t="n"/>
-      <c r="G8" s="41" t="n"/>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>Propuesto por la Dra. Omidres el 29/09 · faltan nombre completo y contacto · PENDIENTE DE INVITAR</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="50" t="n">
@@ -3484,7 +3485,7 @@
       </c>
       <c r="G11" s="41" t="inlineStr">
         <is>
-          <t>Jiménez declinó 25/09 · candidata con charla ya preparada · PENDIENTE DE INVITAR</t>
+          <t>INVITADA el 29/09/2026 · esperando respuesta</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dr. Fabrizio Salas, candidato a M7-C3
Su perfil de WhatsApp Business aporta los datos que faltaban: se llama
Fabrizio Salas, con zeta, es medico epidemiologo y experto en salud
digital, y su numero es +593 99 381 4728. Verificado que no choca con
ningun otro numero de la matriz.

El nombre importa: en la conversacion se le habia llamado «Fabricio» y
asi habria salido impreso en el certificado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3378,13 +3378,17 @@
       </c>
       <c r="E8" s="41" t="inlineStr">
         <is>
-          <t>Dr. Fabricio (apellido por confirmar) — linkedin.com/in/fslg</t>
-        </is>
-      </c>
-      <c r="F8" s="41" t="n"/>
+          <t>Dr. Fabrizio Salas — médico epidemiólogo, experto en salud digital</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 381 4728</t>
+        </is>
+      </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>Propuesto por la Dra. Omidres el 29/09 · faltan nombre completo y contacto · PENDIENTE DE INVITAR</t>
+          <t>Propuesto por la Dra. Omidres el 29/09 · PENDIENTE DE INVITAR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dra. Ana Maria Gomez, candidata a M7-C2
Endocrinologa colombiana experta en monitoreo de glucosa, propuesta por la
Dra. Omidres. Encaja con M7-C2, monitoreo digital y tecnologias.

La invitacion delimita su clase desde el primer mensaje, porque el
programa tiene dos clases que tocan monitoreo continuo: M4-C2, que da la
lectura clinica del AGP y las metas, y M7-C2, que da la implementacion
digital. Sin esa precision lo natural seria que desarrolle la lectura del
AGP, que es lo que domina, y pise a la Dra. Palacio, que graba tres
semanas antes.

Queda anotado que, si acepta, el cuerpo docente pasa de cuatro paises
extranjeros a cinco, y el correo a la comision de avales dice hoy cuatro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3353,9 +3353,21 @@
           <t>Endocrinólogo con experiencia en MCG/tecnología en diabetes</t>
         </is>
       </c>
-      <c r="E7" s="62" t="n"/>
-      <c r="F7" s="41" t="n"/>
-      <c r="G7" s="63" t="n"/>
+      <c r="E7" s="62" t="inlineStr">
+        <is>
+          <t>Dra. Ana María Gómez — endocrinóloga, Colombia</t>
+        </is>
+      </c>
+      <c r="F7" s="41" t="inlineStr">
+        <is>
+          <t>+57 310 488 4626</t>
+        </is>
+      </c>
+      <c r="G7" s="63" t="inlineStr">
+        <is>
+          <t>Propuesta por la Dra. Omidres el 29/09: experta en monitoreo de glucosa. PENDIENTE DE INVITAR. Si acepta, sería el QUINTO país extranjero del cuerpo docente y habría que añadir Colombia en el correo a la comisión de avales.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="50" t="n">

</xml_diff>

<commit_message>
M5-C2 se reasigna a la Lcda. Maria Augusta Vasquez
La Dra. Gaby Villavicencio no respondio en seis dias a la invitacion del
23/09, y el tema tampoco lo tomo nadie de la Carrera de Nutricion.

La invitacion incorpora desde el primer mensaje el reparto con M2-C2, que
es el solapamiento mas literal del programa: ambas clases declaran dieta
mediterranea, restriccion de carbohidratos y ayuno intermitente. M2 lo
enfoca en obesidad y M5 en diabetes; la Dra. Piedra entrega tres semanas
antes, asi que sin esa precision las dos grabarian lo mismo.

Queda anotado que ya hay dos Maria Augusta en el cuerpo docente: la Dra.
Astudillo, endocrinologa, en M1-C3, y esta, de nutricion, en M5-C2.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3289,13 +3289,17 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>Gaby Villavicencio — nutrióloga</t>
-        </is>
-      </c>
-      <c r="F5" s="41" t="n"/>
+          <t>Lcda. María Augusta Vásquez — nutrición</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 994 9812</t>
+        </is>
+      </c>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>INVITADO 23/09/2026 · esperando respuesta</t>
+          <t>La Dra. Gaby Villavicencio no respondió en seis días a la invitación del 23/09. Se reasigna la gestión el 29/09. PENDIENTE DE INVITAR.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gomez y Salas aceptan: el modulo 7 queda completo
- M7-C2: la Dra. Ana Maria Gomez, endocrinologa colombiana experta en
  monitoreo de glucosa, confirmo el 29/09. Es el QUINTO pais extranjero
  del cuerpo docente.
- M7-C3: el Dr. Fabrizio Salas confirmo el mismo dia. Negocio el alcance:
  el proponia acotar el tema a un solo punto y la Dra. Omidres pidio el
  panorama general de los tres, porque para el publico del curso estos
  temas «se ven como ciencia ficcion» y hace falta la base. Queda
  registrado en la matriz y en la delimitacion de su clase.

El modulo 7 cierra con Perez (C1 y C4), Gomez (C2) y Salas (C3).

Resumen verificado: 28 = 17 confirmadas + 8 por confirmar + 3 vacantes.
Cuerpo docente de 22 personas, 20 con telefono.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="17">
-        <f>COUNTA('Ponentes - datos aval'!B4:B23)</f>
+        <f>COUNTA('Ponentes - datos aval'!B4:B25)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!J4:J23,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!J4:J25,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="17">
-        <f>COUNTA('Ponentes - datos aval'!F4:F23)</f>
+        <f>COUNTA('Ponentes - datos aval'!F4:F25)</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!L4:L23,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!L4:L25,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -2031,10 +2031,14 @@
           <t>MCG y AGP en entornos digitales; monitoreo remoto (RPM), apps y wearables; salud conectada</t>
         </is>
       </c>
-      <c r="E28" s="28" t="inlineStr"/>
-      <c r="F28" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Dra. Ana María Gómez</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G28" s="23" t="n">
@@ -2042,7 +2046,7 @@
       </c>
       <c r="H28" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Puede asumirlo Dra. Omidres o un invitado en tecnología en diabetes.</t>
+          <t>Aceptó el 29/09/2026. Endocrinóloga, Colombia, experta en monitoreo de glucosa. QUINTO PAÍS EXTRANJERO del cuerpo docente. Se le delimitó su clase frente a M4 · C2 en la propia invitación. Falta toda la documentación.</t>
         </is>
       </c>
     </row>
@@ -2063,10 +2067,14 @@
           <t>Terapias digitales (DTx); IA en tamizaje y apoyo a la decisión; educación digital y adherencia</t>
         </is>
       </c>
-      <c r="E29" s="28" t="inlineStr"/>
-      <c r="F29" s="29" t="inlineStr">
-        <is>
-          <t>VACANTE</t>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Dr. Fabrizio Salas</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G29" s="23" t="n">
@@ -2074,7 +2082,7 @@
       </c>
       <c r="H29" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: informática médica / IA en salud.</t>
+          <t>Aceptó el 29/09/2026. Médico epidemiólogo, experto en salud digital. ALCANCE ACORDADO: panorama general de los tres puntos, no profundizar en uno. Él propuso acotar; la Dra. Omidres pidió el panorama porque para el público del curso estos temas «se ven como ciencia ficción» y hace falta la base. Pidió la plantilla y coordinar fecha. Falta toda la documentación.</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N23"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3151,6 +3159,98 @@
       <c r="N23" s="65" t="inlineStr">
         <is>
           <t>CONFIRMADO — faltan especialidad, institución y documentación</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="54" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Ana María Gómez</t>
+        </is>
+      </c>
+      <c r="C24" s="53" t="inlineStr">
+        <is>
+          <t>Endocrinología · experta en monitoreo de glucosa</t>
+        </is>
+      </c>
+      <c r="D24" s="53" t="inlineStr">
+        <is>
+          <t>Colombia (institución y ciudad por confirmar)</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>+57 310 488 4626</t>
+        </is>
+      </c>
+      <c r="G24" s="41" t="n"/>
+      <c r="H24" s="41" t="n"/>
+      <c r="I24" s="54" t="inlineStr">
+        <is>
+          <t>M7 · C2</t>
+        </is>
+      </c>
+      <c r="J24" s="42" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="42" t="n"/>
+      <c r="M24" s="42" t="inlineStr">
+        <is>
+          <t>03/12/2026</t>
+        </is>
+      </c>
+      <c r="N24" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — falta toda la documentación</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="54" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>Dr. Fabrizio Salas</t>
+        </is>
+      </c>
+      <c r="C25" s="53" t="inlineStr">
+        <is>
+          <t>Medicina · Epidemiología · Salud digital e interoperabilidad</t>
+        </is>
+      </c>
+      <c r="D25" s="53" t="inlineStr">
+        <is>
+          <t>Ecuador (institución por confirmar)</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 381 4728</t>
+        </is>
+      </c>
+      <c r="G25" s="41" t="n"/>
+      <c r="H25" s="41" t="n"/>
+      <c r="I25" s="54" t="inlineStr">
+        <is>
+          <t>M7 · C3</t>
+        </is>
+      </c>
+      <c r="J25" s="42" t="n"/>
+      <c r="K25" s="42" t="n"/>
+      <c r="L25" s="42" t="n"/>
+      <c r="M25" s="42" t="inlineStr">
+        <is>
+          <t>03/12/2026</t>
+        </is>
+      </c>
+      <c r="N25" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — falta toda la documentación</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3469,7 @@
       </c>
       <c r="G7" s="63" t="inlineStr">
         <is>
-          <t>INVITADA el 29/09/2026 · esperando respuesta. Si acepta, sería el quinto país extranjero y habría que añadir Colombia en el correo a la comisión de avales.</t>
+          <t>CUBIERTA — aceptó el 29/09/2026</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3504,7 @@
       </c>
       <c r="G8" s="41" t="inlineStr">
         <is>
-          <t>Propuesto por la Dra. Omidres el 29/09 · PENDIENTE DE INVITAR</t>
+          <t>CUBIERTA — aceptó el 29/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Los seis que faltaban confirmaron: ninguna clase queda sin confirmar
Ruilova, Vanegas, Astudillo, Jimenez, Molina y Andrade confirmaron el
29/09. Son las ocho clases que seguian como POR CONFIRMAR desde el
principio del proyecto.

Resumen verificado: 28 = 25 confirmadas + 0 por confirmar + 3 vacantes.

Se actualiza el grupo de WhatsApp: entran los 20 confirmados con
telefono, no los 14 de hace un rato.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1124,9 +1124,9 @@
           <t>Dra. Lizbet Ruilova</t>
         </is>
       </c>
-      <c r="F3" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F3" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G3" s="23" t="n">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
-          <t>Coordinadora académica. Confirmar por escrito + hoja de vida + declaración COI.</t>
+          <t>Confirmado el 29/09/2026. Coordinadora académica. Confirmar por escrito + hoja de vida + declaración COI.</t>
         </is>
       </c>
     </row>
@@ -1160,9 +1160,9 @@
           <t>Dr. Pablo Vanegas</t>
         </is>
       </c>
-      <c r="F4" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G4" s="23" t="n">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
-          <t>Coordinador académico. Confirmar por escrito + hoja de vida + declaración COI.</t>
+          <t>Confirmado el 29/09/2026. Coordinador académico. Confirmar por escrito + hoja de vida + declaración COI.</t>
         </is>
       </c>
     </row>
@@ -1196,9 +1196,9 @@
           <t>Dra. María Augusta Astudillo</t>
         </is>
       </c>
-      <c r="F5" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G5" s="23" t="n">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="H5" s="24" t="inlineStr">
         <is>
-          <t>Pedir aceptación formal, datos de contacto y hoja de vida.</t>
+          <t>Confirmado el 29/09/2026. Pedir aceptación formal, datos de contacto y hoja de vida.</t>
         </is>
       </c>
     </row>
@@ -1416,9 +1416,9 @@
           <t>Dr. Pablo Vanegas</t>
         </is>
       </c>
-      <c r="F11" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G11" s="23" t="n">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="H11" s="24" t="inlineStr">
         <is>
-          <t>Segunda charla del mismo docente. Confirmar carga y disponibilidad.</t>
+          <t>Confirmado el 29/09/2026. Segunda charla del mismo docente. Confirmar carga y disponibilidad.</t>
         </is>
       </c>
     </row>
@@ -1632,9 +1632,9 @@
           <t>Dra. Gabriela Jiménez</t>
         </is>
       </c>
-      <c r="F17" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G17" s="23" t="n">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="H17" s="24" t="inlineStr">
         <is>
-          <t>Segunda charla del mismo docente. Confirmar carga y disponibilidad.</t>
+          <t>Confirmado el 29/09/2026. Segunda charla del mismo docente. Confirmar carga y disponibilidad.</t>
         </is>
       </c>
     </row>
@@ -1668,9 +1668,9 @@
           <t>Dr. Juan Molina</t>
         </is>
       </c>
-      <c r="F18" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G18" s="23" t="n">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="H18" s="24" t="inlineStr">
         <is>
-          <t>Pedir aceptación formal, datos de contacto y hoja de vida.</t>
+          <t>Confirmado el 29/09/2026. Pedir aceptación formal, datos de contacto y hoja de vida.</t>
         </is>
       </c>
     </row>
@@ -1812,9 +1812,9 @@
           <t>Dra. Lizbet Ruilova</t>
         </is>
       </c>
-      <c r="F22" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F22" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G22" s="23" t="n">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="H22" s="24" t="inlineStr">
         <is>
-          <t>Segunda charla de la coordinadora. Revisar solapamiento con M1·C4 (Dra. Jiménez).</t>
+          <t>Confirmado el 29/09/2026. Segunda charla de la coordinadora. Revisar solapamiento con M1·C4 (Dra. Jiménez).</t>
         </is>
       </c>
     </row>
@@ -1852,9 +1852,9 @@
           <t>Dra. Valeria Andrade</t>
         </is>
       </c>
-      <c r="F23" s="25" t="inlineStr">
-        <is>
-          <t>POR CONFIRMAR</t>
+      <c r="F23" s="27" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G23" s="23" t="n">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="H23" s="24" t="inlineStr">
         <is>
-          <t>Pedir aceptación formal, datos de contacto y hoja de vida.</t>
+          <t>Confirmado el 29/09/2026. Pedir aceptación formal, datos de contacto y hoja de vida.</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       <c r="M12" s="42" t="n"/>
       <c r="N12" s="44" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       <c r="M13" s="42" t="n"/>
       <c r="N13" s="44" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       <c r="M14" s="42" t="n"/>
       <c r="N14" s="44" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR — declinó M4 · C1 el 25/09</t>
+          <t>CONFIRMADO — declinó M4 · C1 el 25/09</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       <c r="M15" s="42" t="n"/>
       <c r="N15" s="44" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR — declinó M1 · C4 el 25/09</t>
+          <t>CONFIRMADO — declinó M1 · C4 el 25/09</t>
         </is>
       </c>
     </row>
@@ -2892,7 +2892,7 @@
       <c r="M16" s="42" t="n"/>
       <c r="N16" s="44" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       <c r="M17" s="42" t="n"/>
       <c r="N17" s="44" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Telefono y especialidad de la Dra. Julia Castro
+593 99 208 7747. Es fisioterapeuta, lo que confirma que su perfil calza
con M2-C4, actividad fisica en obesidad, y cierra el hueco de contacto mas
urgente del proyecto: su entrega es el 29 de octubre, la mas proxima del
curso, y hasta ahora no habia forma de escribirle.

Entra al grupo de WhatsApp, que pasa a 21 miembros. Solo queda sin
telefono la Dra. Maria Paz Castillo, que ademas sigue sin tema asignado.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3065,10 +3065,18 @@
           <t>Dra. Julia Castro</t>
         </is>
       </c>
-      <c r="C21" s="53" t="n"/>
+      <c r="C21" s="53" t="inlineStr">
+        <is>
+          <t>Fisioterapia</t>
+        </is>
+      </c>
       <c r="D21" s="53" t="n"/>
       <c r="E21" s="41" t="n"/>
-      <c r="F21" s="41" t="n"/>
+      <c r="F21" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 208 7747</t>
+        </is>
+      </c>
       <c r="G21" s="41" t="n"/>
       <c r="H21" s="41" t="n"/>
       <c r="I21" s="54" t="inlineStr">
@@ -3079,10 +3087,14 @@
       <c r="J21" s="42" t="n"/>
       <c r="K21" s="42" t="n"/>
       <c r="L21" s="42" t="n"/>
-      <c r="M21" s="42" t="n"/>
+      <c r="M21" s="42" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
       <c r="N21" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — faltan especialidad, contacto y documentación</t>
+          <t>CONFIRMADO — falta documentación · ENTREGA MÁS PRÓXIMA DEL CURSO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
La Dra. Adriana Gonzalez acepta M1-C4: el modulo 1 queda completo
Acepto el 29/09. Es la entrega mas proxima del curso, el 29 de octubre,
porque el modulo 1 abre el programa.

- Matriz: M1-C4 pasa a CONFIRMADO. Entra como docente 23; los rangos de
  las formulas llegan a la fila 26.
- whatsapp-adriana-gonzalez-detalles.md: los detalles de su clase, con la
  fecha subrayada y apoyandose en que ya tiene la charla de Curitiba
  preparada, mas la delimitacion frente a M5-C4, M5-C3 y M2-C4.
- Se regeneran la pagina de documentos y la del grupo de WhatsApp, que
  pasa a 22 integrantes.

Resumen verificado: 28 = 26 confirmadas + 0 por confirmar + 2 vacantes.
Solo quedan M4-C1 y M5-C2, las dos con mensaje redactado sin enviar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="C23" s="16" t="n"/>
       <c r="D23" s="17">
-        <f>COUNTA('Ponentes - datos aval'!B4:B25)</f>
+        <f>COUNTA('Ponentes - datos aval'!B4:B26)</f>
         <v/>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C24" s="16" t="n"/>
       <c r="D24" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!J4:J25,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!J4:J26,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C25" s="16" t="n"/>
       <c r="D25" s="17">
-        <f>COUNTA('Ponentes - datos aval'!F4:F25)</f>
+        <f>COUNTA('Ponentes - datos aval'!F4:F26)</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C26" s="16" t="n"/>
       <c r="D26" s="17">
-        <f>COUNTIF('Ponentes - datos aval'!L4:L25,"SÍ")</f>
+        <f>COUNTIF('Ponentes - datos aval'!L4:L26,"SÍ")</f>
         <v/>
       </c>
     </row>
@@ -1227,10 +1227,14 @@
           <t>IMC y sus limitaciones; circunferencia abdominal; bioimpedancia; obesidad sarcopénica</t>
         </is>
       </c>
-      <c r="E6" s="64" t="n"/>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>Dra. Adriana González</t>
+        </is>
+      </c>
       <c r="F6" s="27" t="inlineStr">
         <is>
-          <t>VACANTE</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G6" s="23" t="n">
@@ -1238,7 +1242,7 @@
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
-          <t>La Dra. Gabriela Jiménez declinó el tema (25/09/2026, vía Lizbet Ruilova): «no quiere sarcopenia». Candidata: Dra. Adriana González, tesorera de ALAD, propuesta por la Dra. Adriana Álvarez — ya tiene preparada una charla de sarcopenia que dictó en Curitiba.</t>
+          <t>Aceptó el 29/09/2026. Tesorera de ALAD, Ecuador. La propuso la Dra. Adriana Álvarez: ya tenía preparada una charla de sarcopenia dictada en Curitiba. ENTREGA MÁS PRÓXIMA DEL CURSO, junto con el resto del módulo 1 y el 2. Falta toda la documentación.</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3261,6 +3265,52 @@
         </is>
       </c>
       <c r="N25" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — falta toda la documentación</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="54" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Adriana González</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="inlineStr">
+        <is>
+          <t>Endocrinología · Tesorera de ALAD</t>
+        </is>
+      </c>
+      <c r="D26" s="53" t="inlineStr">
+        <is>
+          <t>Ecuador (institución y ciudad por confirmar)</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="41" t="inlineStr">
+        <is>
+          <t>+593 99 602 1221</t>
+        </is>
+      </c>
+      <c r="G26" s="41" t="n"/>
+      <c r="H26" s="41" t="n"/>
+      <c r="I26" s="54" t="inlineStr">
+        <is>
+          <t>M1 · C4</t>
+        </is>
+      </c>
+      <c r="J26" s="42" t="n"/>
+      <c r="K26" s="42" t="n"/>
+      <c r="L26" s="42" t="n"/>
+      <c r="M26" s="42" t="inlineStr">
+        <is>
+          <t>29/10/2026</t>
+        </is>
+      </c>
+      <c r="N26" s="65" t="inlineStr">
         <is>
           <t>CONFIRMADO — falta toda la documentación</t>
         </is>
@@ -3617,7 +3667,7 @@
       </c>
       <c r="G11" s="41" t="inlineStr">
         <is>
-          <t>INVITADA el 29/09/2026 · esperando respuesta</t>
+          <t>CUBIERTA — aceptó el 29/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
El programa en PDF, sin nombres de ponentes y con fecha de entrega por clase
Por indicacion de la Dra. Omidres. El documento se publica sin decir quien
dicta cada clase: desaparecen las dos que decian «por asignar» y las
referencias cruzadas quedan solo con el codigo de la clase. Cada clase
lleva ahora su propia fecha de entrega, ademas de la del modulo.

Se corrigen dos cosas detectadas al revisar el PDF generado: se colaba la
marca interna «ATENCION» en varias referencias, y el titulo decia «y quien
lo cubre» cuando ya no hay nombres; ahora dice «y donde se cubre».

Ademas se registra el telefono de la Dra. Maria Paz Castillo Cabrera. Su
prefijo es +52, de Mexico, lo que habria que confirmar antes de darla por
extranjera: con el Dr. Espinoza y la Dra. Alvarez el prefijo resulto
coincidir con el pais, pero no es una regla.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B19" s="52" t="inlineStr">
         <is>
-          <t>Dra. María Paz Castillo</t>
+          <t>Dra. María Paz Castillo Cabrera</t>
         </is>
       </c>
       <c r="C19" s="53" t="inlineStr">
@@ -3002,9 +3002,17 @@
           <t>Endocrinología</t>
         </is>
       </c>
-      <c r="D19" s="53" t="n"/>
+      <c r="D19" s="53" t="inlineStr">
+        <is>
+          <t>Prefijo +52 (México) — CONFIRMAR dónde ejerce antes de darla por extranjera</t>
+        </is>
+      </c>
       <c r="E19" s="41" t="n"/>
-      <c r="F19" s="41" t="n"/>
+      <c r="F19" s="41" t="inlineStr">
+        <is>
+          <t>+52 1 56 2489 0698</t>
+        </is>
+      </c>
       <c r="G19" s="41" t="n"/>
       <c r="H19" s="41" t="n"/>
       <c r="I19" s="54" t="inlineStr">
@@ -3018,7 +3026,7 @@
       <c r="M19" s="42" t="n"/>
       <c r="N19" s="65" t="inlineStr">
         <is>
-          <t>ACEPTÓ — falta tema y datos de contacto</t>
+          <t>ACEPTÓ — sin tema asignado. La Dra. Ruilova pide incluirla (29/09)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M4-C1 para la Dra. Maria Paz Castillo Cabrera: queda una sola vacante
El Dr. Jose Luis Valverde, invitado el 28/09, no respondio, de modo que la
clase quedo libre y no hubo que quitarle ninguna a la Dra. Ruilova, que
habia ofrecido ceder una suya con tal de incluirla.

Es endocrinologia pura y abre el modulo de diabetes: lo que viene despues
—monitoreo, farmacos, insulinoterapia— se apoya en lo que ella plantee.

El mensaje le pide «cedula o pasaporte, segun donde ejerza», sin dar por
hecho que vive en Mexico solo porque su prefijo es +52.

Resumen verificado: 28 = 27 confirmadas + 0 por confirmar + 1 vacante.
Solo queda M5-C2, con la Lcda. Maria Augusta Vasquez pendiente de invitar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1563,10 +1563,14 @@
           <t>Defectos fisiopatológicos de la DM2; clasificación actual; diagnóstico temprano</t>
         </is>
       </c>
-      <c r="E15" s="64" t="n"/>
+      <c r="E15" s="24" t="inlineStr">
+        <is>
+          <t>Dra. María Paz Castillo Cabrera</t>
+        </is>
+      </c>
       <c r="F15" s="27" t="inlineStr">
         <is>
-          <t>VACANTE</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G15" s="23" t="n">
@@ -1574,7 +1578,7 @@
       </c>
       <c r="H15" s="24" t="inlineStr">
         <is>
-          <t>La Dra. María Augusta Astudillo declinó este tema (25/09/2026, vía Lizbet Ruilova). Conserva M1 · C3, que no ha rechazado. SIN CANDIDATO.</t>
+          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. Confirmar si ejerce en México antes de pedirle cédula: su teléfono es +52. Falta toda la documentación.</t>
         </is>
       </c>
     </row>
@@ -3017,16 +3021,20 @@
       <c r="H19" s="41" t="n"/>
       <c r="I19" s="54" t="inlineStr">
         <is>
-          <t>POR ASIGNAR</t>
+          <t>M4 · C1</t>
         </is>
       </c>
       <c r="J19" s="42" t="n"/>
       <c r="K19" s="42" t="n"/>
       <c r="L19" s="42" t="n"/>
-      <c r="M19" s="42" t="n"/>
+      <c r="M19" s="42" t="inlineStr">
+        <is>
+          <t>12/11/2026</t>
+        </is>
+      </c>
       <c r="N19" s="65" t="inlineStr">
         <is>
-          <t>ACEPTÓ — sin tema asignado. La Dra. Ruilova pide incluirla (29/09)</t>
+          <t>CONFIRMADO — falta documentación y confirmar país</t>
         </is>
       </c>
     </row>
@@ -3775,17 +3783,17 @@
       </c>
       <c r="E15" s="41" t="inlineStr">
         <is>
-          <t>Dr. José Luis Valverde — endocrinólogo</t>
+          <t>Dra. María Paz Castillo Cabrera</t>
         </is>
       </c>
       <c r="F15" s="41" t="inlineStr">
         <is>
-          <t>+593 99 111 0822 (móvil) · +593 95 903 2963 (anterior)</t>
+          <t>+52 1 56 2489 0698</t>
         </is>
       </c>
       <c r="G15" s="41" t="inlineStr">
         <is>
-          <t>Propuesto por la Dra. Lizbet Ruilova el 28/09: está en el grupo de delegados y todavía no tiene charla asignada. PENDIENTE DE INVITAR.</t>
+          <t>CUBIERTA — asignada el 29/09/2026 (el Dr. Valverde no respondió)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
María Paz Castillo: ponente internacional en México
Registra en la matriz que la Dra. Castillo ejerce en México (país por
institución y ciudad pendientes) y marca su estado como ponente
internacional, y reescribe su mensaje de WhatsApp en consecuencia:

- pide pasaporte en lugar de «cédula o pasaporte, según dónde ejerza»
- pone institución, ciudad y estado mexicanos al inicio del expediente
- menciona la diferencia horaria con Cuenca al coordinar la grabación
- la sitúa como la segunda colega mexicana del cuerpo docente

Deja anotado que a la Comisión de Avales se le dijo «cuatro ponentes
extranjeros: México, Costa Rica, Perú y Argentina» y que hoy son seis en
cinco países, para revisarlo antes de entregar el expediente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1578,7 +1578,7 @@
       </c>
       <c r="H15" s="24" t="inlineStr">
         <is>
-          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. Confirmar si ejerce en México antes de pedirle cédula: su teléfono es +52. Falta toda la documentación.</t>
+          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. Ejerce en México: ponente internacional, se le pide pasaporte. Falta toda la documentación.</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D19" s="53" t="inlineStr">
         <is>
-          <t>Prefijo +52 (México) — CONFIRMAR dónde ejerce antes de darla por extranjera</t>
+          <t>México (institución y ciudad por confirmar)</t>
         </is>
       </c>
       <c r="E19" s="41" t="n"/>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="N19" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — falta documentación y confirmar país</t>
+          <t>CONFIRMADO — ponente internacional · falta documentación</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
María Paz Castillo: congelar el envío hasta verificar identidad
Podría ser la misma persona vinculada al trámite de avales de la
Universidad de Cuenca. Hasta confirmarlo con la Dra. Ruilova:

- el mensaje queda marcado NO ENVIAR y el borrador de México, congelado
- la matriz deja de afirmar que ejerce en México y pasa a POR VERIFICAR
- se documenta el conflicto de interés y las dos salidas posibles
  (declarar y excusarse del trámite, o no figurar como docente)
- se añade el texto para preguntárselo a la Dra. Ruilova, que fue quien
  la propuso

En la correspondencia archivada del aval ella no aparece: los nombres son
Dra. Nancy Auquilla (Decanato), Dra. Silvia Aguirre (Comisión de Avales)
y Lcda. Fabiola Palacios. El vínculo no se puede confirmar ni descartar
desde los archivos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1578,7 +1578,7 @@
       </c>
       <c r="H15" s="24" t="inlineStr">
         <is>
-          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. Ejerce en México: ponente internacional, se le pide pasaporte. Falta toda la documentación.</t>
+          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. EN ESPERA: verificar con la Dra. Ruilova si es la misma María Paz Castillo vinculada al trámite de avales de la Universidad de Cuenca. Si lo es, hay conflicto de interés que declarar y el teléfono +52 no cuadra. No escribirle hasta aclararlo.</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D19" s="53" t="inlineStr">
         <is>
-          <t>México (institución y ciudad por confirmar)</t>
+          <t>POR VERIFICAR — el teléfono es +52 (México), pero podría ser la misma persona vinculada al trámite de avales en Cuenca</t>
         </is>
       </c>
       <c r="E19" s="41" t="n"/>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="N19" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — ponente internacional · falta documentación</t>
+          <t>CONFIRMADO — identidad y país por verificar con la Dra. Ruilova · posible conflicto de interés</t>
         </is>
       </c>
     </row>
@@ -3332,6 +3332,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="J4:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
María Paz Castillo ejerce en Cuenca: ponente nacional
La Dra. Ruilova confirma el país. El mensaje se rehace en clave
ecuatoriana:

- cédula en lugar de pasaporte
- sin diferencia horaria ni encuadre internacional
- se le ofrece el video tutorial de grabación y el fondo institucional
- el conteo de ponentes internacionales vuelve a cinco en cinco países;
  frente a lo declarado a la Comisión de Avales la única diferencia es
  Colombia

Sigue sin enviarse: Liz contestó el país, no si es la misma persona
vinculada al trámite de avales. Ese punto y las dos salidas posibles
quedan documentados.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1578,7 +1578,7 @@
       </c>
       <c r="H15" s="24" t="inlineStr">
         <is>
-          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. EN ESPERA: verificar con la Dra. Ruilova si es la misma María Paz Castillo vinculada al trámite de avales de la Universidad de Cuenca. Si lo es, hay conflicto de interés que declarar y el teléfono +52 no cuadra. No escribirle hasta aclararlo.</t>
+          <t>Asignada el 29/09/2026 a petición de la Dra. Lizbet Ruilova. El Dr. José Luis Valverde, invitado el 28/09, no respondió. La Dra. Ruilova confirma el 29/09 que ejerce en CUENCA: ponente nacional, se le pide cédula (el +52 es un número mexicano conservado). PENDIENTE: aclarar si es la misma persona vinculada al trámite de avales de la Universidad de Cuenca. No escribirle hasta resolverlo.</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="D19" s="53" t="inlineStr">
         <is>
-          <t>POR VERIFICAR — el teléfono es +52 (México), pero podría ser la misma persona vinculada al trámite de avales en Cuenca</t>
+          <t>Cuenca, Ecuador (institución por confirmar) — confirmado por la Dra. Ruilova el 29/09</t>
         </is>
       </c>
       <c r="E19" s="41" t="n"/>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="N19" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — identidad y país por verificar con la Dra. Ruilova · posible conflicto de interés</t>
+          <t>CONFIRMADO — ponente nacional · PENDIENTE aclarar si interviene en el trámite del aval</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M5C2 se mantiene vacante tras declinar la Lcda. Vásquez
Decisión de la Dra. Omidres. Se deja constancia en la matriz del
historial de la vacante: la Dra. Villavicencio no respondió, la Carrera
de Nutrición no la tomó y la Lcda. Vásquez declinó el 5 de octubre.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1758,7 +1758,7 @@
       </c>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: nutricionista clínico con experiencia en diabetes.</t>
+          <t>SIN PONENTE. Perfil sugerido: nutricionista clínico con experiencia en diabetes. Historial: la Dra. Gaby Villavicencio no respondió (23/09). La Carrera de Nutrición de la U. Cuenca recibió la lista de temas y no lo tomó. La Lcda. María Augusta Vásquez declinó el 05/10. Se mantiene vacante por decisión de la Dra. Omidres.</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3332,7 +3332,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="J4:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Historial completo de la vacante M5C2 en la matriz
Queda registrado quién declinó y con qué número, para no volver a
contactar a las mismas personas por este tema: la Dra. Villavicencio, la
Carrera de Nutrición de la U. Cuenca y la Lcda. Vásquez.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1758,7 +1758,12 @@
       </c>
       <c r="H20" s="24" t="inlineStr">
         <is>
-          <t>SIN PONENTE. Perfil sugerido: nutricionista clínico con experiencia en diabetes. Historial: la Dra. Gaby Villavicencio declinó y recomendó a otras personas, pendientes de contactar. La Carrera de Nutrición de la U. Cuenca recibió la lista de temas y no la tomó. La Lcda. María Augusta Vásquez declinó el 05/10. Se mantiene vacante por decisión de la Dra. Omidres.</t>
+          <t>SIN PONENTE. Perfil sugerido: nutricionista clínico con experiencia en diabetes.
+HISTORIAL DE GESTIÓN:
+· Dra. Gaby Villavicencio — DECLINÓ. Recomendó a otras personas, pendientes de contactar.
+· Carrera de Nutrición, U. Cuenca (Lcda. Daniela Vintimilla) — recibió la lista de temas el 23/09 y no tomó este.
+· Lcda. María Augusta Vásquez (+593 99 994 9812) — DECLINÓ el 05/10.
+Se mantiene vacante por decisión de la Dra. Omidres. NO volver a contactar a las tres anteriores para este tema.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Primeros documentos del expediente archivados
Entran la fotografía y el pasaporte del Dr. Chen Ku, que queda como el
primer docente completo, y la declaración firmada de la Dra. Bermeo, que
llevaba once días pendiente por la firma electrónica. Se archivan también
las hojas de vida de la Dra. Piedra, la Dra. Ruilova y la Dra. Palacio.

La matriz recoge los datos que traían los documentos: cédula, institución
y correo de la Dra. Bermeo, que además declara no tener conflictos de
interés, y correo e instituciones de la Dra. Ruilova.

Marcador: 5 hojas de vida, 1 fotografía, 2 declaraciones y 4 documentos de
identidad de 23.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2226,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2616,7 +2616,11 @@
           <t>+506 8392 7083</t>
         </is>
       </c>
-      <c r="G10" s="41" t="n"/>
+      <c r="G10" s="54" t="inlineStr">
+        <is>
+          <t>Pasaporte de Costa Rica (copia en expediente)</t>
+        </is>
+      </c>
       <c r="H10" s="41" t="n"/>
       <c r="I10" s="40" t="inlineStr">
         <is>
@@ -2628,7 +2632,11 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="K10" s="42" t="n"/>
+      <c r="K10" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="L10" s="42" t="inlineStr">
         <is>
           <t>SÍ</t>
@@ -2717,12 +2725,12 @@
           <t>Endocrinología · Medicina Interna</t>
         </is>
       </c>
-      <c r="D12" s="53" t="inlineStr">
-        <is>
-          <t>SOLCA, Hospital Monte Sinaí y Universidad de Cuenca · Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E12" s="53" t="inlineStr">
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>SOLCA Cuenca · Hospital Monte Sinaí · Universidad de Cuenca</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
         <is>
           <t>lizrg@hotmail.com</t>
         </is>
@@ -2961,12 +2969,12 @@
           <t>Medicina Interna · Subespecialista en Endocrinología · Alta especialidad en Obesidad y Enfermedades Tiroideas (UNAM)</t>
         </is>
       </c>
-      <c r="D18" s="53" t="inlineStr">
+      <c r="D18" s="42" t="inlineStr">
         <is>
           <t>Hospital del Río · Cuenca, Ecuador</t>
         </is>
       </c>
-      <c r="E18" s="41" t="inlineStr">
+      <c r="E18" s="42" t="inlineStr">
         <is>
           <t>jbendocrino@hotmail.com</t>
         </is>
@@ -2976,7 +2984,11 @@
           <t>+593 96 198 1203</t>
         </is>
       </c>
-      <c r="G18" s="41" t="n"/>
+      <c r="G18" s="42" t="inlineStr">
+        <is>
+          <t>0104851001</t>
+        </is>
+      </c>
       <c r="H18" s="41" t="n"/>
       <c r="I18" s="54" t="inlineStr">
         <is>
@@ -2989,7 +3001,11 @@
         </is>
       </c>
       <c r="K18" s="42" t="n"/>
-      <c r="L18" s="42" t="n"/>
+      <c r="L18" s="42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
       <c r="M18" s="42" t="n"/>
       <c r="N18" s="65" t="inlineStr">
         <is>
@@ -3337,6 +3353,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="J4:L18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Cédula de la Dra. Bermeo archivada y nombre corregido
Las dos caras del documento confirman la cédula 0104851001 que ya
declaraba el formulario firmado. En la matriz figuraba como Janneth
Bermeo Cabrera y pasa a su nombre completo, Marcia Janneth, que es como
debe constar en el expediente.

Solo le falta la fotografía.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2959,9 +2959,9 @@
       <c r="A18" s="54" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="52" t="inlineStr">
-        <is>
-          <t>Dra. Janneth Bermeo Cabrera</t>
+      <c r="B18" s="42" t="inlineStr">
+        <is>
+          <t>Dra. Marcia Janneth Bermeo Cabrera</t>
         </is>
       </c>
       <c r="C18" s="53" t="inlineStr">
@@ -2986,7 +2986,7 @@
       </c>
       <c r="G18" s="42" t="inlineStr">
         <is>
-          <t>0104851001</t>
+          <t>0104851001 (copia de cédula en expediente)</t>
         </is>
       </c>
       <c r="H18" s="41" t="n"/>

</xml_diff>

<commit_message>
Archivar la declaración de la Dra. Castro de González y validar las cédulas
Su declaración llegó completa, firmada y marcando «sin conflicto», y corrige
tres datos que estaban mal en la matriz: se apellida Castro de González, su
especialidad es Medicina Física y Rehabilitación —figuraba como
fisioterapia— y ejerce en el IESS de Cuenca. Declara un correo distinto de
aquel desde el que escribió, así que queda anotado el dilema en vez de
elegir uno por cuenta propia.

Los seis números de cédula recibidos se pasaron por el dígito verificador
del Registro Civil y los seis cuadran. Queda dicho en el expediente que eso
solo prueba que están bien transcritos, no que la cédula exista ni que sea
de esa persona.

Con esto son 6 declaraciones firmadas de 23 y la Dra. Castro queda a una
fotografía de completar su expediente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3201,20 +3201,24 @@
       <c r="A21" s="54" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="52" t="inlineStr">
-        <is>
-          <t>Dra. Julia Castro</t>
-        </is>
-      </c>
-      <c r="C21" s="53" t="inlineStr">
-        <is>
-          <t>Fisioterapia</t>
-        </is>
-      </c>
-      <c r="D21" s="53" t="n"/>
+      <c r="B21" s="54" t="inlineStr">
+        <is>
+          <t>Dra. Julia Castro de González</t>
+        </is>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t>Medicina Física y Rehabilitación</t>
+        </is>
+      </c>
+      <c r="D21" s="54" t="inlineStr">
+        <is>
+          <t>Instituto Ecuatoriano de Seguridad Social (IESS) — Cuenca, Ecuador</t>
+        </is>
+      </c>
       <c r="E21" s="54" t="inlineStr">
         <is>
-          <t>castromezajulia@gmail.com</t>
+          <t>dracastrorehabilitacion@gmail.com (escribió desde castromezajulia@gmail.com — confirmar cuál usar)</t>
         </is>
       </c>
       <c r="F21" s="41" t="inlineStr">
@@ -3224,7 +3228,7 @@
       </c>
       <c r="G21" s="54" t="inlineStr">
         <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+          <t>0151826435 — dígito verificador correcto; copia enviada por correo, falta guardarla en el expediente</t>
         </is>
       </c>
       <c r="H21" s="41" t="n"/>
@@ -3239,10 +3243,14 @@
         </is>
       </c>
       <c r="K21" s="42" t="n"/>
-      <c r="L21" s="42" t="n"/>
-      <c r="M21" s="42" t="inlineStr">
-        <is>
-          <t>29/10/2026</t>
+      <c r="L21" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="M21" s="54" t="inlineStr">
+        <is>
+          <t>29 de octubre de 2026</t>
         </is>
       </c>
       <c r="N21" s="65" t="inlineStr">

</xml_diff>

<commit_message>
Archivar como provisional la fotografía de la Dra. Castro de González
La imagen recibida mide 150 × 150 píxeles y pesa 4 KB: es una miniatura de
perfil, no un retrato. Impresa a 300 ppp daría 1,3 cm de lado. Se archiva
con el nombre marcado como provisional y en la matriz consta como
PROVISIONAL, no como cumplida, para que nadie dé por resuelta su fotografía
al armar el expediente. Hay que pedirle el archivo original.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3242,7 +3242,11 @@
           <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
         </is>
       </c>
-      <c r="K21" s="42" t="n"/>
+      <c r="K21" s="54" t="inlineStr">
+        <is>
+          <t>PROVISIONAL — solo hay una miniatura de 150×150 px (4 KB), insuficiente para el expediente. Pedirle el archivo original.</t>
+        </is>
+      </c>
       <c r="L21" s="54" t="inlineStr">
         <is>
           <t>SÍ</t>

</xml_diff>

<commit_message>
Ampliar el título de M5·C1 a petición de la docente
La Lcda. Gabriela Molina Ochoa propuso en su formulario ampliar el título de
su clase, y la coordinación lo aprueba añadiendo Ecuador: «Nutrición de
precisión en diabetes y obesidad: innovación, equidad y desafíos para
América Latina y Ecuador».

Queda anotado en la matriz que su declaración firmada lleva el título
anterior, más corto. No hace falta que la rehaga —la declaración identifica
la clase, no la titula—, pero el programa que va al expediente lleva el
título nuevo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1703,7 +1703,7 @@
       </c>
       <c r="C19" s="24" t="inlineStr">
         <is>
-          <t>Nutrición de precisión en diabetes y obesidad</t>
+          <t>Nutrición de precisión en diabetes y obesidad: innovación, equidad y desafíos para América Latina y Ecuador</t>
         </is>
       </c>
       <c r="D19" s="24" t="inlineStr">
@@ -1726,7 +1726,7 @@
       </c>
       <c r="H19" s="24" t="inlineStr">
         <is>
-          <t>Aceptó el 28/09/2026. La propuso la Lcda. Daniela Vintimilla, Directora de la Carrera de Nutrición de la U. Cuenca. Condicionó su participación a recibir certificado de docente, que se le confirmó. Faltan sus documentos.</t>
+          <t>Aceptó el 28/09/2026. La propuso la Lcda. Daniela Vintimilla, Directora de la Carrera de Nutrición de la U. Cuenca. Condicionó su participación a recibir certificado de docente, que se le confirmó. Faltan sus documentos. TÍTULO ACTUALIZADO el 09/10/2026: la docente propuso ampliarlo en su formulario y la coordinación lo aprueba añadiendo «y Ecuador». Su declaración firmada lleva el título anterior, más corto; no hace falta rehacerla, pero el programa que va al expediente lleva este.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Poner al día la hoja de vacantes: solo queda M5·C2
La hoja seguía diciendo «9 clases sin ponente» y daba a la Lcda. María
Augusta Vásquez como pendiente de invitar, cuando declinó el 05/10. Se
alinea con lo que ya registraba la Matriz 28 clases y se regenera el
pedido de documentos, que lee esta hoja.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3612,7 +3612,7 @@
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>LAS 9 CLASES SIN PONENTE · Prioridad de gestión</t>
+          <t>CLASES QUE QUEDARON SIN PONENTE · Queda 1 vacante: M5 · C2 (al 09/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3716,17 +3716,13 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>Lcda. María Augusta Vásquez — nutrición</t>
-        </is>
-      </c>
-      <c r="F5" s="41" t="inlineStr">
-        <is>
-          <t>+593 99 994 9812</t>
-        </is>
-      </c>
+          <t>SIN CANDIDATO — VACANTE</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="n"/>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>La Dra. Gaby Villavicencio no respondió en seis días a la invitación del 23/09. Se reasigna la gestión el 29/09. PENDIENTE DE INVITAR.</t>
+          <t>VACANTE. Declinaron la Dra. Gaby Villavicencio (recomendó a otras personas, pendientes de contactar), la Carrera de Nutrición de la U. Cuenca (recibió los temas el 23/09 y no tomó este) y la Lcda. María Augusta Vásquez (05/10). Se mantiene vacante por decisión de la Dra. Omidres. No volver a contactar a esas tres para este tema.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Armar un borrador de hoja de vida para la Dra. Adriana Álvarez
Con los cargos que ella envió y sus publicaciones en PubMed, separadas
en confirmadas (firma con nombre completo y afiliación al HIBA) y
probables (solo «Alvarez A»). La formación queda POR CONFIRMAR. No
cuenta como entregada ni va al expediente hasta que ella la apruebe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2761,7 +2761,11 @@
           <t>M6 · C4 (MASLD y complicaciones metabólicas)</t>
         </is>
       </c>
-      <c r="J11" s="42" t="n"/>
+      <c r="J11" s="42" t="inlineStr">
+        <is>
+          <t>BORRADOR — la coordinación la armó el 10/10/2026 con los datos de la docente y PubMed (SEDA_HojaVida_Alvarez_BORRADOR.pdf). PENDIENTE de que la Dra. Álvarez la revise, complete su formación y la apruebe.</t>
+        </is>
+      </c>
       <c r="K11" s="42" t="inlineStr">
         <is>
           <t>PARCIAL — solo la del pasaporte</t>

</xml_diff>

<commit_message>
Archivar las hojas de vida de Salas, González y Álvarez
· Dr. Ronald Fabricio Salas Guerrero y Dra. Adriana Victoria González
  Neira: hojas de vida propias, revisadas y contadas. Se corrigen sus
  nombres completos (Fabricio, no Fabrizio) y se añaden correo e
  institución tal como figuran en ellas.
· Dra. Adriana Álvarez: se archiva la versión final que cerró la
  coordinación, pero no se cuenta hasta saber si la docente la aprobó.

El directorio pasa a 14 de 22 hojas de vida. El grupo de WhatsApp se
regenera y recoge además los nombres completos que ya tenía la matriz.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2082,7 +2082,7 @@
       </c>
       <c r="E29" s="24" t="inlineStr">
         <is>
-          <t>Dr. Fabrizio Salas</t>
+          <t>Dr. Fabricio Salas Guerrero</t>
         </is>
       </c>
       <c r="F29" s="27" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="J11" s="42" t="inlineStr">
         <is>
-          <t>BORRADOR — la coordinación la armó el 10/10/2026 con los datos de la docente y PubMed (SEDA_HojaVida_Alvarez_BORRADOR.pdf). PENDIENTE de que la Dra. Álvarez la revise, complete su formación y la apruebe.</t>
+          <t>POR CONFIRMAR — la coordinación cerró el 10/10/2026 la versión final (CV_Alvarez_Adriana-Mabel.pdf), pero falta saber si la Dra. Álvarez la aprobó. Esa versión da como suyas cinco publicaciones firmadas solo «Alvarez A».</t>
         </is>
       </c>
       <c r="K11" s="42" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="B25" s="52" t="inlineStr">
         <is>
-          <t>Dr. Fabrizio Salas</t>
+          <t>Dr. Ronald Fabricio Salas Guerrero</t>
         </is>
       </c>
       <c r="C25" s="53" t="inlineStr">
@@ -3509,10 +3509,14 @@
       </c>
       <c r="D25" s="53" t="inlineStr">
         <is>
-          <t>Ecuador (institución por confirmar)</t>
-        </is>
-      </c>
-      <c r="E25" s="41" t="n"/>
+          <t>Ministerio de Salud Pública del Ecuador (epidemiólogo, 2026)</t>
+        </is>
+      </c>
+      <c r="E25" s="41" t="inlineStr">
+        <is>
+          <t>fabriciosalasguerrero@gmail.com</t>
+        </is>
+      </c>
       <c r="F25" s="41" t="inlineStr">
         <is>
           <t>+593 99 381 4728</t>
@@ -3525,7 +3529,11 @@
           <t>M7 · C3</t>
         </is>
       </c>
-      <c r="J25" s="42" t="n"/>
+      <c r="J25" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 10/10/2026 y archivada (CV_Salas-Guerrero_Ronald-Fabricio.pdf). Ojo: los dos registros SENESCYT que figuran en ella parecen intercambiados entre el título de médico y la maestría.</t>
+        </is>
+      </c>
       <c r="K25" s="42" t="n"/>
       <c r="L25" s="42" t="n"/>
       <c r="M25" s="42" t="inlineStr">
@@ -3545,20 +3553,24 @@
       </c>
       <c r="B26" s="52" t="inlineStr">
         <is>
-          <t>Dra. Adriana González</t>
+          <t>Dra. Adriana Victoria González Neira</t>
         </is>
       </c>
       <c r="C26" s="53" t="inlineStr">
         <is>
-          <t>Endocrinología · Tesorera de ALAD</t>
+          <t>Medicina Interna · Endocrinología · Diabetes · Tesorera de ALAD (2026–2028)</t>
         </is>
       </c>
       <c r="D26" s="53" t="inlineStr">
         <is>
-          <t>Ecuador (institución y ciudad por confirmar)</t>
-        </is>
-      </c>
-      <c r="E26" s="41" t="n"/>
+          <t>Hospital Clínica Kennedy · Hospital General Naval (HOSNAG) — Guayaquil, Ecuador</t>
+        </is>
+      </c>
+      <c r="E26" s="41" t="inlineStr">
+        <is>
+          <t>adrianagn26@yahoo.com</t>
+        </is>
+      </c>
       <c r="F26" s="41" t="inlineStr">
         <is>
           <t>+593 99 602 1221</t>
@@ -3571,7 +3583,11 @@
           <t>M1 · C4</t>
         </is>
       </c>
-      <c r="J26" s="42" t="n"/>
+      <c r="J26" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 10/10/2026 y archivada (CV_Gonzalez-Neira_Adriana-Victoria.pdf)</t>
+        </is>
+      </c>
       <c r="K26" s="42" t="n"/>
       <c r="L26" s="42" t="n"/>
       <c r="M26" s="42" t="inlineStr">
@@ -3821,7 +3837,7 @@
       </c>
       <c r="E8" s="41" t="inlineStr">
         <is>
-          <t>Dr. Fabrizio Salas — médico epidemiólogo, experto en salud digital</t>
+          <t>Dr. Fabricio Salas Guerrero — médico epidemiólogo, experto en salud digital</t>
         </is>
       </c>
       <c r="F8" s="41" t="inlineStr">

</xml_diff>

<commit_message>
Contar la hoja de vida de la Dra. Álvarez y archivar la de la Dra. Cuatecontzi
· Dra. Adriana Álvarez: la Dra. Omidres confirma que aprobó la versión
  final de su hoja de vida.
· Dra. E. Teresa Cuatecontzi Xochitiotzi: hoja de vida propia y
  fotografía profesional (441×478 px). Se completan nombre,
  especialidad, institución y correo tal como figuran en su CV.

El directorio pasa a 16 de 22 hojas de vida y 12 fotografías.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2573,16 +2573,24 @@
       </c>
       <c r="B8" s="39" t="inlineStr">
         <is>
-          <t>Dra. Teresa Cuatecontzi</t>
-        </is>
-      </c>
-      <c r="C8" s="41" t="n"/>
+          <t>Dra. E. Teresa Cuatecontzi Xochitiotzi</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Medicina Interna · Endocrinología · Alta especialidad en Obesidad · Maestría en Ciencias Médicas y Nutrición (INCMNSZ/UNAM)</t>
+        </is>
+      </c>
       <c r="D8" s="53" t="inlineStr">
         <is>
-          <t>México (institución y ciudad por confirmar)</t>
-        </is>
-      </c>
-      <c r="E8" s="41" t="n"/>
+          <t>Clínica Especializada en el Manejo de la Diabetes — Ciudad de México, México</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>xochitiotzi1@gmail.com</t>
+        </is>
+      </c>
       <c r="F8" s="41" t="inlineStr">
         <is>
           <t>+52 1 55 5405 6619</t>
@@ -2595,8 +2603,16 @@
           <t>M3 · C3</t>
         </is>
       </c>
-      <c r="J8" s="42" t="n"/>
-      <c r="K8" s="42" t="n"/>
+      <c r="J8" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 11/10/2026 y archivada (CV_Cuatecontzi-Xochitiotzi_Teresa.pdf). En el encabezado dice «TERES» por «TERESA».</t>
+        </is>
+      </c>
+      <c r="K8" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 11/10/2026 (441×478 px, retrato profesional), archivada como Foto_Cuatecontzi-Xochitiotzi_Teresa.jpg</t>
+        </is>
+      </c>
       <c r="L8" s="42" t="n"/>
       <c r="M8" s="42" t="n"/>
       <c r="N8" s="43" t="inlineStr">
@@ -2763,7 +2779,7 @@
       </c>
       <c r="J11" s="42" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR — la coordinación cerró el 10/10/2026 la versión final (CV_Alvarez_Adriana-Mabel.pdf), pero falta saber si la Dra. Álvarez la aprobó. Esa versión da como suyas cinco publicaciones firmadas solo «Alvarez A».</t>
+          <t>SÍ — versión final cerrada por la coordinación el 10/10/2026 y APROBADA por la Dra. Álvarez, según la Dra. Omidres (10/10/2026). Archivada como CV_Alvarez_Adriana-Mabel.pdf. Incluye cinco publicaciones firmadas «Alvarez A» que ella da por suyas al aprobarla.</t>
         </is>
       </c>
       <c r="K11" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Registrar que los recomendados para M5·C2 no respondieron
La Dra. Omidres escribió a las personas que recomendó la Dra.
Villavicencio y no hubo respuesta al 12/10/2026. La clase sigue
vacante.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1760,7 +1760,7 @@
         <is>
           <t>SIN PONENTE. Perfil sugerido: nutricionista clínico con experiencia en diabetes.
 HISTORIAL DE GESTIÓN:
-· Dra. Gaby Villavicencio — DECLINÓ. Recomendó a otras personas, pendientes de contactar.
+· Dra. Gaby Villavicencio — DECLINÓ. Recomendó a otras personas: la Dra. Omidres les escribió y no respondieron (al 12/10/2026).
 · Carrera de Nutrición, U. Cuenca (Lcda. Daniela Vintimilla) — recibió la lista de temas el 23/09 y no tomó este.
 · Lcda. María Augusta Vásquez (+593 99 994 9812) — DECLINÓ el 05/10.
 Se mantiene vacante por decisión de la Dra. Omidres. NO volver a contactar a las tres anteriores para este tema.</t>
@@ -2135,6 +2135,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="C32" s="31" t="inlineStr">
         <is>
@@ -2190,6 +2191,7 @@
         <v/>
       </c>
     </row>
+    <row r="37"/>
     <row r="38">
       <c r="C38" s="34" t="inlineStr">
         <is>
@@ -3758,7 +3760,7 @@
       <c r="F5" s="41" t="n"/>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>VACANTE. Declinaron la Dra. Gaby Villavicencio (recomendó a otras personas, pendientes de contactar), la Carrera de Nutrición de la U. Cuenca (recibió los temas el 23/09 y no tomó este) y la Lcda. María Augusta Vásquez (05/10). Se mantiene vacante por decisión de la Dra. Omidres. No volver a contactar a esas tres para este tema.</t>
+          <t>VACANTE. Declinaron la Dra. Gaby Villavicencio (recomendó a otras personas; se les escribió y no respondieron al 12/10/2026), la Carrera de Nutrición de la U. Cuenca (recibió los temas el 23/09 y no tomó este) y la Lcda. María Augusta Vásquez (05/10). Se mantiene vacante por decisión de la Dra. Omidres. No volver a contactar a esas tres para este tema.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registrar que llegó la hoja de vida de la Dra. María Paz Castillo
La envió la Dra. Ruilova por correo el 12/10/2026. Queda POR CONFIRMAR
hasta abrirla y comprobar que es suya. Su tarjeta en la página de
mensajes avisa que ya no hace falta pedírsela.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2135,7 +2135,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="C32" s="31" t="inlineStr">
         <is>
@@ -2191,7 +2190,6 @@
         <v/>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="C38" s="34" t="inlineStr">
         <is>
@@ -3227,7 +3225,11 @@
           <t>M4 · C1</t>
         </is>
       </c>
-      <c r="J19" s="42" t="n"/>
+      <c r="J19" s="42" t="inlineStr">
+        <is>
+          <t>POR CONFIRMAR — llegó por correo el 12/10/2026, enviada por la Dra. Ruilova («hoja de vida completa 22-9-2026.pdf», unos 17 MB). Falta abrirla, comprobar que es suya y guardarla en el expediente.</t>
+        </is>
+      </c>
       <c r="K19" s="42" t="n"/>
       <c r="L19" s="42" t="n"/>
       <c r="M19" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Archivar la hoja de vida de la Dra. Gabriela Jiménez Encalada
Hoja de vida propia. Se completan nombre, institución y correo tal como
figuran en ella, y sale de la lista de mensajes pendientes. El
directorio pasa a 18 de 22.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2995,16 +2995,24 @@
       </c>
       <c r="B15" s="39" t="inlineStr">
         <is>
-          <t>Dra. Gabriela Jiménez</t>
+          <t>Dra. Marcia Gabriela Jiménez Encalada</t>
         </is>
       </c>
       <c r="C15" s="41" t="inlineStr">
         <is>
-          <t>Endocrinología</t>
-        </is>
-      </c>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="41" t="n"/>
+          <t>Medicina Interna · Endocrinología</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Centro de Especialidades Médicas de la Universidad de Cuenca · Hospital Santa Inés — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>gabriela.jimeneze@ucuenca.edu.ec</t>
+        </is>
+      </c>
       <c r="F15" s="60" t="inlineStr">
         <is>
           <t>+593 99 807 8964</t>
@@ -3017,7 +3025,11 @@
           <t>M4 · C3</t>
         </is>
       </c>
-      <c r="J15" s="42" t="n"/>
+      <c r="J15" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 12/10/2026 y archivada (CV_Jimenez-Encalada_Marcia-Gabriela.docx). Última modificación del archivo: diciembre de 2024.</t>
+        </is>
+      </c>
       <c r="K15" s="42" t="n"/>
       <c r="L15" s="42" t="n"/>
       <c r="M15" s="42" t="n"/>

</xml_diff>

<commit_message>
Archivar las hojas de vida de María Paz y Cristian Castillo Cabrera
Las dos se revisaron y se guardan en el expediente. La de la Dra.
Castillo la sitúa en Ciudad de México desde junio de 2026 y no menciona
cargos en la Universidad de Cuenca; queda anotado en la matriz. La
hoja de vida «actualizada» de la Dra. Ruilova tiene el mismo contenido
que la ya archivada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2841,7 +2841,7 @@
       </c>
       <c r="J12" s="54" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>SÍ — archivada (CV_Ruilova-Gonzalez_Lizbet.pdf). La «actualizada» que reenvió el 12/10/2026 tiene el mismo contenido.</t>
         </is>
       </c>
       <c r="K12" s="54" t="inlineStr">
@@ -3216,15 +3216,19 @@
       </c>
       <c r="C19" s="53" t="inlineStr">
         <is>
-          <t>Endocrinología</t>
+          <t>Medicina Interna · Endocrinología · Alta especialidad en Enfermedades Tiroideas (UNAM)</t>
         </is>
       </c>
       <c r="D19" s="53" t="inlineStr">
         <is>
-          <t>Cuenca, Ecuador (institución por confirmar) — confirmado por la Dra. Ruilova el 29/09</t>
-        </is>
-      </c>
-      <c r="E19" s="41" t="n"/>
+          <t>Centro Metropolitano de Oncología Integral, Hospital Ángeles — Ciudad de México, México (según su hoja de vida de 22/09/2026)</t>
+        </is>
+      </c>
+      <c r="E19" s="41" t="inlineStr">
+        <is>
+          <t>mariapazcc22@hotmail.com</t>
+        </is>
+      </c>
       <c r="F19" s="41" t="inlineStr">
         <is>
           <t>+52 1 56 2489 0698</t>
@@ -3239,7 +3243,7 @@
       </c>
       <c r="J19" s="42" t="inlineStr">
         <is>
-          <t>SÍ — la envió la Dra. Ruilova por correo el 12/10/2026 («hoja de vida completa 22-9-2026.pdf»); la Dra. Omidres la revisó y la da por buena (12/10/2026). El archivo sigue en el correo, falta guardarlo en el expediente.</t>
+          <t>SÍ — llegó por la Dra. Ruilova el 12/10/2026; revisada y archivada (CV_Castillo-Cabrera_Maria-Paz.pdf). Ojo: su hoja de vida la sitúa trabajando en Ciudad de México desde junio de 2026, no en Cuenca, y no menciona ningún cargo en la Universidad de Cuenca.</t>
         </is>
       </c>
       <c r="K19" s="42" t="n"/>
@@ -3261,7 +3265,7 @@
       </c>
       <c r="B20" s="54" t="inlineStr">
         <is>
-          <t>Dr. Cristian Castillo Cabrera</t>
+          <t>Dr. Cristian Oswaldo Castillo Cabrera</t>
         </is>
       </c>
       <c r="C20" s="53" t="inlineStr">
@@ -3269,7 +3273,11 @@
           <t>Cirugía bariátrica y metabólica</t>
         </is>
       </c>
-      <c r="D20" s="53" t="n"/>
+      <c r="D20" s="53" t="inlineStr">
+        <is>
+          <t>Hospital Santa Inés — Cuenca, Ecuador</t>
+        </is>
+      </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
           <t>cristiancastillodr@gmail.com</t>
@@ -3293,7 +3301,7 @@
       </c>
       <c r="J20" s="54" t="inlineStr">
         <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+          <t>SÍ — recibida el 07/10/2026 (y reenviada por la Dra. Ruilova el 12/10/2026); revisada y archivada (CV_Castillo-Cabrera_Cristian-Oswaldo.pdf)</t>
         </is>
       </c>
       <c r="K20" s="54" t="inlineStr">

</xml_diff>

<commit_message>
Armar un borrador de hoja de vida para la Dra. Ana María Gómez
Con sus artículos y afiliaciones en PubMed, suponiendo que es la Dra.
Ana María Gómez Medina, de la Javeriana. Formación y cargos docentes
quedan POR CONFIRMAR. No cuenta como entregada hasta que ella la
apruebe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3519,7 +3519,11 @@
           <t>M7 · C2</t>
         </is>
       </c>
-      <c r="J24" s="42" t="n"/>
+      <c r="J24" s="42" t="inlineStr">
+        <is>
+          <t>BORRADOR — la coordinación la armó el 12/10/2026 con PubMed (SEDA_HojaVida_Gomez_BORRADOR.pdf), suponiendo que es la Dra. Ana María Gómez Medina (Hospital Universitario San Ignacio, Javeriana). PENDIENTE de confirmar y de que ella la apruebe.</t>
+        </is>
+      </c>
       <c r="K24" s="42" t="n"/>
       <c r="L24" s="42" t="n"/>
       <c r="M24" s="42" t="inlineStr">

</xml_diff>

<commit_message>
Contar la hoja de vida de la Dra. Ana María Gómez Medina
La Dra. Omidres confirma que la docente aprobó la versión armada por la
coordinación. Se archiva, se completa su nombre e institución y sale de
la lista de mensajes pendientes. El directorio pasa a 19 de 22.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3493,17 +3493,17 @@
       </c>
       <c r="B24" s="52" t="inlineStr">
         <is>
-          <t>Dra. Ana María Gómez</t>
+          <t>Dra. Ana María Gómez Medina</t>
         </is>
       </c>
       <c r="C24" s="53" t="inlineStr">
         <is>
-          <t>Endocrinología · experta en monitoreo de glucosa</t>
+          <t>Medicina Interna · Endocrinología · Tecnología en diabetes</t>
         </is>
       </c>
       <c r="D24" s="53" t="inlineStr">
         <is>
-          <t>Colombia (institución y ciudad por confirmar)</t>
+          <t>Hospital Universitario San Ignacio · Pontificia Universidad Javeriana — Bogotá, Colombia</t>
         </is>
       </c>
       <c r="E24" s="41" t="n"/>
@@ -3521,7 +3521,7 @@
       </c>
       <c r="J24" s="42" t="inlineStr">
         <is>
-          <t>BORRADOR — la coordinación la armó el 12/10/2026 con PubMed (SEDA_HojaVida_Gomez_BORRADOR.pdf), suponiendo que es la Dra. Ana María Gómez Medina (Hospital Universitario San Ignacio, Javeriana). PENDIENTE de confirmar y de que ella la apruebe.</t>
+          <t>SÍ — versión armada por la coordinación con PubMed y APROBADA por la Dra. Gómez, según la Dra. Omidres (12/10/2026). Archivada como CV_Gomez-Medina_Ana-Maria.pdf.</t>
         </is>
       </c>
       <c r="K24" s="42" t="n"/>

</xml_diff>

<commit_message>
Archivar la hoja de vida de la Dra. Andrea Valeria Andrade Izquierdo
Hoja de vida propia. Se completan nombre, especialidad, institución y
correo, y sale de la lista de mensajes pendientes. El directorio pasa
a 20 de 22.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3111,16 +3111,24 @@
       </c>
       <c r="B17" s="39" t="inlineStr">
         <is>
-          <t>Dra. Valeria Andrade</t>
-        </is>
-      </c>
-      <c r="C17" s="41" t="n"/>
+          <t>Dra. Andrea Valeria Andrade Izquierdo</t>
+        </is>
+      </c>
+      <c r="C17" s="41" t="inlineStr">
+        <is>
+          <t>Nefrología · Trasplante renal · PhD en Ciencias (Nefrología), Universidad de São Paulo</t>
+        </is>
+      </c>
       <c r="D17" s="41" t="inlineStr">
         <is>
-          <t>Ecuador (institución y ciudad por confirmar)</t>
-        </is>
-      </c>
-      <c r="E17" s="41" t="n"/>
+          <t>Hospital Santa Inés · Universidad de Cuenca — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E17" s="41" t="inlineStr">
+        <is>
+          <t>vale19_ec@yahoo.com</t>
+        </is>
+      </c>
       <c r="F17" s="41" t="inlineStr">
         <is>
           <t>+593 98 335 5686</t>
@@ -3133,7 +3141,11 @@
           <t>M6 · C1</t>
         </is>
       </c>
-      <c r="J17" s="42" t="n"/>
+      <c r="J17" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 12/10/2026 y archivada (CV_Andrade-Izquierdo_Andrea-Valeria.pdf). Fechada en septiembre de 2025.</t>
+        </is>
+      </c>
       <c r="K17" s="42" t="n"/>
       <c r="L17" s="42" t="n"/>
       <c r="M17" s="42" t="n"/>

</xml_diff>

<commit_message>
Styp Canto acepta M7 · C4; la Dra. Omidres conserva M7 · C1
- Matriz: M7 · C4 asignada y fila nueva en Ponentes (datos POR CONFIRMAR)
- Declaración COI de la Dra. Omidres: se quita M7 · C4
- Registro del vínculo MEDDI en conflictos-de-interes-expediente.md
- Directorio regenerado (23 docentes) y delimitación actualizada

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2118,7 +2118,7 @@
       </c>
       <c r="E30" s="24" t="inlineStr">
         <is>
-          <t>Dra. Omidres Pérez de Carvelli</t>
+          <t>Ing. Styp Canto</t>
         </is>
       </c>
       <c r="F30" s="27" t="inlineStr">
@@ -2226,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I4" s="40" t="inlineStr">
         <is>
-          <t>M7 · C1  /  M7 · C4</t>
+          <t>M7 · C1</t>
         </is>
       </c>
       <c r="J4" s="54" t="inlineStr">
@@ -3656,6 +3656,52 @@
           <t>CONFIRMADO — falta toda la documentación</t>
         </is>
       </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="54" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="52" t="inlineStr">
+        <is>
+          <t>Ing. Styp Canto</t>
+        </is>
+      </c>
+      <c r="C27" s="53" t="inlineStr">
+        <is>
+          <t>Ingeniería — especialidad POR CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="D27" s="53" t="inlineStr">
+        <is>
+          <t>POR CONFIRMAR</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="inlineStr">
+        <is>
+          <t>styp611@outlook.com</t>
+        </is>
+      </c>
+      <c r="F27" s="41" t="n"/>
+      <c r="G27" s="41" t="n"/>
+      <c r="H27" s="41" t="n"/>
+      <c r="I27" s="54" t="inlineStr">
+        <is>
+          <t>M7 · C4</t>
+        </is>
+      </c>
+      <c r="J27" s="42" t="n"/>
+      <c r="K27" s="42" t="n"/>
+      <c r="L27" s="42" t="inlineStr">
+        <is>
+          <t>PENDIENTE — debe declarar su vínculo profesional con la Dra. Omidres (MEDDI)</t>
+        </is>
+      </c>
+      <c r="M27" s="42" t="inlineStr">
+        <is>
+          <t>03/12/2026</t>
+        </is>
+      </c>
+      <c r="N27" s="65" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3928,17 +3974,17 @@
       </c>
       <c r="E9" s="41" t="inlineStr">
         <is>
-          <t>Dra. Omidres Pérez de Carvelli</t>
+          <t>Ing. Styp Canto</t>
         </is>
       </c>
       <c r="F9" s="41" t="inlineStr">
         <is>
-          <t>info@draomidresperez.com</t>
+          <t>styp611@outlook.com · WhatsApp POR CONFIRMAR</t>
         </is>
       </c>
       <c r="G9" s="41" t="inlineStr">
         <is>
-          <t>CUBIERTA — la asume la Dra. Omidres (23/09/2026)</t>
+          <t>CUBIERTA — aceptó el 12/10/2026. La Dra. Omidres la tenía desde el 23/09 y se la cedió; ella conserva M7 · C1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Datos de la hoja de vida de Styp Canto Rondón en la matriz y en conflictos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2118,7 +2118,7 @@
       </c>
       <c r="E30" s="24" t="inlineStr">
         <is>
-          <t>Ing. Styp Canto</t>
+          <t>Ing. Styp Canto Rondón</t>
         </is>
       </c>
       <c r="F30" s="27" t="inlineStr">
@@ -3663,17 +3663,17 @@
       </c>
       <c r="B27" s="52" t="inlineStr">
         <is>
-          <t>Ing. Styp Canto</t>
+          <t>Ing. Styp Bill Roy Canto Rondón</t>
         </is>
       </c>
       <c r="C27" s="53" t="inlineStr">
         <is>
-          <t>Ingeniería — especialidad POR CONFIRMAR</t>
+          <t>Ingeniería de Telecomunicaciones · TI en salud, telemedicina e interoperabilidad (HL7 FHIR)</t>
         </is>
       </c>
       <c r="D27" s="53" t="inlineStr">
         <is>
-          <t>POR CONFIRMAR</t>
+          <t>Centro Nacional de Telemedicina (CENATE) – EsSalud · Lima, Perú</t>
         </is>
       </c>
       <c r="E27" s="41" t="inlineStr">
@@ -3681,19 +3681,31 @@
           <t>styp611@outlook.com</t>
         </is>
       </c>
-      <c r="F27" s="41" t="n"/>
+      <c r="F27" s="41" t="inlineStr">
+        <is>
+          <t>+51 956 194 180</t>
+        </is>
+      </c>
       <c r="G27" s="41" t="n"/>
-      <c r="H27" s="41" t="n"/>
+      <c r="H27" s="41" t="inlineStr">
+        <is>
+          <t>CIP 131278 (Colegio de Ingenieros del Perú)</t>
+        </is>
+      </c>
       <c r="I27" s="54" t="inlineStr">
         <is>
           <t>M7 · C4</t>
         </is>
       </c>
-      <c r="J27" s="42" t="n"/>
+      <c r="J27" s="42" t="inlineStr">
+        <is>
+          <t>PARCIAL — el contenido llegó pegado como texto el 12/10/2026; falta el archivo PDF o Word para el expediente</t>
+        </is>
+      </c>
       <c r="K27" s="42" t="n"/>
       <c r="L27" s="42" t="inlineStr">
         <is>
-          <t>PENDIENTE — debe declarar su vínculo profesional con la Dra. Omidres (MEDDI)</t>
+          <t>PENDIENTE — debe declarar: vínculo profesional con la Dra. Omidres en MEDDI Hub (su CV dice consultor 02/2022–12/2023, pero en 09/2026 usa styp@meddi.com: POR CONFIRMAR si sigue) y que es miembro vocal y fundador de la OITT, que preside la Dra. Omidres</t>
         </is>
       </c>
       <c r="M27" s="42" t="inlineStr">
@@ -3701,7 +3713,11 @@
           <t>03/12/2026</t>
         </is>
       </c>
-      <c r="N27" s="65" t="n"/>
+      <c r="N27" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — aceptó el 12/10/2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3974,12 +3990,12 @@
       </c>
       <c r="E9" s="41" t="inlineStr">
         <is>
-          <t>Ing. Styp Canto</t>
+          <t>Ing. Styp Canto Rondón — ingeniero en TI en salud, CENATE-EsSalud, Perú</t>
         </is>
       </c>
       <c r="F9" s="41" t="inlineStr">
         <is>
-          <t>styp611@outlook.com · WhatsApp POR CONFIRMAR</t>
+          <t>+51 956 194 180 · styp611@outlook.com</t>
         </is>
       </c>
       <c r="G9" s="41" t="inlineStr">

</xml_diff>

<commit_message>
Solicitud de aval y expediente para la Universidad de Cuenca; Isabel Reinoso en M5 · C2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1747,10 +1747,14 @@
           <t>Dieta mediterránea; restricción de carbohidratos; ayuno intermitente</t>
         </is>
       </c>
-      <c r="E20" s="28" t="inlineStr"/>
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>Lcda. Isabel Reinoso</t>
+        </is>
+      </c>
       <c r="F20" s="29" t="inlineStr">
         <is>
-          <t>VACANTE</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G20" s="23" t="n">
@@ -2438,7 +2442,7 @@
       <c r="H5" s="41" t="n"/>
       <c r="I5" s="40" t="inlineStr">
         <is>
-          <t>M2 · C1</t>
+          <t>M2 · C1  /  M5 · C2</t>
         </is>
       </c>
       <c r="J5" s="54" t="inlineStr">
@@ -3750,7 +3754,7 @@
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>CLASES QUE QUEDARON SIN PONENTE · Queda 1 vacante: M5 · C2 (al 09/10/2026)</t>
+          <t>CLASES QUE QUEDARON SIN PONENTE · No quedan vacantes: M5 · C2 asignada a la Lcda. Isabel Reinoso (13/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3854,13 +3858,17 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>SIN CANDIDATO — VACANTE</t>
-        </is>
-      </c>
-      <c r="F5" s="41" t="n"/>
+          <t>Lcda. María Isabel Reinoso Pesántez</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>+593 98 736 8816</t>
+        </is>
+      </c>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>VACANTE. Declinaron la Dra. Gaby Villavicencio (recomendó a otras personas; se les escribió y no respondieron al 12/10/2026), la Carrera de Nutrición de la U. Cuenca (recibió los temas el 23/09 y no tomó este) y la Lcda. María Augusta Vásquez (05/10). Se mantiene vacante por decisión de la Dra. Omidres. No volver a contactar a esas tres para este tema.</t>
+          <t>CUBIERTA — asignada por la Dra. Omidres el 13/10/2026, con enfoque en diabetes para no repetir M2 · C2. Antes declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca y la Lcda. Vásquez.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Isabel Reinoso declina M5 · C2: vuelve a vacante; expediente, desglose y directorio regenerados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1747,14 +1747,10 @@
           <t>Dieta mediterránea; restricción de carbohidratos; ayuno intermitente</t>
         </is>
       </c>
-      <c r="E20" s="28" t="inlineStr">
-        <is>
-          <t>Lcda. Isabel Reinoso</t>
-        </is>
-      </c>
+      <c r="E20" s="28" t="n"/>
       <c r="F20" s="29" t="inlineStr">
         <is>
-          <t>CONFIRMADO</t>
+          <t>VACANTE</t>
         </is>
       </c>
       <c r="G20" s="23" t="n">
@@ -2442,7 +2438,7 @@
       <c r="H5" s="41" t="n"/>
       <c r="I5" s="40" t="inlineStr">
         <is>
-          <t>M2 · C1  /  M5 · C2</t>
+          <t>M2 · C1</t>
         </is>
       </c>
       <c r="J5" s="54" t="inlineStr">
@@ -3754,7 +3750,7 @@
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>CLASES QUE QUEDARON SIN PONENTE · No quedan vacantes: M5 · C2 asignada a la Lcda. Isabel Reinoso (13/10/2026)</t>
+          <t>CLASES QUE QUEDARON SIN PONENTE · Queda 1 vacante: M5 · C2 (al 13/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3858,17 +3854,13 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>Lcda. María Isabel Reinoso Pesántez</t>
-        </is>
-      </c>
-      <c r="F5" s="41" t="inlineStr">
-        <is>
-          <t>+593 98 736 8816</t>
-        </is>
-      </c>
+          <t>SIN CANDIDATO — VACANTE</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="n"/>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>CUBIERTA — asignada por la Dra. Omidres el 13/10/2026, con enfoque en diabetes para no repetir M2 · C2. Antes declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca y la Lcda. Vásquez.</t>
+          <t>VACANTE. Declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca, la Lcda. Vásquez y la Lcda. Isabel Reinoso (13/10/2026). Las personas que recomendó la Dra. Villavicencio no respondieron.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M5 · C2: declinan Isabel Reinoso y Johanna Piedra; invitación al Dr. Ramón de Cangas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3854,13 +3854,13 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>SIN CANDIDATO — VACANTE</t>
+          <t>Dr. Ramón de Cangas — propuesto por la Dra. Omidres (13/10/2026), invitación por enviar</t>
         </is>
       </c>
       <c r="F5" s="41" t="n"/>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>VACANTE. Declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca, la Lcda. Vásquez y la Lcda. Isabel Reinoso (13/10/2026). Las personas que recomendó la Dra. Villavicencio no respondieron.</t>
+          <t>VACANTE. Declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca, la Lcda. Vásquez, la Lcda. Isabel Reinoso y la Dra. Johanna Piedra (13/10/2026). Las personas que recomendó la Dra. Villavicencio no respondieron.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dr. Ramón de Cangas acepta M5 · C2: 28 de 28 clases con docente; expediente y anexos regenerados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1747,10 +1747,14 @@
           <t>Dieta mediterránea; restricción de carbohidratos; ayuno intermitente</t>
         </is>
       </c>
-      <c r="E20" s="28" t="n"/>
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>Dr. Ramón de Cangas Morán</t>
+        </is>
+      </c>
       <c r="F20" s="29" t="inlineStr">
         <is>
-          <t>VACANTE</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
       <c r="G20" s="23" t="n">
@@ -2226,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3716,6 +3720,56 @@
       <c r="N27" s="65" t="inlineStr">
         <is>
           <t>CONFIRMADO — aceptó el 12/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="54" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>Dr. Ramón de Cangas Morán</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="inlineStr">
+        <is>
+          <t>Dietista-nutricionista · Biología · Doctor en Biología Funcional y Molecular</t>
+        </is>
+      </c>
+      <c r="D28" s="53" t="inlineStr">
+        <is>
+          <t>Clínicas Nutrigroup · Fundación Alimenta Tu Salud — Oviedo, España</t>
+        </is>
+      </c>
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="41" t="n"/>
+      <c r="G28" s="41" t="n"/>
+      <c r="H28" s="41" t="n"/>
+      <c r="I28" s="54" t="inlineStr">
+        <is>
+          <t>M5 · C2</t>
+        </is>
+      </c>
+      <c r="J28" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — resumen curricular armado por la coordinación y aprobado (13/10/2026); archivado como CV_de-Cangas-Moran_Ramon.pdf</t>
+        </is>
+      </c>
+      <c r="K28" s="42" t="n"/>
+      <c r="L28" s="42" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M28" s="42" t="inlineStr">
+        <is>
+          <t>Jueves 19 de noviembre de 2026</t>
+        </is>
+      </c>
+      <c r="N28" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — aceptó el 13/10/2026</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3804,7 @@
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>CLASES QUE QUEDARON SIN PONENTE · Queda 1 vacante: M5 · C2 (al 13/10/2026)</t>
+          <t>CLASES QUE QUEDARON SIN PONENTE · No quedan vacantes (13/10/2026)</t>
         </is>
       </c>
     </row>
@@ -3854,13 +3908,17 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>Dr. Ramón de Cangas — propuesto por la Dra. Omidres (13/10/2026), invitación por enviar</t>
-        </is>
-      </c>
-      <c r="F5" s="41" t="n"/>
+          <t>Dr. Ramón de Cangas Morán — dietista-nutricionista, Oviedo (España)</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>POR CONFIRMAR</t>
+        </is>
+      </c>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>VACANTE. Declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca, la Lcda. Vásquez, la Lcda. Isabel Reinoso y la Dra. Johanna Piedra (13/10/2026). Las personas que recomendó la Dra. Villavicencio no respondieron.</t>
+          <t>CUBIERTA — aceptó el 13/10/2026. Antes declinaron la Dra. Villavicencio, la Carrera de Nutrición de la U. Cuenca, la Lcda. Vásquez, la Lcda. Isabel Reinoso y la Dra. Johanna Piedra.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hojas de vida de Astudillo, Castro y Machado archivadas; Cangas sin conflicto; expediente y anexos regenerados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2969,7 +2969,7 @@
       </c>
       <c r="J14" s="54" t="inlineStr">
         <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Astudillo-Calle_Maria-Augusta.docx, fechada octubre 2024)</t>
         </is>
       </c>
       <c r="K14" s="54" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="D21" s="54" t="inlineStr">
         <is>
-          <t>Instituto Ecuatoriano de Seguridad Social (IESS) — Cuenca, Ecuador</t>
+          <t>Hospital de Especialidades José Carrasco Arteaga (IESS) — Cuenca, Ecuador</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="J21" s="54" t="inlineStr">
         <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Castro-de-Gonzalez_Julia.pdf)</t>
         </is>
       </c>
       <c r="K21" s="54" t="inlineStr">
@@ -3475,12 +3475,24 @@
       </c>
       <c r="B23" s="52" t="inlineStr">
         <is>
-          <t>Dra. Gabriela Machado</t>
-        </is>
-      </c>
-      <c r="C23" s="53" t="n"/>
-      <c r="D23" s="53" t="n"/>
-      <c r="E23" s="41" t="n"/>
+          <t>Dra. María Gabriela Machado Orellana</t>
+        </is>
+      </c>
+      <c r="C23" s="53" t="inlineStr">
+        <is>
+          <t>Medicina · Nutrición clínica · Máster en Nutrición y Metabolismo (Universitat de Barcelona)</t>
+        </is>
+      </c>
+      <c r="D23" s="53" t="inlineStr">
+        <is>
+          <t>Consultorios Arupo · docente de la Facultad de Ciencias Médicas, Universidad de Cuenca — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E23" s="41" t="inlineStr">
+        <is>
+          <t>gabi_machado25@hotmail.com</t>
+        </is>
+      </c>
       <c r="F23" s="41" t="inlineStr">
         <is>
           <t>+593 99 502 5774</t>
@@ -3493,7 +3505,11 @@
           <t>M5 · C3</t>
         </is>
       </c>
-      <c r="J23" s="42" t="n"/>
+      <c r="J23" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Machado-Orellana_Maria-Gabriela.pdf, versión 2022)</t>
+        </is>
+      </c>
       <c r="K23" s="42" t="n"/>
       <c r="L23" s="42" t="n"/>
       <c r="M23" s="42" t="n"/>
@@ -3759,7 +3775,7 @@
       <c r="K28" s="42" t="n"/>
       <c r="L28" s="42" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>PENDIENTE — sin conflicto, según la Dra. Omidres (13/10/2026); no lo exige la Universidad</t>
         </is>
       </c>
       <c r="M28" s="42" t="inlineStr">

</xml_diff>

<commit_message>
M3 · C2 pasa a la Dra. Omidres; expediente completo (24 docentes), declaración y conflictos actualizados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -1453,7 +1453,7 @@
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
-          <t>Dr. Frank Espinoza</t>
+          <t>Dra. Omidres Pérez de Carvelli</t>
         </is>
       </c>
       <c r="F12" s="27" t="inlineStr">
@@ -2230,7 +2230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="I4" s="40" t="inlineStr">
         <is>
-          <t>M7 · C1</t>
+          <t>M3 · C2  /  M7 · C1</t>
         </is>
       </c>
       <c r="J4" s="54" t="inlineStr">
@@ -2539,30 +2539,46 @@
       </c>
       <c r="B7" s="39" t="inlineStr">
         <is>
-          <t>Dr. Frank Espinoza</t>
-        </is>
-      </c>
-      <c r="C7" s="41" t="n"/>
-      <c r="D7" s="41" t="inlineStr">
-        <is>
-          <t>Perú (institución y ciudad por confirmar)</t>
-        </is>
-      </c>
-      <c r="E7" s="41" t="n"/>
+          <t>Dra. E. Teresa Cuatecontzi Xochitiotzi</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Medicina Interna · Endocrinología · Alta especialidad en Obesidad · Maestría en Ciencias Médicas y Nutrición (INCMNSZ/UNAM)</t>
+        </is>
+      </c>
+      <c r="D7" s="53" t="inlineStr">
+        <is>
+          <t>Clínica Especializada en el Manejo de la Diabetes — Ciudad de México, México</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr">
+        <is>
+          <t>xochitiotzi1@gmail.com</t>
+        </is>
+      </c>
       <c r="F7" s="41" t="inlineStr">
         <is>
-          <t>+51 936 260 715</t>
+          <t>+52 1 55 5405 6619</t>
         </is>
       </c>
       <c r="G7" s="41" t="n"/>
       <c r="H7" s="41" t="n"/>
       <c r="I7" s="40" t="inlineStr">
         <is>
-          <t>M3 · C2</t>
-        </is>
-      </c>
-      <c r="J7" s="42" t="n"/>
-      <c r="K7" s="42" t="n"/>
+          <t>M3 · C3</t>
+        </is>
+      </c>
+      <c r="J7" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 11/10/2026 y archivada (CV_Cuatecontzi-Xochitiotzi_Teresa.pdf). En el encabezado dice «TERES» por «TERESA».</t>
+        </is>
+      </c>
+      <c r="K7" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 11/10/2026 (441×478 px, retrato profesional), archivada como Foto_Cuatecontzi-Xochitiotzi_Teresa.jpg</t>
+        </is>
+      </c>
       <c r="L7" s="42" t="n"/>
       <c r="M7" s="42" t="n"/>
       <c r="N7" s="43" t="inlineStr">
@@ -2575,46 +2591,46 @@
       <c r="A8" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="39" t="inlineStr">
-        <is>
-          <t>Dra. E. Teresa Cuatecontzi Xochitiotzi</t>
-        </is>
-      </c>
-      <c r="C8" s="41" t="inlineStr">
-        <is>
-          <t>Medicina Interna · Endocrinología · Alta especialidad en Obesidad · Maestría en Ciencias Médicas y Nutrición (INCMNSZ/UNAM)</t>
+      <c r="B8" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Josefa Elizabeth Palacio Riofrío</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>Endocrinología · Diabetes y Metabolismo</t>
         </is>
       </c>
       <c r="D8" s="53" t="inlineStr">
         <is>
-          <t>Clínica Especializada en el Manejo de la Diabetes — Ciudad de México, México</t>
-        </is>
-      </c>
-      <c r="E8" s="41" t="inlineStr">
-        <is>
-          <t>xochitiotzi1@gmail.com</t>
-        </is>
-      </c>
-      <c r="F8" s="41" t="inlineStr">
-        <is>
-          <t>+52 1 55 5405 6619</t>
-        </is>
-      </c>
-      <c r="G8" s="41" t="n"/>
+          <t>Omni Hospital e Interhospital · Guayaquil, Ecuador</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="53" t="inlineStr">
+        <is>
+          <t>+593 96 816 1654</t>
+        </is>
+      </c>
+      <c r="G8" s="53" t="inlineStr">
+        <is>
+          <t>1103520233</t>
+        </is>
+      </c>
       <c r="H8" s="41" t="n"/>
       <c r="I8" s="40" t="inlineStr">
         <is>
-          <t>M3 · C3</t>
-        </is>
-      </c>
-      <c r="J8" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — recibida el 11/10/2026 y archivada (CV_Cuatecontzi-Xochitiotzi_Teresa.pdf). En el encabezado dice «TERES» por «TERESA».</t>
-        </is>
-      </c>
-      <c r="K8" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — recibida el 11/10/2026 (441×478 px, retrato profesional), archivada como Foto_Cuatecontzi-Xochitiotzi_Teresa.jpg</t>
+          <t>M4 · C2</t>
+        </is>
+      </c>
+      <c r="J8" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="K8" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="L8" s="42" t="n"/>
@@ -2631,34 +2647,38 @@
       </c>
       <c r="B9" s="52" t="inlineStr">
         <is>
-          <t>Dra. Josefa Elizabeth Palacio Riofrío</t>
+          <t>Dr. Chih Hao Chen Ku, M.Sc.</t>
         </is>
       </c>
       <c r="C9" s="53" t="inlineStr">
         <is>
-          <t>Endocrinología · Diabetes y Metabolismo</t>
+          <t>Endocrinología · Farmacología</t>
         </is>
       </c>
       <c r="D9" s="53" t="inlineStr">
         <is>
-          <t>Omni Hospital e Interhospital · Guayaquil, Ecuador</t>
-        </is>
-      </c>
-      <c r="E9" s="41" t="n"/>
-      <c r="F9" s="53" t="inlineStr">
-        <is>
-          <t>+593 96 816 1654</t>
-        </is>
-      </c>
-      <c r="G9" s="53" t="inlineStr">
-        <is>
-          <t>1103520233</t>
+          <t>Clínica Los Yoses · San José, Costa Rica</t>
+        </is>
+      </c>
+      <c r="E9" s="60" t="inlineStr">
+        <is>
+          <t>chenku2409@gmail.com</t>
+        </is>
+      </c>
+      <c r="F9" s="60" t="inlineStr">
+        <is>
+          <t>+506 8392 7083</t>
+        </is>
+      </c>
+      <c r="G9" s="54" t="inlineStr">
+        <is>
+          <t>Pasaporte de Costa Rica (copia en expediente)</t>
         </is>
       </c>
       <c r="H9" s="41" t="n"/>
       <c r="I9" s="40" t="inlineStr">
         <is>
-          <t>M4 · C2</t>
+          <t>M6 · C2  /  M6 · C3</t>
         </is>
       </c>
       <c r="J9" s="54" t="inlineStr">
@@ -2671,8 +2691,16 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="L9" s="42" t="n"/>
-      <c r="M9" s="42" t="n"/>
+      <c r="L9" s="42" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="M9" s="42" t="inlineStr">
+        <is>
+          <t>26/11/2026</t>
+        </is>
+      </c>
       <c r="N9" s="43" t="inlineStr">
         <is>
           <t>CONFIRMADO</t>
@@ -2683,55 +2711,51 @@
       <c r="A10" s="38" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="52" t="inlineStr">
-        <is>
-          <t>Dr. Chih Hao Chen Ku, M.Sc.</t>
-        </is>
-      </c>
-      <c r="C10" s="53" t="inlineStr">
-        <is>
-          <t>Endocrinología · Farmacología</t>
-        </is>
-      </c>
-      <c r="D10" s="53" t="inlineStr">
-        <is>
-          <t>Clínica Los Yoses · San José, Costa Rica</t>
-        </is>
-      </c>
-      <c r="E10" s="60" t="inlineStr">
-        <is>
-          <t>chenku2409@gmail.com</t>
-        </is>
-      </c>
-      <c r="F10" s="60" t="inlineStr">
-        <is>
-          <t>+506 8392 7083</t>
-        </is>
-      </c>
-      <c r="G10" s="54" t="inlineStr">
-        <is>
-          <t>Pasaporte de Costa Rica (copia en expediente)</t>
+      <c r="B10" s="39" t="inlineStr">
+        <is>
+          <t>Dra. Adriana Mabel Álvarez</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Endocrinología · Comité de Esteatosis Hepática Metabólica (SAD) · Coordinadora del Grupo Obesidad-MASH de ALAD · Vocal Región Sur de ALAD</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Hospital Italiano de Buenos Aires · Buenos Aires, Argentina</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>+54 9 11 6708-1708</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="inlineStr">
+        <is>
+          <t>Pasaporte AAI843846 (vence 28/03/2033) · DNI 14.456.727 — copia archivada el 10/10/2026; los cinco dígitos de control de la zona de lectura mecánica son correctos y coinciden con estos datos</t>
         </is>
       </c>
       <c r="H10" s="41" t="n"/>
       <c r="I10" s="40" t="inlineStr">
         <is>
-          <t>M6 · C2  /  M6 · C3</t>
-        </is>
-      </c>
-      <c r="J10" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="K10" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
+          <t>M6 · C4 (MASLD y complicaciones metabólicas)</t>
+        </is>
+      </c>
+      <c r="J10" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — versión final cerrada por la coordinación el 10/10/2026 y APROBADA por la Dra. Álvarez, según la Dra. Omidres (10/10/2026). Archivada como CV_Alvarez_Adriana-Mabel.pdf. Incluye cinco publicaciones firmadas «Alvarez A» que ella da por suyas al aprobarla.</t>
+        </is>
+      </c>
+      <c r="K10" s="42" t="inlineStr">
+        <is>
+          <t>PARCIAL — solo la del pasaporte</t>
         </is>
       </c>
       <c r="L10" s="42" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>PENDIENTE — declaró sin conflicto de palabra; falta el formato firmado</t>
         </is>
       </c>
       <c r="M10" s="42" t="inlineStr">
@@ -2741,7 +2765,7 @@
       </c>
       <c r="N10" s="43" t="inlineStr">
         <is>
-          <t>CONFIRMADO</t>
+          <t>CONFIRMADO — faltan hoja de vida, foto profesional y COI firmada</t>
         </is>
       </c>
     </row>
@@ -2749,61 +2773,57 @@
       <c r="A11" s="38" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="39" t="inlineStr">
-        <is>
-          <t>Dra. Adriana Mabel Álvarez</t>
-        </is>
-      </c>
-      <c r="C11" s="41" t="inlineStr">
-        <is>
-          <t>Endocrinología · Comité de Esteatosis Hepática Metabólica (SAD) · Coordinadora del Grupo Obesidad-MASH de ALAD · Vocal Región Sur de ALAD</t>
-        </is>
-      </c>
-      <c r="D11" s="41" t="inlineStr">
-        <is>
-          <t>Hospital Italiano de Buenos Aires · Buenos Aires, Argentina</t>
-        </is>
-      </c>
-      <c r="E11" s="41" t="n"/>
-      <c r="F11" s="41" t="inlineStr">
-        <is>
-          <t>+54 9 11 6708-1708</t>
-        </is>
-      </c>
-      <c r="G11" s="41" t="inlineStr">
-        <is>
-          <t>Pasaporte AAI843846 (vence 28/03/2033) · DNI 14.456.727 — copia archivada el 10/10/2026; los cinco dígitos de control de la zona de lectura mecánica son correctos y coinciden con estos datos</t>
-        </is>
-      </c>
+      <c r="B11" s="52" t="inlineStr">
+        <is>
+          <t>Dra. Lizbet Yolanda Ruilova González</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="inlineStr">
+        <is>
+          <t>Endocrinología · Medicina Interna</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>SOLCA Cuenca · Hospital Monte Sinaí · Universidad de Cuenca</t>
+        </is>
+      </c>
+      <c r="E11" s="54" t="inlineStr">
+        <is>
+          <t>lizrg@hotmail.com</t>
+        </is>
+      </c>
+      <c r="F11" s="60" t="inlineStr">
+        <is>
+          <t>+593 99 907 3471</t>
+        </is>
+      </c>
+      <c r="G11" s="41" t="n"/>
       <c r="H11" s="41" t="n"/>
       <c r="I11" s="40" t="inlineStr">
         <is>
-          <t>M6 · C4 (MASLD y complicaciones metabólicas)</t>
-        </is>
-      </c>
-      <c r="J11" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — versión final cerrada por la coordinación el 10/10/2026 y APROBADA por la Dra. Álvarez, según la Dra. Omidres (10/10/2026). Archivada como CV_Alvarez_Adriana-Mabel.pdf. Incluye cinco publicaciones firmadas «Alvarez A» que ella da por suyas al aprobarla.</t>
-        </is>
-      </c>
-      <c r="K11" s="42" t="inlineStr">
-        <is>
-          <t>PARCIAL — solo la del pasaporte</t>
-        </is>
-      </c>
-      <c r="L11" s="42" t="inlineStr">
-        <is>
-          <t>PENDIENTE — declaró sin conflicto de palabra; falta el formato firmado</t>
-        </is>
-      </c>
-      <c r="M11" s="42" t="inlineStr">
-        <is>
-          <t>26/11/2026</t>
-        </is>
-      </c>
-      <c r="N11" s="43" t="inlineStr">
-        <is>
-          <t>CONFIRMADO — faltan hoja de vida, foto profesional y COI firmada</t>
+          <t>M1 · C1  /  M5 · C4</t>
+        </is>
+      </c>
+      <c r="J11" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — archivada (CV_Ruilova-Gonzalez_Lizbet.pdf). La «actualizada» que reenvió el 12/10/2026 tiene el mismo contenido.</t>
+        </is>
+      </c>
+      <c r="K11" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="L11" s="54" t="inlineStr">
+        <is>
+          <t>EN BLANCO — el formato llegó sin llenar, sin casilla marcada y sin firma. Debe rehacerla.</t>
+        </is>
+      </c>
+      <c r="M11" s="42" t="n"/>
+      <c r="N11" s="44" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
         </is>
       </c>
     </row>
@@ -2811,41 +2831,45 @@
       <c r="A12" s="38" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="52" t="inlineStr">
-        <is>
-          <t>Dra. Lizbet Yolanda Ruilova González</t>
-        </is>
-      </c>
-      <c r="C12" s="53" t="inlineStr">
-        <is>
-          <t>Endocrinología · Medicina Interna</t>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>Dr. Pablo Esteban Vanegas Cedillo</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>Medicina Interna · Endocrinología · Obesidad y Trastornos de la Conducta Alimentaria</t>
         </is>
       </c>
       <c r="D12" s="54" t="inlineStr">
         <is>
-          <t>SOLCA Cuenca · Hospital Monte Sinaí · Universidad de Cuenca</t>
+          <t>Hospital Santa Inés — Cuenca, Ecuador</t>
         </is>
       </c>
       <c r="E12" s="54" t="inlineStr">
         <is>
-          <t>lizrg@hotmail.com</t>
+          <t>pablo.vanegas90@gmail.com</t>
         </is>
       </c>
       <c r="F12" s="60" t="inlineStr">
         <is>
-          <t>+593 99 907 3471</t>
-        </is>
-      </c>
-      <c r="G12" s="41" t="n"/>
+          <t>+593 98 765 3136</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>0103838058 — leída de la cédula y contrastada con su declaración y su hoja de vida: coinciden</t>
+        </is>
+      </c>
       <c r="H12" s="41" t="n"/>
       <c r="I12" s="40" t="inlineStr">
         <is>
-          <t>M1 · C1  /  M5 · C4</t>
+          <t>M1 · C2  /  M3 · C1</t>
         </is>
       </c>
       <c r="J12" s="54" t="inlineStr">
         <is>
-          <t>SÍ — archivada (CV_Ruilova-Gonzalez_Lizbet.pdf). La «actualizada» que reenvió el 12/10/2026 tiene el mismo contenido.</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="K12" s="54" t="inlineStr">
@@ -2855,7 +2879,7 @@
       </c>
       <c r="L12" s="54" t="inlineStr">
         <is>
-          <t>EN BLANCO — el formato llegó sin llenar, sin casilla marcada y sin firma. Debe rehacerla.</t>
+          <t>SÍ — DECLARA CONFLICTO: honorarios de Boehringer Ingelheim. Debe mencionarlo al inicio de la grabación de M3·C1. Falta completar producto/área, periodo y la fecha de firma.</t>
         </is>
       </c>
       <c r="M12" s="42" t="n"/>
@@ -2871,59 +2895,63 @@
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>Dr. Pablo Esteban Vanegas Cedillo</t>
+          <t>Dra. María Augusta Astudillo Calle</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>Medicina Interna · Endocrinología · Obesidad y Trastornos de la Conducta Alimentaria</t>
+          <t>Medicina Interna · Endocrinología</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr">
         <is>
-          <t>Hospital Santa Inés — Cuenca, Ecuador</t>
+          <t>Hospital Santa Inés · Casa de la Diabetes — Cuenca, Ecuador</t>
         </is>
       </c>
       <c r="E13" s="54" t="inlineStr">
         <is>
-          <t>pablo.vanegas90@gmail.com</t>
+          <t>medimagu@yahoo.com</t>
         </is>
       </c>
       <c r="F13" s="60" t="inlineStr">
         <is>
-          <t>+593 98 765 3136</t>
+          <t>+593 99 811 1635</t>
         </is>
       </c>
       <c r="G13" s="54" t="inlineStr">
         <is>
-          <t>0103838058 — leída de la cédula y contrastada con su declaración y su hoja de vida: coinciden</t>
+          <t>YA PEDIDA por la coordinación el 09/10/2026. Identidad dada por buena: la Dra. Omidres la verificó directamente con ella. El número manuscrito del formulario no es legible en el escaneo y por eso aquí no se transcribe ninguna cifra.</t>
         </is>
       </c>
       <c r="H13" s="41" t="n"/>
       <c r="I13" s="40" t="inlineStr">
         <is>
-          <t>M1 · C2  /  M3 · C1</t>
+          <t>M1 · C3</t>
         </is>
       </c>
       <c r="J13" s="54" t="inlineStr">
         <is>
+          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Astudillo-Calle_Maria-Augusta.docx, fechada octubre 2024)</t>
+        </is>
+      </c>
+      <c r="K13" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+        </is>
+      </c>
+      <c r="L13" s="54" t="inlineStr">
+        <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="K13" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="L13" s="54" t="inlineStr">
-        <is>
-          <t>SÍ — DECLARA CONFLICTO: honorarios de Boehringer Ingelheim. Debe mencionarlo al inicio de la grabación de M3·C1. Falta completar producto/área, periodo y la fecha de firma.</t>
-        </is>
-      </c>
-      <c r="M13" s="42" t="n"/>
+      <c r="M13" s="54" t="inlineStr">
+        <is>
+          <t>28 de octubre de 2026</t>
+        </is>
+      </c>
       <c r="N13" s="44" t="inlineStr">
         <is>
-          <t>CONFIRMADO</t>
+          <t>CONFIRMADO — declinó M4 · C1 el 25/09</t>
         </is>
       </c>
     </row>
@@ -2931,65 +2959,49 @@
       <c r="A14" s="38" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="54" t="inlineStr">
-        <is>
-          <t>Dra. María Augusta Astudillo Calle</t>
-        </is>
-      </c>
-      <c r="C14" s="54" t="inlineStr">
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>Dra. Marcia Gabriela Jiménez Encalada</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
         <is>
           <t>Medicina Interna · Endocrinología</t>
         </is>
       </c>
-      <c r="D14" s="54" t="inlineStr">
-        <is>
-          <t>Hospital Santa Inés · Casa de la Diabetes — Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E14" s="54" t="inlineStr">
-        <is>
-          <t>medimagu@yahoo.com</t>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Centro de Especialidades Médicas de la Universidad de Cuenca · Hospital Santa Inés — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>gabriela.jimeneze@ucuenca.edu.ec</t>
         </is>
       </c>
       <c r="F14" s="60" t="inlineStr">
         <is>
-          <t>+593 99 811 1635</t>
-        </is>
-      </c>
-      <c r="G14" s="54" t="inlineStr">
-        <is>
-          <t>YA PEDIDA por la coordinación el 09/10/2026. Identidad dada por buena: la Dra. Omidres la verificó directamente con ella. El número manuscrito del formulario no es legible en el escaneo y por eso aquí no se transcribe ninguna cifra.</t>
-        </is>
-      </c>
+          <t>+593 99 807 8964</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="n"/>
       <c r="H14" s="41" t="n"/>
       <c r="I14" s="40" t="inlineStr">
         <is>
-          <t>M1 · C3</t>
-        </is>
-      </c>
-      <c r="J14" s="54" t="inlineStr">
-        <is>
-          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Astudillo-Calle_Maria-Augusta.docx, fechada octubre 2024)</t>
-        </is>
-      </c>
-      <c r="K14" s="54" t="inlineStr">
-        <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
-        </is>
-      </c>
-      <c r="L14" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="M14" s="54" t="inlineStr">
-        <is>
-          <t>28 de octubre de 2026</t>
-        </is>
-      </c>
+          <t>M4 · C3</t>
+        </is>
+      </c>
+      <c r="J14" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 12/10/2026 y archivada (CV_Jimenez-Encalada_Marcia-Gabriela.docx). Última modificación del archivo: diciembre de 2024.</t>
+        </is>
+      </c>
+      <c r="K14" s="42" t="n"/>
+      <c r="L14" s="42" t="n"/>
+      <c r="M14" s="42" t="n"/>
       <c r="N14" s="44" t="inlineStr">
         <is>
-          <t>CONFIRMADO — declinó M4 · C1 el 25/09</t>
+          <t>CONFIRMADO — declinó M1 · C4 el 25/09</t>
         </is>
       </c>
     </row>
@@ -2997,49 +3009,65 @@
       <c r="A15" s="38" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="39" t="inlineStr">
-        <is>
-          <t>Dra. Marcia Gabriela Jiménez Encalada</t>
-        </is>
-      </c>
-      <c r="C15" s="41" t="inlineStr">
-        <is>
-          <t>Medicina Interna · Endocrinología</t>
-        </is>
-      </c>
-      <c r="D15" s="41" t="inlineStr">
-        <is>
-          <t>Centro de Especialidades Médicas de la Universidad de Cuenca · Hospital Santa Inés — Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E15" s="41" t="inlineStr">
-        <is>
-          <t>gabriela.jimeneze@ucuenca.edu.ec</t>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>Dr. Juan Fernando Molina Galarza</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>Medicina Interna · Endocrinología · Máster en infección por VIH</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>Hospital General Vicente Corral Moscoso · Corporación Médica Monte Sinaí — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E15" s="54" t="inlineStr">
+        <is>
+          <t>molinagalarza.jf@gmail.com</t>
         </is>
       </c>
       <c r="F15" s="60" t="inlineStr">
         <is>
-          <t>+593 99 807 8964</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="n"/>
+          <t>+593 99 862 5711</t>
+        </is>
+      </c>
+      <c r="G15" s="54" t="inlineStr">
+        <is>
+          <t>0104904313 — la copia está en Drive (formulario), falta guardarla en el expediente</t>
+        </is>
+      </c>
       <c r="H15" s="41" t="n"/>
       <c r="I15" s="40" t="inlineStr">
         <is>
-          <t>M4 · C3</t>
-        </is>
-      </c>
-      <c r="J15" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — recibida el 12/10/2026 y archivada (CV_Jimenez-Encalada_Marcia-Gabriela.docx). Última modificación del archivo: diciembre de 2024.</t>
-        </is>
-      </c>
-      <c r="K15" s="42" t="n"/>
-      <c r="L15" s="42" t="n"/>
-      <c r="M15" s="42" t="n"/>
+          <t>M4 · C4</t>
+        </is>
+      </c>
+      <c r="J15" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="K15" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="L15" s="54" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="M15" s="54" t="inlineStr">
+        <is>
+          <t>12 de noviembre de 2026</t>
+        </is>
+      </c>
       <c r="N15" s="44" t="inlineStr">
         <is>
-          <t>CONFIRMADO — declinó M1 · C4 el 25/09</t>
+          <t>CONFIRMADO</t>
         </is>
       </c>
     </row>
@@ -3047,115 +3075,111 @@
       <c r="A16" s="38" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="54" t="inlineStr">
-        <is>
-          <t>Dr. Juan Fernando Molina Galarza</t>
-        </is>
-      </c>
-      <c r="C16" s="54" t="inlineStr">
-        <is>
-          <t>Medicina Interna · Endocrinología · Máster en infección por VIH</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr">
-        <is>
-          <t>Hospital General Vicente Corral Moscoso · Corporación Médica Monte Sinaí — Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E16" s="54" t="inlineStr">
-        <is>
-          <t>molinagalarza.jf@gmail.com</t>
-        </is>
-      </c>
-      <c r="F16" s="60" t="inlineStr">
-        <is>
-          <t>+593 99 862 5711</t>
-        </is>
-      </c>
-      <c r="G16" s="54" t="inlineStr">
-        <is>
-          <t>0104904313 — la copia está en Drive (formulario), falta guardarla en el expediente</t>
-        </is>
-      </c>
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>Dra. Andrea Valeria Andrade Izquierdo</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>Nefrología · Trasplante renal · PhD en Ciencias (Nefrología), Universidad de São Paulo</t>
+        </is>
+      </c>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Hospital Santa Inés · Universidad de Cuenca — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>vale19_ec@yahoo.com</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="inlineStr">
+        <is>
+          <t>+593 98 335 5686</t>
+        </is>
+      </c>
+      <c r="G16" s="41" t="n"/>
       <c r="H16" s="41" t="n"/>
       <c r="I16" s="40" t="inlineStr">
         <is>
-          <t>M4 · C4</t>
-        </is>
-      </c>
-      <c r="J16" s="54" t="inlineStr">
+          <t>M6 · C1</t>
+        </is>
+      </c>
+      <c r="J16" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — versión actualizada 2026 recibida el 12/10/2026 y archivada como CV_Andrade-Izquierdo_Andrea-Valeria.pdf (reemplaza la de sept. 2025: ahora Presidenta de la Sociedad de Nefrología del Austro)</t>
+        </is>
+      </c>
+      <c r="K16" s="42" t="n"/>
+      <c r="L16" s="42" t="n"/>
+      <c r="M16" s="42" t="n"/>
+      <c r="N16" s="44" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="54" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Dra. Marcia Janneth Bermeo Cabrera</t>
+        </is>
+      </c>
+      <c r="C17" s="53" t="inlineStr">
+        <is>
+          <t>Medicina Interna · Subespecialista en Endocrinología · Alta especialidad en Obesidad y Enfermedades Tiroideas (UNAM)</t>
+        </is>
+      </c>
+      <c r="D17" s="42" t="inlineStr">
+        <is>
+          <t>Hospital del Río · Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E17" s="42" t="inlineStr">
+        <is>
+          <t>jbendocrino@hotmail.com</t>
+        </is>
+      </c>
+      <c r="F17" s="41" t="inlineStr">
+        <is>
+          <t>+593 96 198 1203</t>
+        </is>
+      </c>
+      <c r="G17" s="42" t="inlineStr">
+        <is>
+          <t>0104851001 (copia de cédula en expediente)</t>
+        </is>
+      </c>
+      <c r="H17" s="41" t="n"/>
+      <c r="I17" s="54" t="inlineStr">
+        <is>
+          <t>M2 · C3</t>
+        </is>
+      </c>
+      <c r="J17" s="42" t="inlineStr">
         <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="K16" s="54" t="inlineStr">
+      <c r="K17" s="54" t="inlineStr">
         <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="L16" s="54" t="inlineStr">
+      <c r="L17" s="42" t="inlineStr">
         <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="M16" s="54" t="inlineStr">
-        <is>
-          <t>12 de noviembre de 2026</t>
-        </is>
-      </c>
-      <c r="N16" s="44" t="inlineStr">
-        <is>
-          <t>CONFIRMADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="38" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="39" t="inlineStr">
-        <is>
-          <t>Dra. Andrea Valeria Andrade Izquierdo</t>
-        </is>
-      </c>
-      <c r="C17" s="41" t="inlineStr">
-        <is>
-          <t>Nefrología · Trasplante renal · PhD en Ciencias (Nefrología), Universidad de São Paulo</t>
-        </is>
-      </c>
-      <c r="D17" s="41" t="inlineStr">
-        <is>
-          <t>Hospital Santa Inés · Universidad de Cuenca — Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E17" s="41" t="inlineStr">
-        <is>
-          <t>vale19_ec@yahoo.com</t>
-        </is>
-      </c>
-      <c r="F17" s="41" t="inlineStr">
-        <is>
-          <t>+593 98 335 5686</t>
-        </is>
-      </c>
-      <c r="G17" s="41" t="n"/>
-      <c r="H17" s="41" t="n"/>
-      <c r="I17" s="40" t="inlineStr">
-        <is>
-          <t>M6 · C1</t>
-        </is>
-      </c>
-      <c r="J17" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — versión actualizada 2026 recibida el 12/10/2026 y archivada como CV_Andrade-Izquierdo_Andrea-Valeria.pdf (reemplaza la de sept. 2025: ahora Presidenta de la Sociedad de Nefrología del Austro)</t>
-        </is>
-      </c>
-      <c r="K17" s="42" t="n"/>
-      <c r="L17" s="42" t="n"/>
       <c r="M17" s="42" t="n"/>
-      <c r="N17" s="44" t="inlineStr">
-        <is>
-          <t>CONFIRMADO</t>
+      <c r="N17" s="65" t="inlineStr">
+        <is>
+          <t>CONFIRMADO — declaración COI llena, pendiente de firma electrónica</t>
         </is>
       </c>
     </row>
@@ -3163,61 +3187,53 @@
       <c r="A18" s="54" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="42" t="inlineStr">
-        <is>
-          <t>Dra. Marcia Janneth Bermeo Cabrera</t>
+      <c r="B18" s="52" t="inlineStr">
+        <is>
+          <t>Dra. María Paz Castillo Cabrera</t>
         </is>
       </c>
       <c r="C18" s="53" t="inlineStr">
         <is>
-          <t>Medicina Interna · Subespecialista en Endocrinología · Alta especialidad en Obesidad y Enfermedades Tiroideas (UNAM)</t>
-        </is>
-      </c>
-      <c r="D18" s="42" t="inlineStr">
-        <is>
-          <t>Hospital del Río · Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E18" s="42" t="inlineStr">
-        <is>
-          <t>jbendocrino@hotmail.com</t>
+          <t>Medicina Interna · Endocrinología · Alta especialidad en Enfermedades Tiroideas (UNAM)</t>
+        </is>
+      </c>
+      <c r="D18" s="53" t="inlineStr">
+        <is>
+          <t>Centro Metropolitano de Oncología Integral, Hospital Ángeles — Ciudad de México, México (según su hoja de vida de 22/09/2026)</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>mariapazcc22@hotmail.com</t>
         </is>
       </c>
       <c r="F18" s="41" t="inlineStr">
         <is>
-          <t>+593 96 198 1203</t>
-        </is>
-      </c>
-      <c r="G18" s="42" t="inlineStr">
-        <is>
-          <t>0104851001 (copia de cédula en expediente)</t>
-        </is>
-      </c>
+          <t>+52 1 56 2489 0698</t>
+        </is>
+      </c>
+      <c r="G18" s="41" t="n"/>
       <c r="H18" s="41" t="n"/>
       <c r="I18" s="54" t="inlineStr">
         <is>
-          <t>M2 · C3</t>
+          <t>M4 · C1</t>
         </is>
       </c>
       <c r="J18" s="42" t="inlineStr">
         <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="K18" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="L18" s="42" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="M18" s="42" t="n"/>
+          <t>SÍ — llegó por la Dra. Ruilova el 12/10/2026; revisada y archivada (CV_Castillo-Cabrera_Maria-Paz.pdf). Ojo: su hoja de vida la sitúa trabajando en Ciudad de México desde junio de 2026, no en Cuenca, y no menciona ningún cargo en la Universidad de Cuenca.</t>
+        </is>
+      </c>
+      <c r="K18" s="42" t="n"/>
+      <c r="L18" s="42" t="n"/>
+      <c r="M18" s="42" t="inlineStr">
+        <is>
+          <t>12/11/2026</t>
+        </is>
+      </c>
       <c r="N18" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — declaración COI llena, pendiente de firma electrónica</t>
+          <t>CONFIRMADO — ponente nacional · PENDIENTE aclarar si interviene en el trámite del aval</t>
         </is>
       </c>
     </row>
@@ -3225,53 +3241,61 @@
       <c r="A19" s="54" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="52" t="inlineStr">
-        <is>
-          <t>Dra. María Paz Castillo Cabrera</t>
+      <c r="B19" s="54" t="inlineStr">
+        <is>
+          <t>Dr. Cristian Oswaldo Castillo Cabrera</t>
         </is>
       </c>
       <c r="C19" s="53" t="inlineStr">
         <is>
-          <t>Medicina Interna · Endocrinología · Alta especialidad en Enfermedades Tiroideas (UNAM)</t>
+          <t>Cirugía bariátrica y metabólica</t>
         </is>
       </c>
       <c r="D19" s="53" t="inlineStr">
         <is>
-          <t>Centro Metropolitano de Oncología Integral, Hospital Ángeles — Ciudad de México, México (según su hoja de vida de 22/09/2026)</t>
-        </is>
-      </c>
-      <c r="E19" s="41" t="inlineStr">
-        <is>
-          <t>mariapazcc22@hotmail.com</t>
+          <t>Hospital Santa Inés — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E19" s="54" t="inlineStr">
+        <is>
+          <t>cristiancastillodr@gmail.com</t>
         </is>
       </c>
       <c r="F19" s="41" t="inlineStr">
         <is>
-          <t>+52 1 56 2489 0698</t>
-        </is>
-      </c>
-      <c r="G19" s="41" t="n"/>
+          <t>+593 97 965 3154</t>
+        </is>
+      </c>
+      <c r="G19" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+        </is>
+      </c>
       <c r="H19" s="41" t="n"/>
       <c r="I19" s="54" t="inlineStr">
         <is>
-          <t>M4 · C1</t>
-        </is>
-      </c>
-      <c r="J19" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — llegó por la Dra. Ruilova el 12/10/2026; revisada y archivada (CV_Castillo-Cabrera_Maria-Paz.pdf). Ojo: su hoja de vida la sitúa trabajando en Ciudad de México desde junio de 2026, no en Cuenca, y no menciona ningún cargo en la Universidad de Cuenca.</t>
-        </is>
-      </c>
-      <c r="K19" s="42" t="n"/>
-      <c r="L19" s="42" t="n"/>
-      <c r="M19" s="42" t="inlineStr">
-        <is>
-          <t>12/11/2026</t>
-        </is>
-      </c>
+          <t>M3 · C4</t>
+        </is>
+      </c>
+      <c r="J19" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — recibida el 07/10/2026 (y reenviada por la Dra. Ruilova el 12/10/2026); revisada y archivada (CV_Castillo-Cabrera_Cristian-Oswaldo.pdf)</t>
+        </is>
+      </c>
+      <c r="K19" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+        </is>
+      </c>
+      <c r="L19" s="54" t="inlineStr">
+        <is>
+          <t>YA PEDIDA la firma por la coordinación el 09/10/2026. Envió el formato el 07/10 pero el archivo no lleva «signed» en el nombre y no se ha podido abrir para comprobar que esté firmado.</t>
+        </is>
+      </c>
+      <c r="M19" s="42" t="n"/>
       <c r="N19" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — ponente nacional · PENDIENTE aclarar si interviene en el trámite del aval</t>
+          <t>CONFIRMADO — falta documentación</t>
         </is>
       </c>
     </row>
@@ -3281,59 +3305,63 @@
       </c>
       <c r="B20" s="54" t="inlineStr">
         <is>
-          <t>Dr. Cristian Oswaldo Castillo Cabrera</t>
-        </is>
-      </c>
-      <c r="C20" s="53" t="inlineStr">
-        <is>
-          <t>Cirugía bariátrica y metabólica</t>
-        </is>
-      </c>
-      <c r="D20" s="53" t="inlineStr">
-        <is>
-          <t>Hospital Santa Inés — Cuenca, Ecuador</t>
+          <t>Dra. Julia Castro de González</t>
+        </is>
+      </c>
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t>Medicina Física y Rehabilitación</t>
+        </is>
+      </c>
+      <c r="D20" s="54" t="inlineStr">
+        <is>
+          <t>Hospital de Especialidades José Carrasco Arteaga (IESS) — Cuenca, Ecuador</t>
         </is>
       </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
-          <t>cristiancastillodr@gmail.com</t>
+          <t>dracastrorehabilitacion@gmail.com (escribió desde castromezajulia@gmail.com — confirmar cuál usar)</t>
         </is>
       </c>
       <c r="F20" s="41" t="inlineStr">
         <is>
-          <t>+593 97 965 3154</t>
+          <t>+593 99 208 7747</t>
         </is>
       </c>
       <c r="G20" s="54" t="inlineStr">
         <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+          <t>0151826435 — dígito verificador correcto; copia enviada por correo, falta guardarla en el expediente</t>
         </is>
       </c>
       <c r="H20" s="41" t="n"/>
       <c r="I20" s="54" t="inlineStr">
         <is>
-          <t>M3 · C4</t>
+          <t>M2 · C4</t>
         </is>
       </c>
       <c r="J20" s="54" t="inlineStr">
         <is>
-          <t>SÍ — recibida el 07/10/2026 (y reenviada por la Dra. Ruilova el 12/10/2026); revisada y archivada (CV_Castillo-Cabrera_Cristian-Oswaldo.pdf)</t>
+          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Castro-de-Gonzalez_Julia.pdf)</t>
         </is>
       </c>
       <c r="K20" s="54" t="inlineStr">
         <is>
-          <t>SÍ — el archivo sigue en el correo, falta guardarlo en el expediente</t>
+          <t>PROVISIONAL — solo hay una miniatura de 150×150 px (4 KB), insuficiente para el expediente. Pedirle el archivo original.</t>
         </is>
       </c>
       <c r="L20" s="54" t="inlineStr">
         <is>
-          <t>YA PEDIDA la firma por la coordinación el 09/10/2026. Envió el formato el 07/10 pero el archivo no lleva «signed» en el nombre y no se ha podido abrir para comprobar que esté firmado.</t>
-        </is>
-      </c>
-      <c r="M20" s="42" t="n"/>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="M20" s="54" t="inlineStr">
+        <is>
+          <t>29 de octubre de 2026</t>
+        </is>
+      </c>
       <c r="N20" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — falta documentación</t>
+          <t>CONFIRMADO — falta documentación · ENTREGA MÁS PRÓXIMA DEL CURSO</t>
         </is>
       </c>
     </row>
@@ -3343,48 +3371,48 @@
       </c>
       <c r="B21" s="54" t="inlineStr">
         <is>
-          <t>Dra. Julia Castro de González</t>
+          <t>Lcda. Gabriela Estefanía Molina Ochoa, Mgt.</t>
         </is>
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
-          <t>Medicina Física y Rehabilitación</t>
+          <t>Nutrición · Diplomado en Educación en Diabetes · Máster en Antropología · Máster en Salud Pública</t>
         </is>
       </c>
       <c r="D21" s="54" t="inlineStr">
         <is>
-          <t>Hospital de Especialidades José Carrasco Arteaga (IESS) — Cuenca, Ecuador</t>
+          <t>Universidad de Cuenca — Cuenca, Ecuador</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
         <is>
-          <t>dracastrorehabilitacion@gmail.com (escribió desde castromezajulia@gmail.com — confirmar cuál usar)</t>
+          <t>gabrielamolinaochoa@gmail.com</t>
         </is>
       </c>
       <c r="F21" s="41" t="inlineStr">
         <is>
-          <t>+593 99 208 7747</t>
+          <t>+593 99 551 4286</t>
         </is>
       </c>
       <c r="G21" s="54" t="inlineStr">
         <is>
-          <t>0151826435 — dígito verificador correcto; copia enviada por correo, falta guardarla en el expediente</t>
+          <t>0105111827</t>
         </is>
       </c>
       <c r="H21" s="41" t="n"/>
       <c r="I21" s="54" t="inlineStr">
         <is>
-          <t>M2 · C4</t>
+          <t>M5 · C1</t>
         </is>
       </c>
       <c r="J21" s="54" t="inlineStr">
         <is>
-          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Castro-de-Gonzalez_Julia.pdf)</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="K21" s="54" t="inlineStr">
         <is>
-          <t>PROVISIONAL — solo hay una miniatura de 150×150 px (4 KB), insuficiente para el expediente. Pedirle el archivo original.</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="L21" s="54" t="inlineStr">
@@ -3394,12 +3422,12 @@
       </c>
       <c r="M21" s="54" t="inlineStr">
         <is>
-          <t>29 de octubre de 2026</t>
+          <t>Jueves 19 de noviembre de 2026</t>
         </is>
       </c>
       <c r="N21" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — falta documentación · ENTREGA MÁS PRÓXIMA DEL CURSO</t>
+          <t>CONFIRMADO — faltan todos los documentos</t>
         </is>
       </c>
     </row>
@@ -3407,65 +3435,49 @@
       <c r="A22" s="54" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="54" t="inlineStr">
-        <is>
-          <t>Lcda. Gabriela Estefanía Molina Ochoa, Mgt.</t>
-        </is>
-      </c>
-      <c r="C22" s="54" t="inlineStr">
-        <is>
-          <t>Nutrición · Diplomado en Educación en Diabetes · Máster en Antropología · Máster en Salud Pública</t>
-        </is>
-      </c>
-      <c r="D22" s="54" t="inlineStr">
-        <is>
-          <t>Universidad de Cuenca — Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E22" s="54" t="inlineStr">
-        <is>
-          <t>gabrielamolinaochoa@gmail.com</t>
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>Dra. María Gabriela Machado Orellana</t>
+        </is>
+      </c>
+      <c r="C22" s="53" t="inlineStr">
+        <is>
+          <t>Medicina · Nutrición clínica · Máster en Nutrición y Metabolismo (Universitat de Barcelona)</t>
+        </is>
+      </c>
+      <c r="D22" s="53" t="inlineStr">
+        <is>
+          <t>Consultorios Arupo · docente de la Facultad de Ciencias Médicas, Universidad de Cuenca — Cuenca, Ecuador</t>
+        </is>
+      </c>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>gabi_machado25@hotmail.com</t>
         </is>
       </c>
       <c r="F22" s="41" t="inlineStr">
         <is>
-          <t>+593 99 551 4286</t>
-        </is>
-      </c>
-      <c r="G22" s="54" t="inlineStr">
-        <is>
-          <t>0105111827</t>
-        </is>
-      </c>
+          <t>+593 99 502 5774</t>
+        </is>
+      </c>
+      <c r="G22" s="41" t="n"/>
       <c r="H22" s="41" t="n"/>
       <c r="I22" s="54" t="inlineStr">
         <is>
-          <t>M5 · C1</t>
-        </is>
-      </c>
-      <c r="J22" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="K22" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="L22" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="M22" s="54" t="inlineStr">
-        <is>
-          <t>Jueves 19 de noviembre de 2026</t>
-        </is>
-      </c>
+          <t>M5 · C3</t>
+        </is>
+      </c>
+      <c r="J22" s="42" t="inlineStr">
+        <is>
+          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Machado-Orellana_Maria-Gabriela.pdf, versión 2022)</t>
+        </is>
+      </c>
+      <c r="K22" s="42" t="n"/>
+      <c r="L22" s="42" t="n"/>
+      <c r="M22" s="42" t="n"/>
       <c r="N22" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — faltan todos los documentos</t>
+          <t>CONFIRMADO — faltan especialidad, institución y documentación</t>
         </is>
       </c>
     </row>
@@ -3475,47 +3487,47 @@
       </c>
       <c r="B23" s="52" t="inlineStr">
         <is>
-          <t>Dra. María Gabriela Machado Orellana</t>
+          <t>Dra. Ana María Gómez Medina</t>
         </is>
       </c>
       <c r="C23" s="53" t="inlineStr">
         <is>
-          <t>Medicina · Nutrición clínica · Máster en Nutrición y Metabolismo (Universitat de Barcelona)</t>
+          <t>Medicina Interna · Endocrinología · Tecnología en diabetes</t>
         </is>
       </c>
       <c r="D23" s="53" t="inlineStr">
         <is>
-          <t>Consultorios Arupo · docente de la Facultad de Ciencias Médicas, Universidad de Cuenca — Cuenca, Ecuador</t>
-        </is>
-      </c>
-      <c r="E23" s="41" t="inlineStr">
-        <is>
-          <t>gabi_machado25@hotmail.com</t>
-        </is>
-      </c>
+          <t>Hospital Universitario San Ignacio · Pontificia Universidad Javeriana — Bogotá, Colombia</t>
+        </is>
+      </c>
+      <c r="E23" s="41" t="n"/>
       <c r="F23" s="41" t="inlineStr">
         <is>
-          <t>+593 99 502 5774</t>
+          <t>+57 310 488 4626</t>
         </is>
       </c>
       <c r="G23" s="41" t="n"/>
       <c r="H23" s="41" t="n"/>
       <c r="I23" s="54" t="inlineStr">
         <is>
-          <t>M5 · C3</t>
+          <t>M7 · C2</t>
         </is>
       </c>
       <c r="J23" s="42" t="inlineStr">
         <is>
-          <t>SÍ — recibida y archivada el 13/10/2026 (CV_Machado-Orellana_Maria-Gabriela.pdf, versión 2022)</t>
+          <t>SÍ — versión armada por la coordinación con PubMed y APROBADA por la Dra. Gómez, según la Dra. Omidres (12/10/2026). Archivada como CV_Gomez-Medina_Ana-Maria.pdf.</t>
         </is>
       </c>
       <c r="K23" s="42" t="n"/>
       <c r="L23" s="42" t="n"/>
-      <c r="M23" s="42" t="n"/>
+      <c r="M23" s="42" t="inlineStr">
+        <is>
+          <t>03/12/2026</t>
+        </is>
+      </c>
       <c r="N23" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — faltan especialidad, institución y documentación</t>
+          <t>CONFIRMADO — falta toda la documentación</t>
         </is>
       </c>
     </row>
@@ -3525,35 +3537,39 @@
       </c>
       <c r="B24" s="52" t="inlineStr">
         <is>
-          <t>Dra. Ana María Gómez Medina</t>
+          <t>Dr. Ronald Fabricio Salas Guerrero</t>
         </is>
       </c>
       <c r="C24" s="53" t="inlineStr">
         <is>
-          <t>Medicina Interna · Endocrinología · Tecnología en diabetes</t>
+          <t>Medicina · Epidemiología · Salud digital e interoperabilidad</t>
         </is>
       </c>
       <c r="D24" s="53" t="inlineStr">
         <is>
-          <t>Hospital Universitario San Ignacio · Pontificia Universidad Javeriana — Bogotá, Colombia</t>
-        </is>
-      </c>
-      <c r="E24" s="41" t="n"/>
+          <t>Ministerio de Salud Pública del Ecuador (epidemiólogo, 2026)</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>fabriciosalasguerrero@gmail.com</t>
+        </is>
+      </c>
       <c r="F24" s="41" t="inlineStr">
         <is>
-          <t>+57 310 488 4626</t>
+          <t>+593 99 381 4728</t>
         </is>
       </c>
       <c r="G24" s="41" t="n"/>
       <c r="H24" s="41" t="n"/>
       <c r="I24" s="54" t="inlineStr">
         <is>
-          <t>M7 · C2</t>
+          <t>M7 · C3</t>
         </is>
       </c>
       <c r="J24" s="42" t="inlineStr">
         <is>
-          <t>SÍ — versión armada por la coordinación con PubMed y APROBADA por la Dra. Gómez, según la Dra. Omidres (12/10/2026). Archivada como CV_Gomez-Medina_Ana-Maria.pdf.</t>
+          <t>SÍ — recibida el 10/10/2026 y archivada (CV_Salas-Guerrero_Ronald-Fabricio.pdf). Ojo: los dos registros SENESCYT que figuran en ella parecen intercambiados entre el título de médico y la maestría.</t>
         </is>
       </c>
       <c r="K24" s="42" t="n"/>
@@ -3575,46 +3591,46 @@
       </c>
       <c r="B25" s="52" t="inlineStr">
         <is>
-          <t>Dr. Ronald Fabricio Salas Guerrero</t>
+          <t>Dra. Adriana Victoria González Neira</t>
         </is>
       </c>
       <c r="C25" s="53" t="inlineStr">
         <is>
-          <t>Medicina · Epidemiología · Salud digital e interoperabilidad</t>
+          <t>Medicina Interna · Endocrinología · Diabetes · Tesorera de ALAD (2026–2028)</t>
         </is>
       </c>
       <c r="D25" s="53" t="inlineStr">
         <is>
-          <t>Ministerio de Salud Pública del Ecuador (epidemiólogo, 2026)</t>
+          <t>Hospital Clínica Kennedy · Hospital General Naval (HOSNAG) — Guayaquil, Ecuador</t>
         </is>
       </c>
       <c r="E25" s="41" t="inlineStr">
         <is>
-          <t>fabriciosalasguerrero@gmail.com</t>
+          <t>adrianagn26@yahoo.com</t>
         </is>
       </c>
       <c r="F25" s="41" t="inlineStr">
         <is>
-          <t>+593 99 381 4728</t>
+          <t>+593 99 602 1221</t>
         </is>
       </c>
       <c r="G25" s="41" t="n"/>
       <c r="H25" s="41" t="n"/>
       <c r="I25" s="54" t="inlineStr">
         <is>
-          <t>M7 · C3</t>
+          <t>M1 · C4</t>
         </is>
       </c>
       <c r="J25" s="42" t="inlineStr">
         <is>
-          <t>SÍ — recibida el 10/10/2026 y archivada (CV_Salas-Guerrero_Ronald-Fabricio.pdf). Ojo: los dos registros SENESCYT que figuran en ella parecen intercambiados entre el título de médico y la maestría.</t>
+          <t>SÍ — recibida el 10/10/2026 y archivada (CV_Gonzalez-Neira_Adriana-Victoria.pdf)</t>
         </is>
       </c>
       <c r="K25" s="42" t="n"/>
       <c r="L25" s="42" t="n"/>
       <c r="M25" s="42" t="inlineStr">
         <is>
-          <t>03/12/2026</t>
+          <t>29/10/2026</t>
         </is>
       </c>
       <c r="N25" s="65" t="inlineStr">
@@ -3629,51 +3645,59 @@
       </c>
       <c r="B26" s="52" t="inlineStr">
         <is>
-          <t>Dra. Adriana Victoria González Neira</t>
+          <t>Ing. Styp Bill Roy Canto Rondón</t>
         </is>
       </c>
       <c r="C26" s="53" t="inlineStr">
         <is>
-          <t>Medicina Interna · Endocrinología · Diabetes · Tesorera de ALAD (2026–2028)</t>
+          <t>Ingeniería de Telecomunicaciones · TI en salud, telemedicina e interoperabilidad (HL7 FHIR)</t>
         </is>
       </c>
       <c r="D26" s="53" t="inlineStr">
         <is>
-          <t>Hospital Clínica Kennedy · Hospital General Naval (HOSNAG) — Guayaquil, Ecuador</t>
+          <t>Centro Nacional de Telemedicina (CENATE) – EsSalud · Lima, Perú</t>
         </is>
       </c>
       <c r="E26" s="41" t="inlineStr">
         <is>
-          <t>adrianagn26@yahoo.com</t>
+          <t>styp611@outlook.com</t>
         </is>
       </c>
       <c r="F26" s="41" t="inlineStr">
         <is>
-          <t>+593 99 602 1221</t>
+          <t>+51 956 194 180</t>
         </is>
       </c>
       <c r="G26" s="41" t="n"/>
-      <c r="H26" s="41" t="n"/>
+      <c r="H26" s="41" t="inlineStr">
+        <is>
+          <t>CIP 131278 (Colegio de Ingenieros del Perú)</t>
+        </is>
+      </c>
       <c r="I26" s="54" t="inlineStr">
         <is>
-          <t>M1 · C4</t>
+          <t>M7 · C4</t>
         </is>
       </c>
       <c r="J26" s="42" t="inlineStr">
         <is>
-          <t>SÍ — recibida el 10/10/2026 y archivada (CV_Gonzalez-Neira_Adriana-Victoria.pdf)</t>
+          <t>SÍ — llegó la versión original sin respaldos (10 páginas, 300 KB) el 12/10/2026 y se archivó como CV_Canto-Rondon_Styp-Bill-Roy.pdf. La versión armada por la coordinación ya no hace falta</t>
         </is>
       </c>
       <c r="K26" s="42" t="n"/>
-      <c r="L26" s="42" t="n"/>
+      <c r="L26" s="42" t="inlineStr">
+        <is>
+          <t>PENDIENTE — debe declarar: (1) consultor externo vigente de MEDDI Hub, empresa en la que la Dra. Omidres es CMO LATAM; (2) miembro vocal y fundador de la OITT, que preside la Dra. Omidres. Sin vínculo con Omisalud (confirmado por la Dra. Omidres el 12/10/2026)</t>
+        </is>
+      </c>
       <c r="M26" s="42" t="inlineStr">
         <is>
-          <t>29/10/2026</t>
+          <t>03/12/2026</t>
         </is>
       </c>
       <c r="N26" s="65" t="inlineStr">
         <is>
-          <t>CONFIRMADO — falta toda la documentación</t>
+          <t>CONFIRMADO — aceptó el 12/10/2026</t>
         </is>
       </c>
     </row>
@@ -3683,107 +3707,45 @@
       </c>
       <c r="B27" s="52" t="inlineStr">
         <is>
-          <t>Ing. Styp Bill Roy Canto Rondón</t>
+          <t>Dr. Ramón de Cangas Morán</t>
         </is>
       </c>
       <c r="C27" s="53" t="inlineStr">
         <is>
-          <t>Ingeniería de Telecomunicaciones · TI en salud, telemedicina e interoperabilidad (HL7 FHIR)</t>
+          <t>Dietista-nutricionista · Biología · Doctor en Biología Funcional y Molecular</t>
         </is>
       </c>
       <c r="D27" s="53" t="inlineStr">
         <is>
-          <t>Centro Nacional de Telemedicina (CENATE) – EsSalud · Lima, Perú</t>
-        </is>
-      </c>
-      <c r="E27" s="41" t="inlineStr">
-        <is>
-          <t>styp611@outlook.com</t>
-        </is>
-      </c>
-      <c r="F27" s="41" t="inlineStr">
-        <is>
-          <t>+51 956 194 180</t>
-        </is>
-      </c>
+          <t>Clínicas Nutrigroup · Fundación Alimenta Tu Salud — Oviedo, España</t>
+        </is>
+      </c>
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="41" t="n"/>
       <c r="G27" s="41" t="n"/>
-      <c r="H27" s="41" t="inlineStr">
-        <is>
-          <t>CIP 131278 (Colegio de Ingenieros del Perú)</t>
-        </is>
-      </c>
+      <c r="H27" s="41" t="n"/>
       <c r="I27" s="54" t="inlineStr">
         <is>
-          <t>M7 · C4</t>
+          <t>M5 · C2</t>
         </is>
       </c>
       <c r="J27" s="42" t="inlineStr">
         <is>
-          <t>SÍ — llegó la versión original sin respaldos (10 páginas, 300 KB) el 12/10/2026 y se archivó como CV_Canto-Rondon_Styp-Bill-Roy.pdf. La versión armada por la coordinación ya no hace falta</t>
+          <t>SÍ — resumen curricular armado por la coordinación y aprobado (13/10/2026); archivado como CV_de-Cangas-Moran_Ramon.pdf</t>
         </is>
       </c>
       <c r="K27" s="42" t="n"/>
       <c r="L27" s="42" t="inlineStr">
         <is>
-          <t>PENDIENTE — debe declarar: (1) consultor externo vigente de MEDDI Hub, empresa en la que la Dra. Omidres es CMO LATAM; (2) miembro vocal y fundador de la OITT, que preside la Dra. Omidres. Sin vínculo con Omisalud (confirmado por la Dra. Omidres el 12/10/2026)</t>
+          <t>PENDIENTE — sin conflicto, según la Dra. Omidres (13/10/2026); no lo exige la Universidad</t>
         </is>
       </c>
       <c r="M27" s="42" t="inlineStr">
         <is>
-          <t>03/12/2026</t>
+          <t>Jueves 19 de noviembre de 2026</t>
         </is>
       </c>
       <c r="N27" s="65" t="inlineStr">
-        <is>
-          <t>CONFIRMADO — aceptó el 12/10/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="54" t="n">
-        <v>25</v>
-      </c>
-      <c r="B28" s="52" t="inlineStr">
-        <is>
-          <t>Dr. Ramón de Cangas Morán</t>
-        </is>
-      </c>
-      <c r="C28" s="53" t="inlineStr">
-        <is>
-          <t>Dietista-nutricionista · Biología · Doctor en Biología Funcional y Molecular</t>
-        </is>
-      </c>
-      <c r="D28" s="53" t="inlineStr">
-        <is>
-          <t>Clínicas Nutrigroup · Fundación Alimenta Tu Salud — Oviedo, España</t>
-        </is>
-      </c>
-      <c r="E28" s="41" t="n"/>
-      <c r="F28" s="41" t="n"/>
-      <c r="G28" s="41" t="n"/>
-      <c r="H28" s="41" t="n"/>
-      <c r="I28" s="54" t="inlineStr">
-        <is>
-          <t>M5 · C2</t>
-        </is>
-      </c>
-      <c r="J28" s="42" t="inlineStr">
-        <is>
-          <t>SÍ — resumen curricular armado por la coordinación y aprobado (13/10/2026); archivado como CV_de-Cangas-Moran_Ramon.pdf</t>
-        </is>
-      </c>
-      <c r="K28" s="42" t="n"/>
-      <c r="L28" s="42" t="inlineStr">
-        <is>
-          <t>PENDIENTE — sin conflicto, según la Dra. Omidres (13/10/2026); no lo exige la Universidad</t>
-        </is>
-      </c>
-      <c r="M28" s="42" t="inlineStr">
-        <is>
-          <t>Jueves 19 de noviembre de 2026</t>
-        </is>
-      </c>
-      <c r="N28" s="65" t="inlineStr">
         <is>
           <t>CONFIRMADO — aceptó el 13/10/2026</t>
         </is>

</xml_diff>

<commit_message>
Josefa Palacio: hoja de vida 2026 y declaración llenada sin firma
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2606,7 +2606,11 @@
           <t>Omni Hospital e Interhospital · Guayaquil, Ecuador</t>
         </is>
       </c>
-      <c r="E8" s="41" t="n"/>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>josefapalacio27@gmail.com</t>
+        </is>
+      </c>
       <c r="F8" s="53" t="inlineStr">
         <is>
           <t>+593 96 816 1654</t>
@@ -2625,15 +2629,19 @@
       </c>
       <c r="J8" s="54" t="inlineStr">
         <is>
+          <t>SÍ — versión 2026 recibida el 13/10/2026 (agrega el podcast En Rango); archivada</t>
+        </is>
+      </c>
+      <c r="K8" s="54" t="inlineStr">
+        <is>
           <t>SÍ</t>
         </is>
       </c>
-      <c r="K8" s="54" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-      <c r="L8" s="42" t="n"/>
+      <c r="L8" s="42" t="inlineStr">
+        <is>
+          <t>POR CONFIRMAR — llenada el 13/10/2026 (declara NO tener conflicto) pero SIN FIRMA ni fecha; falta firmarla</t>
+        </is>
+      </c>
       <c r="M8" s="42" t="n"/>
       <c r="N8" s="43" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Gabriela Molina: hoja de vida localizada en Drive (formulario) y verificada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012B5UyXLL9ubxzuQGBWyzbg
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -3389,7 +3389,7 @@
       </c>
       <c r="D21" s="54" t="inlineStr">
         <is>
-          <t>Universidad de Cuenca — Cuenca, Ecuador</t>
+          <t>Universidad de Cuenca · Universidad Católica de Cuenca · Casa de la Diabetes — Cuenca, Ecuador</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="J21" s="54" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>SÍ — llegó por el formulario el 06/10/2026 (Drive: «CV_Gabriela_Molina julio 2026 - Gabriela Molina.docx»); contenido verificado el 13/10/2026. FALTA copiarla a expediente/hojas-de-vida/</t>
         </is>
       </c>
       <c r="K21" s="54" t="inlineStr">

</xml_diff>

<commit_message>
Incorporar lo llegado entre el 10 y el 17 de octubre
La Dra. Ruilova envió el 12 de octubre cuatro hojas de vida: la de la Dra.
María Paz Castillo y la de la Dra. Valeria Andrade, que no tenían nada, y
las del Dr. Cristian Castillo y la suya propia, que ya constaban. Con eso el
documento obligatorio baja de diez faltantes a ocho.

La Dra. Palacio Riofrío escribió el 13 de octubre con su hoja de vida y su
declaración, y de paso queda registrado su correo, que era el otro dato que
faltaba de ella. La declaración llegó completa pero sin firma ni fecha al
pie; la coordinación ya le pidió que la reenvíe firmada, así que queda como
pedida y no como faltante.

El formulario sigue en tres respuestas: desde el 6 de octubre no ha entrado
nada por ahí y todo lo demás ha llegado por correo directo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GZ8Kkm9KwxHQZEVf8yg4N
</commit_message>
<xml_diff>
--- a/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
+++ b/curso-obesidad-seda/SEDA_Matriz_Ponentes_Curso_Obesidad.xlsx
@@ -2624,7 +2624,11 @@
           <t>Omni Hospital e Interhospital · Guayaquil, Ecuador</t>
         </is>
       </c>
-      <c r="E9" s="41" t="n"/>
+      <c r="E9" s="54" t="inlineStr">
+        <is>
+          <t>josefapalacio27@gmail.com</t>
+        </is>
+      </c>
       <c r="F9" s="53" t="inlineStr">
         <is>
           <t>+593 96 816 1654</t>
@@ -2651,7 +2655,11 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="L9" s="42" t="n"/>
+      <c r="L9" s="54" t="inlineStr">
+        <is>
+          <t>YA PEDIDA la firma el 13/10/2026. Envió la declaración completa pero sin firma ni fecha al pie.</t>
+        </is>
+      </c>
       <c r="M9" s="42" t="n"/>
       <c r="N9" s="43" t="inlineStr">
         <is>
@@ -3101,7 +3109,11 @@
           <t>M6 · C1</t>
         </is>
       </c>
-      <c r="J17" s="42" t="n"/>
+      <c r="J17" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — enviada por la Dra. Ruilova el 12/10/2026; el archivo sigue en el correo, falta guardarlo en el expediente</t>
+        </is>
+      </c>
       <c r="K17" s="42" t="n"/>
       <c r="L17" s="42" t="n"/>
       <c r="M17" s="42" t="n"/>
@@ -3205,7 +3217,11 @@
           <t>M4 · C1</t>
         </is>
       </c>
-      <c r="J19" s="42" t="n"/>
+      <c r="J19" s="54" t="inlineStr">
+        <is>
+          <t>SÍ — enviada por la Dra. Ruilova el 12/10/2026; el archivo sigue en el correo, falta guardarlo en el expediente</t>
+        </is>
+      </c>
       <c r="K19" s="42" t="n"/>
       <c r="L19" s="42" t="n"/>
       <c r="M19" s="42" t="inlineStr">

</xml_diff>